<commit_message>
Update Test Analysis Report from local execution run
</commit_message>
<xml_diff>
--- a/tests/reports/Test_Analysis_Report.xlsx
+++ b/tests/reports/Test_Analysis_Report.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="805" uniqueCount="313">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="805" uniqueCount="311">
   <si>
     <t>Test ID</t>
   </si>
@@ -56,7 +56,7 @@
     <t>Passed</t>
   </si>
   <si>
-    <t>2396ms</t>
+    <t>1974ms</t>
   </si>
   <si>
     <t>Assertion passed successfully</t>
@@ -68,7 +68,7 @@
     <t>Verify brand name PayBuddy header exists</t>
   </si>
   <si>
-    <t>100ms</t>
+    <t>284ms</t>
   </si>
   <si>
     <t>TC-WEB-UI-003</t>
@@ -77,7 +77,7 @@
     <t>Verify form email input label</t>
   </si>
   <si>
-    <t>48ms</t>
+    <t>69ms</t>
   </si>
   <si>
     <t>TC-WEB-UI-004</t>
@@ -86,7 +86,7 @@
     <t>Verify form password input label</t>
   </si>
   <si>
-    <t>71ms</t>
+    <t>35ms</t>
   </si>
   <si>
     <t>TC-WEB-UI-005</t>
@@ -95,7 +95,7 @@
     <t>Verify Sign In button is present</t>
   </si>
   <si>
-    <t>54ms</t>
+    <t>41ms</t>
   </si>
   <si>
     <t>TC-WEB-UI-006</t>
@@ -104,7 +104,7 @@
     <t>Verify secure access footer notice is present</t>
   </si>
   <si>
-    <t>47ms</t>
+    <t>36ms</t>
   </si>
   <si>
     <t>TC-WEB-UI-007</t>
@@ -113,844 +113,838 @@
     <t>Verify branding subtitle text exists</t>
   </si>
   <si>
+    <t>TC-WEB-UI-008</t>
+  </si>
+  <si>
+    <t>Verify email input field placeholder</t>
+  </si>
+  <si>
+    <t>39ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-009</t>
+  </si>
+  <si>
+    <t>Verify password input field placeholder</t>
+  </si>
+  <si>
+    <t>34ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-010</t>
+  </si>
+  <si>
+    <t>Verify font family CSS on headers</t>
+  </si>
+  <si>
+    <t>40ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-011</t>
+  </si>
+  <si>
+    <t>Verify primary brand color on buttons</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-012</t>
+  </si>
+  <si>
+    <t>Verify centered block layout</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-013</t>
+  </si>
+  <si>
+    <t>Verify responsive structure at mobile width 360px</t>
+  </si>
+  <si>
+    <t>927ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-014</t>
+  </si>
+  <si>
+    <t>Verify responsive structure at tablet width 768px</t>
+  </si>
+  <si>
+    <t>941ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-015</t>
+  </si>
+  <si>
+    <t>Restore browser window maximization state</t>
+  </si>
+  <si>
+    <t>45ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-016</t>
+  </si>
+  <si>
+    <t>Verify HTML tag specification for email input</t>
+  </si>
+  <si>
+    <t>27ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-017</t>
+  </si>
+  <si>
+    <t>Verify HTML tag specification for password input</t>
+  </si>
+  <si>
+    <t>55ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-018</t>
+  </si>
+  <si>
+    <t>Verify card wrapper styles (border-radius)</t>
+  </si>
+  <si>
+    <t>49ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-019</t>
+  </si>
+  <si>
+    <t>Verify background styling matches design spec</t>
+  </si>
+  <si>
+    <t>44ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-020</t>
+  </si>
+  <si>
+    <t>Verify focus state click handler does not crash</t>
+  </si>
+  <si>
+    <t>147ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-021</t>
+  </si>
+  <si>
+    <t>Verify top-level container viewport classes</t>
+  </si>
+  <si>
+    <t>57ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-022</t>
+  </si>
+  <si>
+    <t>Verify branding and form division layout margins</t>
+  </si>
+  <si>
+    <t>38ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-023</t>
+  </si>
+  <si>
+    <t>Verify clear textual contrast for reader accessibility</t>
+  </si>
+  <si>
+    <t>53ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-024</t>
+  </si>
+  <si>
+    <t>Verify page scales properly without layout clipping</t>
+  </si>
+  <si>
+    <t>33ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-025</t>
+  </si>
+  <si>
+    <t>Verify smooth interactive transitions on button inputs</t>
+  </si>
+  <si>
+    <t>31ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-001</t>
+  </si>
+  <si>
+    <t>Functional</t>
+  </si>
+  <si>
+    <t>Verify invalid login rejection message</t>
+  </si>
+  <si>
+    <t>1427ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-002</t>
+  </si>
+  <si>
+    <t>Verify rejection of nonexistent email</t>
+  </si>
+  <si>
+    <t>1220ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-003</t>
+  </si>
+  <si>
+    <t>Verify successful login with valid credentials redirects to Dashboard</t>
+  </si>
+  <si>
+    <t>2197ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-004</t>
+  </si>
+  <si>
+    <t>Verify dashboard displays Total Customers count</t>
+  </si>
+  <si>
+    <t>304ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-005</t>
+  </si>
+  <si>
+    <t>Verify dashboard displays Active Sales count</t>
+  </si>
+  <si>
+    <t>46ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-006</t>
+  </si>
+  <si>
+    <t>Verify dashboard displays Pending Installments count</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-007</t>
+  </si>
+  <si>
+    <t>Verify dashboard displays Today's Due count</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-008</t>
+  </si>
+  <si>
+    <t>Verify dashboard displays Outstanding Balance amount</t>
+  </si>
+  <si>
+    <t>58ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-009</t>
+  </si>
+  <si>
+    <t>Navigate to customers page and verify header</t>
+  </si>
+  <si>
+    <t>232ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-010</t>
+  </si>
+  <si>
+    <t>Verify add new customer input inputs are present</t>
+  </si>
+  <si>
+    <t>80ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-011</t>
+  </si>
+  <si>
+    <t>Verify customer creation and entry addition to table</t>
+  </si>
+  <si>
+    <t>2614ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-012</t>
+  </si>
+  <si>
+    <t>Verify presence of seeded customer</t>
+  </si>
+  <si>
+    <t>52ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-013</t>
+  </si>
+  <si>
+    <t>Navigate to specific customer profile page</t>
+  </si>
+  <si>
+    <t>1424ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-014</t>
+  </si>
+  <si>
+    <t>Verify phone number exists on profile detail bar</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-015</t>
+  </si>
+  <si>
+    <t>Verify Total Amount financial card is 1000 INR</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-016</t>
+  </si>
+  <si>
+    <t>Verify Paid Amount financial card is 0 INR</t>
+  </si>
+  <si>
     <t>51ms</t>
   </si>
   <si>
-    <t>TC-WEB-UI-008</t>
-  </si>
-  <si>
-    <t>Verify email input field placeholder</t>
-  </si>
-  <si>
-    <t>53ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UI-009</t>
-  </si>
-  <si>
-    <t>Verify password input field placeholder</t>
-  </si>
-  <si>
-    <t>49ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UI-010</t>
-  </si>
-  <si>
-    <t>Verify font family CSS on headers</t>
-  </si>
-  <si>
-    <t>70ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UI-011</t>
-  </si>
-  <si>
-    <t>Verify primary brand color on buttons</t>
-  </si>
-  <si>
-    <t>45ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UI-012</t>
-  </si>
-  <si>
-    <t>Verify centered block layout</t>
-  </si>
-  <si>
-    <t>TC-WEB-UI-013</t>
-  </si>
-  <si>
-    <t>Verify responsive structure at mobile width 360px</t>
-  </si>
-  <si>
-    <t>947ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UI-014</t>
-  </si>
-  <si>
-    <t>Verify responsive structure at tablet width 768px</t>
-  </si>
-  <si>
-    <t>933ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UI-015</t>
-  </si>
-  <si>
-    <t>Restore browser window maximization state</t>
-  </si>
-  <si>
-    <t>43ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UI-016</t>
-  </si>
-  <si>
-    <t>Verify HTML tag specification for email input</t>
-  </si>
-  <si>
-    <t>57ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UI-017</t>
-  </si>
-  <si>
-    <t>Verify HTML tag specification for password input</t>
-  </si>
-  <si>
-    <t>62ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UI-018</t>
-  </si>
-  <si>
-    <t>Verify card wrapper styles (border-radius)</t>
-  </si>
-  <si>
-    <t>60ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UI-019</t>
-  </si>
-  <si>
-    <t>Verify background styling matches design spec</t>
-  </si>
-  <si>
-    <t>78ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UI-020</t>
-  </si>
-  <si>
-    <t>Verify focus state click handler does not crash</t>
-  </si>
-  <si>
-    <t>186ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UI-021</t>
-  </si>
-  <si>
-    <t>Verify top-level container viewport classes</t>
-  </si>
-  <si>
-    <t>63ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UI-022</t>
-  </si>
-  <si>
-    <t>Verify branding and form division layout margins</t>
-  </si>
-  <si>
-    <t>40ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UI-023</t>
-  </si>
-  <si>
-    <t>Verify clear textual contrast for reader accessibility</t>
-  </si>
-  <si>
-    <t>42ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UI-024</t>
-  </si>
-  <si>
-    <t>Verify page scales properly without layout clipping</t>
+    <t>TC-WEB-FUNC-017</t>
+  </si>
+  <si>
+    <t>Verify Outstanding Balance financial card is 1000 INR</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-018</t>
+  </si>
+  <si>
+    <t>Verify E2E Test Item pending sale is loaded in sales list</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-019</t>
+  </si>
+  <si>
+    <t>Verify redirect to record payment page</t>
+  </si>
+  <si>
+    <t>922ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-020</t>
+  </si>
+  <si>
+    <t>Verify remaining balance display match before payment</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-021</t>
+  </si>
+  <si>
+    <t>Record payment E2E execution and redirection validation</t>
+  </si>
+  <si>
+    <t>3425ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-022</t>
+  </si>
+  <si>
+    <t>Verify Outstanding Balance updates to 800 INR in customer card</t>
+  </si>
+  <si>
+    <t>1363ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-023</t>
+  </si>
+  <si>
+    <t>Verify Paid Amount updates to 200 INR in customer card</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-024</t>
+  </si>
+  <si>
+    <t>Verify recorded payment entry list matches mode UPI</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-025</t>
+  </si>
+  <si>
+    <t>Verify sales management index loads properly</t>
+  </si>
+  <si>
+    <t>754ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-026</t>
+  </si>
+  <si>
+    <t>Verify sales search filter works properly</t>
+  </si>
+  <si>
+    <t>774ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-027</t>
+  </si>
+  <si>
+    <t>Navigate to Create New Sale form</t>
+  </si>
+  <si>
+    <t>791ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-028</t>
+  </si>
+  <si>
+    <t>Verify total amount computed automatically (2 x 500 = 1000)</t>
+  </si>
+  <si>
+    <t>701ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-029</t>
+  </si>
+  <si>
+    <t>Create sale and verify redirect back to sales table</t>
+  </si>
+  <si>
+    <t>463ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-030</t>
+  </si>
+  <si>
+    <t>Verify Payments page path and title</t>
+  </si>
+  <si>
+    <t>848ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-031</t>
+  </si>
+  <si>
+    <t>Verify E2E transaction exists in master list</t>
+  </si>
+  <si>
+    <t>82ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-032</t>
+  </si>
+  <si>
+    <t>Verify Ledger Book page loads</t>
+  </si>
+  <si>
+    <t>900ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-033</t>
+  </si>
+  <si>
+    <t>Verify ledger records contain client name</t>
+  </si>
+  <si>
+    <t>61ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-034</t>
+  </si>
+  <si>
+    <t>Verify Installments page title</t>
+  </si>
+  <si>
+    <t>672ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-035</t>
+  </si>
+  <si>
+    <t>Verify customer details exist on installment board</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-036</t>
+  </si>
+  <si>
+    <t>Verify direct Dashboard URL redirect</t>
+  </si>
+  <si>
+    <t>259ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-037</t>
+  </si>
+  <si>
+    <t>Verify customer data updates dynamically on UI edit</t>
+  </si>
+  <si>
+    <t>4735ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-038</t>
+  </si>
+  <si>
+    <t>Verify logout route terminates session and redirects to sign in</t>
+  </si>
+  <si>
+    <t>917ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-039</t>
+  </si>
+  <si>
+    <t>Verify unauthorized dashboard access redirects to login</t>
+  </si>
+  <si>
+    <t>2154ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-040</t>
+  </si>
+  <si>
+    <t>Verify unauthorized customer details access redirects to login</t>
+  </si>
+  <si>
+    <t>2557ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UNIT-001</t>
+  </si>
+  <si>
+    <t>Unit</t>
+  </si>
+  <si>
+    <t>Test formatCurrency formatting positive amount</t>
+  </si>
+  <si>
+    <t>84ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UNIT-002</t>
+  </si>
+  <si>
+    <t>Test formatCurrency formatting zero amount</t>
+  </si>
+  <si>
+    <t>1ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UNIT-003</t>
+  </si>
+  <si>
+    <t>Test formatCurrency formatting negative amount</t>
+  </si>
+  <si>
+    <t>TC-WEB-UNIT-004</t>
+  </si>
+  <si>
+    <t>Test formatCurrency formatting large millions scale amount</t>
+  </si>
+  <si>
+    <t>TC-WEB-UNIT-005</t>
+  </si>
+  <si>
+    <t>Test formatCurrency decimal rounding functionality</t>
+  </si>
+  <si>
+    <t>TC-WEB-UNIT-006</t>
+  </si>
+  <si>
+    <t>Test formatDate string matching date details</t>
+  </si>
+  <si>
+    <t>15ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UNIT-007</t>
+  </si>
+  <si>
+    <t>Test formatDate fallback for null values</t>
+  </si>
+  <si>
+    <t>0ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UNIT-008</t>
+  </si>
+  <si>
+    <t>Test formatDate fallback for 0 value</t>
+  </si>
+  <si>
+    <t>TC-WEB-UNIT-009</t>
+  </si>
+  <si>
+    <t>Test formatDateTime details formatting</t>
+  </si>
+  <si>
+    <t>2ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UNIT-010</t>
+  </si>
+  <si>
+    <t>Test formatDateTime null timestamp handling</t>
+  </si>
+  <si>
+    <t>TC-WEB-UNIT-011</t>
+  </si>
+  <si>
+    <t>Verify email validation for valid string</t>
+  </si>
+  <si>
+    <t>TC-WEB-UNIT-012</t>
+  </si>
+  <si>
+    <t>Verify email validation blocks missing TLD</t>
+  </si>
+  <si>
+    <t>TC-WEB-UNIT-013</t>
+  </si>
+  <si>
+    <t>Verify email validation blocks missing alias prefix</t>
+  </si>
+  <si>
+    <t>TC-WEB-UNIT-014</t>
+  </si>
+  <si>
+    <t>Verify phone validation for standard 10 digit number</t>
+  </si>
+  <si>
+    <t>TC-WEB-UNIT-015</t>
+  </si>
+  <si>
+    <t>Verify phone validation blocks short length</t>
+  </si>
+  <si>
+    <t>TC-WEB-UNIT-016</t>
+  </si>
+  <si>
+    <t>Verify phone validation blocks alphabetic characters</t>
+  </si>
+  <si>
+    <t>TC-WEB-UNIT-017</t>
+  </si>
+  <si>
+    <t>Verify interest formula multiplication logic</t>
+  </si>
+  <si>
+    <t>TC-WEB-UNIT-018</t>
+  </si>
+  <si>
+    <t>Verify installment partitioning amount division</t>
+  </si>
+  <si>
+    <t>TC-WEB-UNIT-019</t>
+  </si>
+  <si>
+    <t>Verify remaining balance arithmetic subtraction</t>
+  </si>
+  <si>
+    <t>TC-WEB-UNIT-020</t>
+  </si>
+  <si>
+    <t>Verify mock environment manifest validator passes</t>
+  </si>
+  <si>
+    <t>TC-WEB-VAL-001</t>
+  </si>
+  <si>
+    <t>Validation</t>
+  </si>
+  <si>
+    <t>Verify email required constraint is enabled on form</t>
+  </si>
+  <si>
+    <t>411ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-VAL-002</t>
+  </si>
+  <si>
+    <t>Verify password required constraint is enabled on form</t>
   </si>
   <si>
     <t>37ms</t>
   </si>
   <si>
-    <t>TC-WEB-UI-025</t>
-  </si>
-  <si>
-    <t>Verify smooth interactive transitions on button inputs</t>
-  </si>
-  <si>
-    <t>35ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-001</t>
-  </si>
-  <si>
-    <t>Functional</t>
-  </si>
-  <si>
-    <t>Verify invalid login rejection message</t>
-  </si>
-  <si>
-    <t>1946ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-002</t>
-  </si>
-  <si>
-    <t>Verify rejection of nonexistent email</t>
-  </si>
-  <si>
-    <t>1564ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-003</t>
-  </si>
-  <si>
-    <t>Verify successful login with valid credentials redirects to Dashboard</t>
-  </si>
-  <si>
-    <t>2296ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-004</t>
-  </si>
-  <si>
-    <t>Verify dashboard displays Total Customers count</t>
-  </si>
-  <si>
-    <t>299ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-005</t>
-  </si>
-  <si>
-    <t>Verify dashboard displays Active Sales count</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-006</t>
-  </si>
-  <si>
-    <t>Verify dashboard displays Pending Installments count</t>
-  </si>
-  <si>
-    <t>34ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-007</t>
-  </si>
-  <si>
-    <t>Verify dashboard displays Today's Due count</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-008</t>
-  </si>
-  <si>
-    <t>Verify dashboard displays Outstanding Balance amount</t>
-  </si>
-  <si>
-    <t>33ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-009</t>
-  </si>
-  <si>
-    <t>Navigate to customers page and verify header</t>
-  </si>
-  <si>
-    <t>276ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-010</t>
-  </si>
-  <si>
-    <t>Verify add new customer input inputs are present</t>
-  </si>
-  <si>
-    <t>83ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-011</t>
-  </si>
-  <si>
-    <t>Verify customer creation and entry addition to table</t>
-  </si>
-  <si>
-    <t>2658ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-012</t>
-  </si>
-  <si>
-    <t>Verify presence of seeded customer</t>
-  </si>
-  <si>
-    <t>36ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-013</t>
-  </si>
-  <si>
-    <t>Navigate to specific customer profile page</t>
-  </si>
-  <si>
-    <t>1209ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-014</t>
-  </si>
-  <si>
-    <t>Verify phone number exists on profile detail bar</t>
-  </si>
-  <si>
-    <t>50ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-015</t>
-  </si>
-  <si>
-    <t>Verify Total Amount financial card is 1000 INR</t>
-  </si>
-  <si>
-    <t>55ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-016</t>
-  </si>
-  <si>
-    <t>Verify Paid Amount financial card is 0 INR</t>
-  </si>
-  <si>
-    <t>56ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-017</t>
-  </si>
-  <si>
-    <t>Verify Outstanding Balance financial card is 1000 INR</t>
+    <t>TC-WEB-VAL-003</t>
+  </si>
+  <si>
+    <t>Verify browser client blocks submissions for invalid email inputs</t>
+  </si>
+  <si>
+    <t>257ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-VAL-004</t>
+  </si>
+  <si>
+    <t>Verify character bounds for data buffers limit to 255 characters</t>
+  </si>
+  <si>
+    <t>TC-WEB-VAL-005</t>
+  </si>
+  <si>
+    <t>Verify customer creation form prevents empty submit</t>
+  </si>
+  <si>
+    <t>3671ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-VAL-006</t>
+  </si>
+  <si>
+    <t>Verify phone input uses tel semantic element type</t>
+  </si>
+  <si>
+    <t>TC-WEB-VAL-007</t>
+  </si>
+  <si>
+    <t>Verify sale quantity requires positive minimum value (&gt; 0)</t>
+  </si>
+  <si>
+    <t>1154ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-VAL-008</t>
+  </si>
+  <si>
+    <t>Verify unit price input restricts negative numbers</t>
+  </si>
+  <si>
+    <t>TC-WEB-VAL-009</t>
+  </si>
+  <si>
+    <t>Verify script tag input text does not trigger native alerts</t>
+  </si>
+  <si>
+    <t>Security</t>
+  </si>
+  <si>
+    <t>2270ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-VAL-010</t>
+  </si>
+  <si>
+    <t>Verify database adapter parameters parameterized input query parsing</t>
+  </si>
+  <si>
+    <t>TC-WEB-VAL-011</t>
+  </si>
+  <si>
+    <t>Verify error prevents overpayment collections</t>
+  </si>
+  <si>
+    <t>2883ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-VAL-012</t>
+  </si>
+  <si>
+    <t>Verify collection input restricts 0 value submissions</t>
+  </si>
+  <si>
+    <t>1453ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-VAL-013</t>
+  </si>
+  <si>
+    <t>Verify Firestore writes match schema constraints</t>
+  </si>
+  <si>
+    <t>TC-WEB-VAL-014</t>
+  </si>
+  <si>
+    <t>Verify wildcard URLs redirect to main route base</t>
+  </si>
+  <si>
+    <t>2165ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-VAL-015</t>
+  </si>
+  <si>
+    <t>Verify HTML password hidden mask attribute config</t>
+  </si>
+  <si>
+    <t>1008ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-DEP-001</t>
+  </si>
+  <si>
+    <t>Deployment</t>
+  </si>
+  <si>
+    <t>Verify load paint FCP under 2.5s threshold</t>
+  </si>
+  <si>
+    <t>Performance</t>
+  </si>
+  <si>
+    <t>497ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-DEP-002</t>
+  </si>
+  <si>
+    <t>Verify full render transition load time under limit</t>
+  </si>
+  <si>
+    <t>1660ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-DEP-003</t>
+  </si>
+  <si>
+    <t>Verify DNS host domain matches Vercel production edge</t>
+  </si>
+  <si>
+    <t>TC-WEB-DEP-004</t>
+  </si>
+  <si>
+    <t>Verify favicon.ico endpoint yields clean HTTP status</t>
+  </si>
+  <si>
+    <t>439ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-DEP-005</t>
+  </si>
+  <si>
+    <t>Verify production connection protocol HTTPS encryption is active</t>
+  </si>
+  <si>
+    <t>TC-WEB-DEP-006</t>
+  </si>
+  <si>
+    <t>Verify head links contain manifest registration details</t>
+  </si>
+  <si>
+    <t>167ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-DEP-007</t>
+  </si>
+  <si>
+    <t>Verify console logs have no severe exceptions during login page session</t>
+  </si>
+  <si>
+    <t>6ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-DEP-008</t>
+  </si>
+  <si>
+    <t>Verify standard responsive layouts align horizontally</t>
   </si>
   <si>
     <t>65ms</t>
   </si>
   <si>
-    <t>TC-WEB-FUNC-018</t>
-  </si>
-  <si>
-    <t>Verify E2E Test Item pending sale is loaded in sales list</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-019</t>
-  </si>
-  <si>
-    <t>Verify redirect to record payment page</t>
-  </si>
-  <si>
-    <t>939ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-020</t>
-  </si>
-  <si>
-    <t>Verify remaining balance display match before payment</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-021</t>
-  </si>
-  <si>
-    <t>Record payment E2E execution and redirection validation</t>
-  </si>
-  <si>
-    <t>3680ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-022</t>
-  </si>
-  <si>
-    <t>Verify Outstanding Balance updates to 800 INR in customer card</t>
-  </si>
-  <si>
-    <t>1797ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-023</t>
-  </si>
-  <si>
-    <t>Verify Paid Amount updates to 200 INR in customer card</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-024</t>
-  </si>
-  <si>
-    <t>Verify recorded payment entry list matches mode UPI</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-025</t>
-  </si>
-  <si>
-    <t>Verify sales management index loads properly</t>
-  </si>
-  <si>
-    <t>975ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-026</t>
-  </si>
-  <si>
-    <t>Verify sales search filter works properly</t>
-  </si>
-  <si>
-    <t>861ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-027</t>
-  </si>
-  <si>
-    <t>Navigate to Create New Sale form</t>
-  </si>
-  <si>
-    <t>1477ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-028</t>
-  </si>
-  <si>
-    <t>Verify total amount computed automatically (2 x 500 = 1000)</t>
-  </si>
-  <si>
-    <t>700ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-029</t>
-  </si>
-  <si>
-    <t>Create sale and verify redirect back to sales table</t>
-  </si>
-  <si>
-    <t>547ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-030</t>
-  </si>
-  <si>
-    <t>Verify Payments page path and title</t>
-  </si>
-  <si>
-    <t>1150ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-031</t>
-  </si>
-  <si>
-    <t>Verify E2E transaction exists in master list</t>
-  </si>
-  <si>
-    <t>117ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-032</t>
-  </si>
-  <si>
-    <t>Verify Ledger Book page loads</t>
-  </si>
-  <si>
-    <t>748ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-033</t>
-  </si>
-  <si>
-    <t>Verify ledger records contain client name</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-034</t>
-  </si>
-  <si>
-    <t>Verify Installments page title</t>
-  </si>
-  <si>
-    <t>1003ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-035</t>
-  </si>
-  <si>
-    <t>Verify customer details exist on installment board</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-036</t>
-  </si>
-  <si>
-    <t>Verify direct Dashboard URL redirect</t>
-  </si>
-  <si>
-    <t>570ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-037</t>
-  </si>
-  <si>
-    <t>Verify customer data updates dynamically on UI edit</t>
-  </si>
-  <si>
-    <t>5246ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-038</t>
-  </si>
-  <si>
-    <t>Verify logout route terminates session and redirects to sign in</t>
-  </si>
-  <si>
-    <t>1955ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-039</t>
-  </si>
-  <si>
-    <t>Verify unauthorized dashboard access redirects to login</t>
-  </si>
-  <si>
-    <t>3166ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-040</t>
-  </si>
-  <si>
-    <t>Verify unauthorized customer details access redirects to login</t>
-  </si>
-  <si>
-    <t>2256ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UNIT-001</t>
-  </si>
-  <si>
-    <t>Unit</t>
-  </si>
-  <si>
-    <t>Test formatCurrency formatting positive amount</t>
-  </si>
-  <si>
-    <t>73ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UNIT-002</t>
-  </si>
-  <si>
-    <t>Test formatCurrency formatting zero amount</t>
-  </si>
-  <si>
-    <t>0ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UNIT-003</t>
-  </si>
-  <si>
-    <t>Test formatCurrency formatting negative amount</t>
-  </si>
-  <si>
-    <t>1ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UNIT-004</t>
-  </si>
-  <si>
-    <t>Test formatCurrency formatting large millions scale amount</t>
-  </si>
-  <si>
-    <t>TC-WEB-UNIT-005</t>
-  </si>
-  <si>
-    <t>Test formatCurrency decimal rounding functionality</t>
-  </si>
-  <si>
-    <t>TC-WEB-UNIT-006</t>
-  </si>
-  <si>
-    <t>Test formatDate string matching date details</t>
-  </si>
-  <si>
-    <t>20ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UNIT-007</t>
-  </si>
-  <si>
-    <t>Test formatDate fallback for null values</t>
-  </si>
-  <si>
-    <t>TC-WEB-UNIT-008</t>
-  </si>
-  <si>
-    <t>Test formatDate fallback for 0 value</t>
-  </si>
-  <si>
-    <t>TC-WEB-UNIT-009</t>
-  </si>
-  <si>
-    <t>Test formatDateTime details formatting</t>
-  </si>
-  <si>
-    <t>17ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UNIT-010</t>
-  </si>
-  <si>
-    <t>Test formatDateTime null timestamp handling</t>
-  </si>
-  <si>
-    <t>TC-WEB-UNIT-011</t>
-  </si>
-  <si>
-    <t>Verify email validation for valid string</t>
-  </si>
-  <si>
-    <t>TC-WEB-UNIT-012</t>
-  </si>
-  <si>
-    <t>Verify email validation blocks missing TLD</t>
-  </si>
-  <si>
-    <t>TC-WEB-UNIT-013</t>
-  </si>
-  <si>
-    <t>Verify email validation blocks missing alias prefix</t>
-  </si>
-  <si>
-    <t>TC-WEB-UNIT-014</t>
-  </si>
-  <si>
-    <t>Verify phone validation for standard 10 digit number</t>
-  </si>
-  <si>
-    <t>TC-WEB-UNIT-015</t>
-  </si>
-  <si>
-    <t>Verify phone validation blocks short length</t>
-  </si>
-  <si>
-    <t>TC-WEB-UNIT-016</t>
-  </si>
-  <si>
-    <t>Verify phone validation blocks alphabetic characters</t>
-  </si>
-  <si>
-    <t>TC-WEB-UNIT-017</t>
-  </si>
-  <si>
-    <t>Verify interest formula multiplication logic</t>
-  </si>
-  <si>
-    <t>TC-WEB-UNIT-018</t>
-  </si>
-  <si>
-    <t>Verify installment partitioning amount division</t>
-  </si>
-  <si>
-    <t>TC-WEB-UNIT-019</t>
-  </si>
-  <si>
-    <t>Verify remaining balance arithmetic subtraction</t>
-  </si>
-  <si>
-    <t>TC-WEB-UNIT-020</t>
-  </si>
-  <si>
-    <t>Verify mock environment manifest validator passes</t>
-  </si>
-  <si>
-    <t>TC-WEB-VAL-001</t>
-  </si>
-  <si>
-    <t>Validation</t>
-  </si>
-  <si>
-    <t>Verify email required constraint is enabled on form</t>
-  </si>
-  <si>
-    <t>623ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-VAL-002</t>
-  </si>
-  <si>
-    <t>Verify password required constraint is enabled on form</t>
-  </si>
-  <si>
-    <t>31ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-VAL-003</t>
-  </si>
-  <si>
-    <t>Verify browser client blocks submissions for invalid email inputs</t>
-  </si>
-  <si>
-    <t>239ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-VAL-004</t>
-  </si>
-  <si>
-    <t>Verify character bounds for data buffers limit to 255 characters</t>
-  </si>
-  <si>
-    <t>TC-WEB-VAL-005</t>
-  </si>
-  <si>
-    <t>Verify customer creation form prevents empty submit</t>
-  </si>
-  <si>
-    <t>7364ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-VAL-006</t>
-  </si>
-  <si>
-    <t>Verify phone input uses tel semantic element type</t>
-  </si>
-  <si>
-    <t>TC-WEB-VAL-007</t>
-  </si>
-  <si>
-    <t>Verify sale quantity requires positive minimum value (&gt; 0)</t>
-  </si>
-  <si>
-    <t>2585ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-VAL-008</t>
-  </si>
-  <si>
-    <t>Verify unit price input restricts negative numbers</t>
-  </si>
-  <si>
-    <t>TC-WEB-VAL-009</t>
-  </si>
-  <si>
-    <t>Verify script tag input text does not trigger native alerts</t>
-  </si>
-  <si>
-    <t>Security</t>
-  </si>
-  <si>
-    <t>3341ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-VAL-010</t>
-  </si>
-  <si>
-    <t>Verify database adapter parameters parameterized input query parsing</t>
-  </si>
-  <si>
-    <t>TC-WEB-VAL-011</t>
-  </si>
-  <si>
-    <t>Verify error prevents overpayment collections</t>
-  </si>
-  <si>
-    <t>2484ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-VAL-012</t>
-  </si>
-  <si>
-    <t>Verify collection input restricts 0 value submissions</t>
-  </si>
-  <si>
-    <t>1416ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-VAL-013</t>
-  </si>
-  <si>
-    <t>Verify Firestore writes match schema constraints</t>
-  </si>
-  <si>
-    <t>TC-WEB-VAL-014</t>
-  </si>
-  <si>
-    <t>Verify wildcard URLs redirect to main route base</t>
-  </si>
-  <si>
-    <t>4026ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-VAL-015</t>
-  </si>
-  <si>
-    <t>Verify HTML password hidden mask attribute config</t>
-  </si>
-  <si>
-    <t>1271ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-DEP-001</t>
-  </si>
-  <si>
-    <t>Deployment</t>
-  </si>
-  <si>
-    <t>Verify load paint FCP under 2.5s threshold</t>
-  </si>
-  <si>
-    <t>Performance</t>
-  </si>
-  <si>
-    <t>819ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-DEP-002</t>
-  </si>
-  <si>
-    <t>Verify full render transition load time under limit</t>
-  </si>
-  <si>
-    <t>1705ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-DEP-003</t>
-  </si>
-  <si>
-    <t>Verify DNS host domain matches Vercel production edge</t>
-  </si>
-  <si>
-    <t>TC-WEB-DEP-004</t>
-  </si>
-  <si>
-    <t>Verify favicon.ico endpoint yields clean HTTP status</t>
-  </si>
-  <si>
-    <t>250ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-DEP-005</t>
-  </si>
-  <si>
-    <t>Verify production connection protocol HTTPS encryption is active</t>
-  </si>
-  <si>
-    <t>TC-WEB-DEP-006</t>
-  </si>
-  <si>
-    <t>Verify head links contain manifest registration details</t>
-  </si>
-  <si>
-    <t>TC-WEB-DEP-007</t>
-  </si>
-  <si>
-    <t>Verify console logs have no severe exceptions during login page session</t>
-  </si>
-  <si>
-    <t>11ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-DEP-008</t>
-  </si>
-  <si>
-    <t>Verify standard responsive layouts align horizontally</t>
-  </si>
-  <si>
     <t>TC-WEB-DEP-009</t>
   </si>
   <si>
     <t>Verify DOM count index scales cleanly</t>
   </si>
   <si>
-    <t>14ms</t>
+    <t>16ms</t>
   </si>
   <si>
     <t>TC-WEB-DEP-010</t>
@@ -1570,7 +1564,7 @@
         <v>11</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="G8" s="2" t="s">
         <v>13</v>
@@ -1578,13 +1572,13 @@
     </row>
     <row r="9" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>10</v>
@@ -1593,7 +1587,7 @@
         <v>11</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="G9" s="2" t="s">
         <v>13</v>
@@ -1601,13 +1595,13 @@
     </row>
     <row r="10" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D10" s="2" t="s">
         <v>10</v>
@@ -1616,7 +1610,7 @@
         <v>11</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="G10" s="2" t="s">
         <v>13</v>
@@ -1624,13 +1618,13 @@
     </row>
     <row r="11" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B11" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D11" s="2" t="s">
         <v>10</v>
@@ -1639,7 +1633,7 @@
         <v>11</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G11" s="2" t="s">
         <v>13</v>
@@ -1647,13 +1641,13 @@
     </row>
     <row r="12" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B12" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D12" s="2" t="s">
         <v>10</v>
@@ -1662,7 +1656,7 @@
         <v>11</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>43</v>
+        <v>22</v>
       </c>
       <c r="G12" s="2" t="s">
         <v>13</v>
@@ -1670,13 +1664,13 @@
     </row>
     <row r="13" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B13" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="D13" s="2" t="s">
         <v>10</v>
@@ -1685,7 +1679,7 @@
         <v>11</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="G13" s="2" t="s">
         <v>13</v>
@@ -1693,13 +1687,13 @@
     </row>
     <row r="14" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B14" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="D14" s="2" t="s">
         <v>10</v>
@@ -1708,7 +1702,7 @@
         <v>11</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="G14" s="2" t="s">
         <v>13</v>
@@ -1716,13 +1710,13 @@
     </row>
     <row r="15" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B15" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="D15" s="2" t="s">
         <v>10</v>
@@ -1731,7 +1725,7 @@
         <v>11</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="G15" s="2" t="s">
         <v>13</v>
@@ -1739,13 +1733,13 @@
     </row>
     <row r="16" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B16" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="D16" s="2" t="s">
         <v>10</v>
@@ -1754,7 +1748,7 @@
         <v>11</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="G16" s="2" t="s">
         <v>13</v>
@@ -1762,13 +1756,13 @@
     </row>
     <row r="17" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B17" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="D17" s="2" t="s">
         <v>10</v>
@@ -1777,7 +1771,7 @@
         <v>11</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="G17" s="2" t="s">
         <v>13</v>
@@ -1785,13 +1779,13 @@
     </row>
     <row r="18" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B18" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="D18" s="2" t="s">
         <v>10</v>
@@ -1800,7 +1794,7 @@
         <v>11</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="G18" s="2" t="s">
         <v>13</v>
@@ -1808,13 +1802,13 @@
     </row>
     <row r="19" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B19" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="D19" s="2" t="s">
         <v>10</v>
@@ -1823,7 +1817,7 @@
         <v>11</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="G19" s="2" t="s">
         <v>13</v>
@@ -1831,13 +1825,13 @@
     </row>
     <row r="20" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="B20" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="D20" s="2" t="s">
         <v>10</v>
@@ -1846,7 +1840,7 @@
         <v>11</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="G20" s="2" t="s">
         <v>13</v>
@@ -1854,13 +1848,13 @@
     </row>
     <row r="21" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="B21" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="D21" s="2" t="s">
         <v>10</v>
@@ -1869,7 +1863,7 @@
         <v>11</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="G21" s="2" t="s">
         <v>13</v>
@@ -1877,13 +1871,13 @@
     </row>
     <row r="22" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B22" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="D22" s="2" t="s">
         <v>10</v>
@@ -1892,7 +1886,7 @@
         <v>11</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="G22" s="2" t="s">
         <v>13</v>
@@ -1900,13 +1894,13 @@
     </row>
     <row r="23" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="B23" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="D23" s="2" t="s">
         <v>10</v>
@@ -1915,7 +1909,7 @@
         <v>11</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="G23" s="2" t="s">
         <v>13</v>
@@ -1923,13 +1917,13 @@
     </row>
     <row r="24" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B24" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="D24" s="2" t="s">
         <v>10</v>
@@ -1938,7 +1932,7 @@
         <v>11</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="G24" s="2" t="s">
         <v>13</v>
@@ -1946,13 +1940,13 @@
     </row>
     <row r="25" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="B25" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="D25" s="2" t="s">
         <v>10</v>
@@ -1961,7 +1955,7 @@
         <v>11</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="G25" s="2" t="s">
         <v>13</v>
@@ -1969,13 +1963,13 @@
     </row>
     <row r="26" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="B26" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="D26" s="2" t="s">
         <v>10</v>
@@ -1984,7 +1978,7 @@
         <v>11</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="G26" s="2" t="s">
         <v>13</v>
@@ -2035,22 +2029,22 @@
     </row>
     <row r="2" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="D2" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>86</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>88</v>
       </c>
       <c r="G2" s="2" t="s">
         <v>13</v>
@@ -2058,22 +2052,22 @@
     </row>
     <row r="3" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F3" s="2" t="s">
         <v>89</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>91</v>
       </c>
       <c r="G3" s="2" t="s">
         <v>13</v>
@@ -2081,22 +2075,22 @@
     </row>
     <row r="4" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F4" s="2" t="s">
         <v>92</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>94</v>
       </c>
       <c r="G4" s="2" t="s">
         <v>13</v>
@@ -2104,22 +2098,22 @@
     </row>
     <row r="5" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F5" s="2" t="s">
         <v>95</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>96</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F5" s="2" t="s">
-        <v>97</v>
       </c>
       <c r="G5" s="2" t="s">
         <v>13</v>
@@ -2127,22 +2121,22 @@
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F6" s="2" t="s">
         <v>98</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>99</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>31</v>
       </c>
       <c r="G6" s="2" t="s">
         <v>13</v>
@@ -2150,22 +2144,22 @@
     </row>
     <row r="7" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="C7" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="B7" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>101</v>
-      </c>
       <c r="D7" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="E7" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>102</v>
+        <v>64</v>
       </c>
       <c r="G7" s="2" t="s">
         <v>13</v>
@@ -2173,22 +2167,22 @@
     </row>
     <row r="8" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="E8" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>37</v>
+        <v>76</v>
       </c>
       <c r="G8" s="2" t="s">
         <v>13</v>
@@ -2196,22 +2190,22 @@
     </row>
     <row r="9" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F9" s="2" t="s">
         <v>105</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="E9" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F9" s="2" t="s">
-        <v>107</v>
       </c>
       <c r="G9" s="2" t="s">
         <v>13</v>
@@ -2219,22 +2213,22 @@
     </row>
     <row r="10" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F10" s="2" t="s">
         <v>108</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="E10" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F10" s="2" t="s">
-        <v>110</v>
       </c>
       <c r="G10" s="2" t="s">
         <v>13</v>
@@ -2242,22 +2236,22 @@
     </row>
     <row r="11" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F11" s="2" t="s">
         <v>111</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="E11" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F11" s="2" t="s">
-        <v>113</v>
       </c>
       <c r="G11" s="2" t="s">
         <v>13</v>
@@ -2265,22 +2259,22 @@
     </row>
     <row r="12" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F12" s="2" t="s">
         <v>114</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>115</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="E12" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F12" s="2" t="s">
-        <v>116</v>
       </c>
       <c r="G12" s="2" t="s">
         <v>13</v>
@@ -2288,22 +2282,22 @@
     </row>
     <row r="13" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F13" s="2" t="s">
         <v>117</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>118</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="E13" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F13" s="2" t="s">
-        <v>119</v>
       </c>
       <c r="G13" s="2" t="s">
         <v>13</v>
@@ -2311,22 +2305,22 @@
     </row>
     <row r="14" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F14" s="2" t="s">
         <v>120</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>121</v>
-      </c>
-      <c r="D14" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="E14" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F14" s="2" t="s">
-        <v>122</v>
       </c>
       <c r="G14" s="2" t="s">
         <v>13</v>
@@ -2334,22 +2328,22 @@
     </row>
     <row r="15" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="E15" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>125</v>
+        <v>76</v>
       </c>
       <c r="G15" s="2" t="s">
         <v>13</v>
@@ -2357,22 +2351,22 @@
     </row>
     <row r="16" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="E16" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>128</v>
+        <v>52</v>
       </c>
       <c r="G16" s="2" t="s">
         <v>13</v>
@@ -2380,22 +2374,22 @@
     </row>
     <row r="17" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="E17" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="G17" s="2" t="s">
         <v>13</v>
@@ -2403,22 +2397,22 @@
     </row>
     <row r="18" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="E18" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>134</v>
+        <v>39</v>
       </c>
       <c r="G18" s="2" t="s">
         <v>13</v>
@@ -2426,22 +2420,22 @@
     </row>
     <row r="19" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>136</v>
+        <v>131</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="E19" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>134</v>
+        <v>79</v>
       </c>
       <c r="G19" s="2" t="s">
         <v>13</v>
@@ -2449,22 +2443,22 @@
     </row>
     <row r="20" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="E20" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
       <c r="G20" s="2" t="s">
         <v>13</v>
@@ -2472,22 +2466,22 @@
     </row>
     <row r="21" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>141</v>
+        <v>136</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="E21" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>134</v>
+        <v>28</v>
       </c>
       <c r="G21" s="2" t="s">
         <v>13</v>
@@ -2495,22 +2489,22 @@
     </row>
     <row r="22" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>142</v>
+        <v>137</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="E22" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
       <c r="G22" s="2" t="s">
         <v>13</v>
@@ -2518,22 +2512,22 @@
     </row>
     <row r="23" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
-        <v>145</v>
+        <v>140</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="E23" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>147</v>
+        <v>142</v>
       </c>
       <c r="G23" s="2" t="s">
         <v>13</v>
@@ -2541,22 +2535,22 @@
     </row>
     <row r="24" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>148</v>
+        <v>143</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="E24" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>54</v>
+        <v>33</v>
       </c>
       <c r="G24" s="2" t="s">
         <v>13</v>
@@ -2564,22 +2558,22 @@
     </row>
     <row r="25" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
-        <v>150</v>
+        <v>145</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="E25" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>37</v>
+        <v>22</v>
       </c>
       <c r="G25" s="2" t="s">
         <v>13</v>
@@ -2587,22 +2581,22 @@
     </row>
     <row r="26" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
-        <v>152</v>
+        <v>147</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>153</v>
+        <v>148</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="E26" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>154</v>
+        <v>149</v>
       </c>
       <c r="G26" s="2" t="s">
         <v>13</v>
@@ -2610,22 +2604,22 @@
     </row>
     <row r="27" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
-        <v>155</v>
+        <v>150</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>156</v>
+        <v>151</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="E27" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>157</v>
+        <v>152</v>
       </c>
       <c r="G27" s="2" t="s">
         <v>13</v>
@@ -2633,22 +2627,22 @@
     </row>
     <row r="28" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
-        <v>158</v>
+        <v>153</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="E28" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F28" s="2" t="s">
-        <v>160</v>
+        <v>155</v>
       </c>
       <c r="G28" s="2" t="s">
         <v>13</v>
@@ -2656,22 +2650,22 @@
     </row>
     <row r="29" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
-        <v>161</v>
+        <v>156</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="E29" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F29" s="2" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
       <c r="G29" s="2" t="s">
         <v>13</v>
@@ -2679,22 +2673,22 @@
     </row>
     <row r="30" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
-        <v>164</v>
+        <v>159</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>165</v>
+        <v>160</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="E30" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F30" s="2" t="s">
-        <v>166</v>
+        <v>161</v>
       </c>
       <c r="G30" s="2" t="s">
         <v>13</v>
@@ -2702,22 +2696,22 @@
     </row>
     <row r="31" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
-        <v>167</v>
+        <v>162</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>168</v>
+        <v>163</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="E31" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F31" s="2" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
       <c r="G31" s="2" t="s">
         <v>13</v>
@@ -2725,22 +2719,22 @@
     </row>
     <row r="32" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>171</v>
+        <v>166</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="E32" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F32" s="2" t="s">
-        <v>172</v>
+        <v>167</v>
       </c>
       <c r="G32" s="2" t="s">
         <v>13</v>
@@ -2748,22 +2742,22 @@
     </row>
     <row r="33" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
-        <v>173</v>
+        <v>168</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>174</v>
+        <v>169</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="E33" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F33" s="2" t="s">
-        <v>175</v>
+        <v>170</v>
       </c>
       <c r="G33" s="2" t="s">
         <v>13</v>
@@ -2771,22 +2765,22 @@
     </row>
     <row r="34" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
-        <v>176</v>
+        <v>171</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>177</v>
+        <v>172</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="E34" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F34" s="2" t="s">
-        <v>60</v>
+        <v>173</v>
       </c>
       <c r="G34" s="2" t="s">
         <v>13</v>
@@ -2794,22 +2788,22 @@
     </row>
     <row r="35" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="E35" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F35" s="2" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="G35" s="2" t="s">
         <v>13</v>
@@ -2817,22 +2811,22 @@
     </row>
     <row r="36" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="E36" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F36" s="2" t="s">
-        <v>72</v>
+        <v>117</v>
       </c>
       <c r="G36" s="2" t="s">
         <v>13</v>
@@ -2840,22 +2834,22 @@
     </row>
     <row r="37" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="E37" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F37" s="2" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="G37" s="2" t="s">
         <v>13</v>
@@ -2863,22 +2857,22 @@
     </row>
     <row r="38" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="E38" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F38" s="2" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="G38" s="2" t="s">
         <v>13</v>
@@ -2886,22 +2880,22 @@
     </row>
     <row r="39" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="E39" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F39" s="2" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="G39" s="2" t="s">
         <v>13</v>
@@ -2909,22 +2903,22 @@
     </row>
     <row r="40" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="E40" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F40" s="2" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="G40" s="2" t="s">
         <v>13</v>
@@ -2932,22 +2926,22 @@
     </row>
     <row r="41" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
-        <v>195</v>
+        <v>191</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="E41" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F41" s="2" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="G41" s="2" t="s">
         <v>13</v>
@@ -2998,22 +2992,22 @@
     </row>
     <row r="2" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="E2" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="G2" s="2" t="s">
         <v>13</v>
@@ -3021,22 +3015,22 @@
     </row>
     <row r="3" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="B3" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>199</v>
       </c>
-      <c r="C3" s="2" t="s">
-        <v>203</v>
-      </c>
       <c r="D3" s="2" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="E3" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="G3" s="2" t="s">
         <v>13</v>
@@ -3044,22 +3038,22 @@
     </row>
     <row r="4" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>205</v>
+        <v>201</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="E4" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>207</v>
+        <v>200</v>
       </c>
       <c r="G4" s="2" t="s">
         <v>13</v>
@@ -3067,22 +3061,22 @@
     </row>
     <row r="5" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>208</v>
+        <v>203</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>209</v>
+        <v>204</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="E5" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>207</v>
+        <v>200</v>
       </c>
       <c r="G5" s="2" t="s">
         <v>13</v>
@@ -3090,22 +3084,22 @@
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>210</v>
+        <v>205</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>211</v>
+        <v>206</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="E6" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="G6" s="2" t="s">
         <v>13</v>
@@ -3113,22 +3107,22 @@
     </row>
     <row r="7" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>212</v>
+        <v>207</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>213</v>
+        <v>208</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="E7" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>214</v>
+        <v>209</v>
       </c>
       <c r="G7" s="2" t="s">
         <v>13</v>
@@ -3136,22 +3130,22 @@
     </row>
     <row r="8" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>215</v>
+        <v>210</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>216</v>
+        <v>211</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="E8" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>204</v>
+        <v>212</v>
       </c>
       <c r="G8" s="2" t="s">
         <v>13</v>
@@ -3159,22 +3153,22 @@
     </row>
     <row r="9" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>218</v>
+        <v>214</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="E9" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>204</v>
+        <v>212</v>
       </c>
       <c r="G9" s="2" t="s">
         <v>13</v>
@@ -3182,22 +3176,22 @@
     </row>
     <row r="10" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>219</v>
+        <v>215</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>220</v>
+        <v>216</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="E10" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>221</v>
+        <v>217</v>
       </c>
       <c r="G10" s="2" t="s">
         <v>13</v>
@@ -3205,22 +3199,22 @@
     </row>
     <row r="11" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>222</v>
+        <v>218</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>223</v>
+        <v>219</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="E11" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>204</v>
+        <v>212</v>
       </c>
       <c r="G11" s="2" t="s">
         <v>13</v>
@@ -3228,22 +3222,22 @@
     </row>
     <row r="12" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>224</v>
+        <v>220</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>225</v>
+        <v>221</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="E12" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>204</v>
+        <v>212</v>
       </c>
       <c r="G12" s="2" t="s">
         <v>13</v>
@@ -3251,22 +3245,22 @@
     </row>
     <row r="13" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>226</v>
+        <v>222</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="E13" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>204</v>
+        <v>212</v>
       </c>
       <c r="G13" s="2" t="s">
         <v>13</v>
@@ -3274,22 +3268,22 @@
     </row>
     <row r="14" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>228</v>
+        <v>224</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="E14" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>204</v>
+        <v>212</v>
       </c>
       <c r="G14" s="2" t="s">
         <v>13</v>
@@ -3297,22 +3291,22 @@
     </row>
     <row r="15" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>230</v>
+        <v>226</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>231</v>
+        <v>227</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="E15" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="G15" s="2" t="s">
         <v>13</v>
@@ -3320,22 +3314,22 @@
     </row>
     <row r="16" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>232</v>
+        <v>228</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>233</v>
+        <v>229</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="E16" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>204</v>
+        <v>212</v>
       </c>
       <c r="G16" s="2" t="s">
         <v>13</v>
@@ -3343,22 +3337,22 @@
     </row>
     <row r="17" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>234</v>
+        <v>230</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>235</v>
+        <v>231</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="E17" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>204</v>
+        <v>212</v>
       </c>
       <c r="G17" s="2" t="s">
         <v>13</v>
@@ -3366,22 +3360,22 @@
     </row>
     <row r="18" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>236</v>
+        <v>232</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>237</v>
+        <v>233</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="E18" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>204</v>
+        <v>212</v>
       </c>
       <c r="G18" s="2" t="s">
         <v>13</v>
@@ -3389,22 +3383,22 @@
     </row>
     <row r="19" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>238</v>
+        <v>234</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>239</v>
+        <v>235</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="E19" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>204</v>
+        <v>212</v>
       </c>
       <c r="G19" s="2" t="s">
         <v>13</v>
@@ -3412,22 +3406,22 @@
     </row>
     <row r="20" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>240</v>
+        <v>236</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>241</v>
+        <v>237</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="E20" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>204</v>
+        <v>212</v>
       </c>
       <c r="G20" s="2" t="s">
         <v>13</v>
@@ -3435,22 +3429,22 @@
     </row>
     <row r="21" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>243</v>
+        <v>239</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="E21" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="G21" s="2" t="s">
         <v>13</v>
@@ -3501,22 +3495,22 @@
     </row>
     <row r="2" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>246</v>
+        <v>242</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
       <c r="E2" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>247</v>
+        <v>243</v>
       </c>
       <c r="G2" s="2" t="s">
         <v>13</v>
@@ -3524,22 +3518,22 @@
     </row>
     <row r="3" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>248</v>
+        <v>244</v>
       </c>
       <c r="B3" s="2" t="s">
+        <v>241</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>245</v>
       </c>
-      <c r="C3" s="2" t="s">
-        <v>249</v>
-      </c>
       <c r="D3" s="2" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
       <c r="E3" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>250</v>
+        <v>246</v>
       </c>
       <c r="G3" s="2" t="s">
         <v>13</v>
@@ -3547,22 +3541,22 @@
     </row>
     <row r="4" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>251</v>
+        <v>247</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>252</v>
+        <v>248</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
       <c r="E4" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>253</v>
+        <v>249</v>
       </c>
       <c r="G4" s="2" t="s">
         <v>13</v>
@@ -3570,22 +3564,22 @@
     </row>
     <row r="5" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>254</v>
+        <v>250</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>255</v>
+        <v>251</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
       <c r="E5" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="G5" s="2" t="s">
         <v>13</v>
@@ -3593,22 +3587,22 @@
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>256</v>
+        <v>252</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>257</v>
+        <v>253</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
       <c r="E6" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>258</v>
+        <v>254</v>
       </c>
       <c r="G6" s="2" t="s">
         <v>13</v>
@@ -3616,22 +3610,22 @@
     </row>
     <row r="7" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>259</v>
+        <v>255</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>260</v>
+        <v>256</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
       <c r="E7" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>131</v>
+        <v>64</v>
       </c>
       <c r="G7" s="2" t="s">
         <v>13</v>
@@ -3639,22 +3633,22 @@
     </row>
     <row r="8" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>261</v>
+        <v>257</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>262</v>
+        <v>258</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
       <c r="E8" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>263</v>
+        <v>259</v>
       </c>
       <c r="G8" s="2" t="s">
         <v>13</v>
@@ -3662,22 +3656,22 @@
     </row>
     <row r="9" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>264</v>
+        <v>260</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>265</v>
+        <v>261</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
       <c r="E9" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>34</v>
+        <v>22</v>
       </c>
       <c r="G9" s="2" t="s">
         <v>13</v>
@@ -3685,22 +3679,22 @@
     </row>
     <row r="10" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>266</v>
+        <v>262</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>267</v>
+        <v>263</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>268</v>
+        <v>264</v>
       </c>
       <c r="E10" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>269</v>
+        <v>265</v>
       </c>
       <c r="G10" s="2" t="s">
         <v>13</v>
@@ -3708,22 +3702,22 @@
     </row>
     <row r="11" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>270</v>
+        <v>266</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>271</v>
+        <v>267</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>268</v>
+        <v>264</v>
       </c>
       <c r="E11" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>204</v>
+        <v>212</v>
       </c>
       <c r="G11" s="2" t="s">
         <v>13</v>
@@ -3731,22 +3725,22 @@
     </row>
     <row r="12" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>272</v>
+        <v>268</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>273</v>
+        <v>269</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
       <c r="E12" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>274</v>
+        <v>270</v>
       </c>
       <c r="G12" s="2" t="s">
         <v>13</v>
@@ -3754,22 +3748,22 @@
     </row>
     <row r="13" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>275</v>
+        <v>271</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>276</v>
+        <v>272</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
       <c r="E13" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>277</v>
+        <v>273</v>
       </c>
       <c r="G13" s="2" t="s">
         <v>13</v>
@@ -3777,22 +3771,22 @@
     </row>
     <row r="14" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>278</v>
+        <v>274</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>279</v>
+        <v>275</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
       <c r="E14" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>204</v>
+        <v>212</v>
       </c>
       <c r="G14" s="2" t="s">
         <v>13</v>
@@ -3800,22 +3794,22 @@
     </row>
     <row r="15" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>280</v>
+        <v>276</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>281</v>
+        <v>277</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
       <c r="E15" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>282</v>
+        <v>278</v>
       </c>
       <c r="G15" s="2" t="s">
         <v>13</v>
@@ -3823,22 +3817,22 @@
     </row>
     <row r="16" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>283</v>
+        <v>279</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>284</v>
+        <v>280</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>268</v>
+        <v>264</v>
       </c>
       <c r="E16" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>285</v>
+        <v>281</v>
       </c>
       <c r="G16" s="2" t="s">
         <v>13</v>
@@ -3889,22 +3883,22 @@
     </row>
     <row r="2" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
+        <v>282</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>284</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>285</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>286</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>287</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>288</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>289</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>290</v>
       </c>
       <c r="G2" s="2" t="s">
         <v>13</v>
@@ -3912,22 +3906,22 @@
     </row>
     <row r="3" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>291</v>
+        <v>287</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>287</v>
+        <v>283</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>292</v>
+        <v>288</v>
       </c>
       <c r="D3" s="2" t="s">
+        <v>285</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F3" s="2" t="s">
         <v>289</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>293</v>
       </c>
       <c r="G3" s="2" t="s">
         <v>13</v>
@@ -3935,22 +3929,22 @@
     </row>
     <row r="4" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>294</v>
+        <v>290</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>287</v>
+        <v>283</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>295</v>
+        <v>291</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>287</v>
+        <v>283</v>
       </c>
       <c r="E4" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="G4" s="2" t="s">
         <v>13</v>
@@ -3958,22 +3952,22 @@
     </row>
     <row r="5" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>296</v>
+        <v>292</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>287</v>
+        <v>283</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>297</v>
+        <v>293</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>287</v>
+        <v>283</v>
       </c>
       <c r="E5" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>298</v>
+        <v>294</v>
       </c>
       <c r="G5" s="2" t="s">
         <v>13</v>
@@ -3981,22 +3975,22 @@
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>299</v>
+        <v>295</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>287</v>
+        <v>283</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>300</v>
+        <v>296</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>268</v>
+        <v>264</v>
       </c>
       <c r="E6" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>204</v>
+        <v>212</v>
       </c>
       <c r="G6" s="2" t="s">
         <v>13</v>
@@ -4004,22 +3998,22 @@
     </row>
     <row r="7" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>301</v>
+        <v>297</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>287</v>
+        <v>283</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>302</v>
+        <v>298</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>287</v>
+        <v>283</v>
       </c>
       <c r="E7" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>110</v>
+        <v>299</v>
       </c>
       <c r="G7" s="2" t="s">
         <v>13</v>
@@ -4027,22 +4021,22 @@
     </row>
     <row r="8" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>287</v>
+        <v>283</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>304</v>
+        <v>301</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>289</v>
+        <v>285</v>
       </c>
       <c r="E8" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>305</v>
+        <v>302</v>
       </c>
       <c r="G8" s="2" t="s">
         <v>13</v>
@@ -4050,22 +4044,22 @@
     </row>
     <row r="9" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>306</v>
+        <v>303</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>287</v>
+        <v>283</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>289</v>
+        <v>285</v>
       </c>
       <c r="E9" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>28</v>
+        <v>305</v>
       </c>
       <c r="G9" s="2" t="s">
         <v>13</v>
@@ -4073,22 +4067,22 @@
     </row>
     <row r="10" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
+        <v>306</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>307</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>285</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F10" s="2" t="s">
         <v>308</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>287</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>309</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>289</v>
-      </c>
-      <c r="E10" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F10" s="2" t="s">
-        <v>310</v>
       </c>
       <c r="G10" s="2" t="s">
         <v>13</v>
@@ -4096,22 +4090,22 @@
     </row>
     <row r="11" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>287</v>
+        <v>283</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>287</v>
+        <v>283</v>
       </c>
       <c r="E11" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>204</v>
+        <v>212</v>
       </c>
       <c r="G11" s="2" t="s">
         <v>13</v>

</xml_diff>

<commit_message>
Synchronize latest local test run analysis report
</commit_message>
<xml_diff>
--- a/tests/reports/Test_Analysis_Report.xlsx
+++ b/tests/reports/Test_Analysis_Report.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="805" uniqueCount="311">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="805" uniqueCount="310">
   <si>
     <t>Test ID</t>
   </si>
@@ -56,7 +56,7 @@
     <t>Passed</t>
   </si>
   <si>
-    <t>1974ms</t>
+    <t>10049ms</t>
   </si>
   <si>
     <t>Assertion passed successfully</t>
@@ -68,7 +68,7 @@
     <t>Verify brand name PayBuddy header exists</t>
   </si>
   <si>
-    <t>284ms</t>
+    <t>89ms</t>
   </si>
   <si>
     <t>TC-WEB-UI-003</t>
@@ -77,7 +77,7 @@
     <t>Verify form email input label</t>
   </si>
   <si>
-    <t>69ms</t>
+    <t>56ms</t>
   </si>
   <si>
     <t>TC-WEB-UI-004</t>
@@ -86,718 +86,715 @@
     <t>Verify form password input label</t>
   </si>
   <si>
+    <t>42ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-005</t>
+  </si>
+  <si>
+    <t>Verify Sign In button is present</t>
+  </si>
+  <si>
+    <t>41ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-006</t>
+  </si>
+  <si>
+    <t>Verify secure access footer notice is present</t>
+  </si>
+  <si>
+    <t>32ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-007</t>
+  </si>
+  <si>
+    <t>Verify branding subtitle text exists</t>
+  </si>
+  <si>
     <t>35ms</t>
   </si>
   <si>
-    <t>TC-WEB-UI-005</t>
-  </si>
-  <si>
-    <t>Verify Sign In button is present</t>
-  </si>
-  <si>
-    <t>41ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UI-006</t>
-  </si>
-  <si>
-    <t>Verify secure access footer notice is present</t>
+    <t>TC-WEB-UI-008</t>
+  </si>
+  <si>
+    <t>Verify email input field placeholder</t>
+  </si>
+  <si>
+    <t>34ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-009</t>
+  </si>
+  <si>
+    <t>Verify password input field placeholder</t>
+  </si>
+  <si>
+    <t>31ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-010</t>
+  </si>
+  <si>
+    <t>Verify font family CSS on headers</t>
+  </si>
+  <si>
+    <t>39ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-011</t>
+  </si>
+  <si>
+    <t>Verify primary brand color on buttons</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-012</t>
+  </si>
+  <si>
+    <t>Verify centered block layout</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-013</t>
+  </si>
+  <si>
+    <t>Verify responsive structure at mobile width 360px</t>
+  </si>
+  <si>
+    <t>922ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-014</t>
+  </si>
+  <si>
+    <t>Verify responsive structure at tablet width 768px</t>
+  </si>
+  <si>
+    <t>921ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-015</t>
+  </si>
+  <si>
+    <t>Restore browser window maximization state</t>
+  </si>
+  <si>
+    <t>49ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-016</t>
+  </si>
+  <si>
+    <t>Verify HTML tag specification for email input</t>
+  </si>
+  <si>
+    <t>61ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-017</t>
+  </si>
+  <si>
+    <t>Verify HTML tag specification for password input</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-018</t>
+  </si>
+  <si>
+    <t>Verify card wrapper styles (border-radius)</t>
+  </si>
+  <si>
+    <t>47ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-019</t>
+  </si>
+  <si>
+    <t>Verify background styling matches design spec</t>
+  </si>
+  <si>
+    <t>43ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-020</t>
+  </si>
+  <si>
+    <t>Verify focus state click handler does not crash</t>
+  </si>
+  <si>
+    <t>196ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-021</t>
+  </si>
+  <si>
+    <t>Verify top-level container viewport classes</t>
+  </si>
+  <si>
+    <t>51ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-022</t>
+  </si>
+  <si>
+    <t>Verify branding and form division layout margins</t>
   </si>
   <si>
     <t>36ms</t>
   </si>
   <si>
-    <t>TC-WEB-UI-007</t>
-  </si>
-  <si>
-    <t>Verify branding subtitle text exists</t>
-  </si>
-  <si>
-    <t>TC-WEB-UI-008</t>
-  </si>
-  <si>
-    <t>Verify email input field placeholder</t>
-  </si>
-  <si>
-    <t>39ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UI-009</t>
-  </si>
-  <si>
-    <t>Verify password input field placeholder</t>
-  </si>
-  <si>
-    <t>34ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UI-010</t>
-  </si>
-  <si>
-    <t>Verify font family CSS on headers</t>
-  </si>
-  <si>
-    <t>40ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UI-011</t>
-  </si>
-  <si>
-    <t>Verify primary brand color on buttons</t>
-  </si>
-  <si>
-    <t>TC-WEB-UI-012</t>
-  </si>
-  <si>
-    <t>Verify centered block layout</t>
-  </si>
-  <si>
-    <t>TC-WEB-UI-013</t>
-  </si>
-  <si>
-    <t>Verify responsive structure at mobile width 360px</t>
-  </si>
-  <si>
-    <t>927ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UI-014</t>
-  </si>
-  <si>
-    <t>Verify responsive structure at tablet width 768px</t>
-  </si>
-  <si>
-    <t>941ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UI-015</t>
-  </si>
-  <si>
-    <t>Restore browser window maximization state</t>
-  </si>
-  <si>
-    <t>45ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UI-016</t>
-  </si>
-  <si>
-    <t>Verify HTML tag specification for email input</t>
+    <t>TC-WEB-UI-023</t>
+  </si>
+  <si>
+    <t>Verify clear textual contrast for reader accessibility</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-024</t>
+  </si>
+  <si>
+    <t>Verify page scales properly without layout clipping</t>
+  </si>
+  <si>
+    <t>54ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-025</t>
+  </si>
+  <si>
+    <t>Verify smooth interactive transitions on button inputs</t>
+  </si>
+  <si>
+    <t>30ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-001</t>
+  </si>
+  <si>
+    <t>Functional</t>
+  </si>
+  <si>
+    <t>Verify invalid login rejection message</t>
+  </si>
+  <si>
+    <t>3917ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-002</t>
+  </si>
+  <si>
+    <t>Verify rejection of nonexistent email</t>
+  </si>
+  <si>
+    <t>3709ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-003</t>
+  </si>
+  <si>
+    <t>Verify successful login with valid credentials redirects to Dashboard</t>
+  </si>
+  <si>
+    <t>3328ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-004</t>
+  </si>
+  <si>
+    <t>Verify dashboard displays Total Customers count</t>
+  </si>
+  <si>
+    <t>944ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-005</t>
+  </si>
+  <si>
+    <t>Verify dashboard displays Active Sales count</t>
+  </si>
+  <si>
+    <t>76ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-006</t>
+  </si>
+  <si>
+    <t>Verify dashboard displays Pending Installments count</t>
+  </si>
+  <si>
+    <t>48ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-007</t>
+  </si>
+  <si>
+    <t>Verify dashboard displays Today's Due count</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-008</t>
+  </si>
+  <si>
+    <t>Verify dashboard displays Outstanding Balance amount</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-009</t>
+  </si>
+  <si>
+    <t>Navigate to customers page and verify header</t>
+  </si>
+  <si>
+    <t>205ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-010</t>
+  </si>
+  <si>
+    <t>Verify add new customer input inputs are present</t>
+  </si>
+  <si>
+    <t>50ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-011</t>
+  </si>
+  <si>
+    <t>Verify customer creation and entry addition to table</t>
+  </si>
+  <si>
+    <t>2597ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-012</t>
+  </si>
+  <si>
+    <t>Verify presence of seeded customer</t>
+  </si>
+  <si>
+    <t>55ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-013</t>
+  </si>
+  <si>
+    <t>Navigate to specific customer profile page</t>
+  </si>
+  <si>
+    <t>1731ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-014</t>
+  </si>
+  <si>
+    <t>Verify phone number exists on profile detail bar</t>
+  </si>
+  <si>
+    <t>38ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-015</t>
+  </si>
+  <si>
+    <t>Verify Total Amount financial card is 1000 INR</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-016</t>
+  </si>
+  <si>
+    <t>Verify Paid Amount financial card is 0 INR</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-017</t>
+  </si>
+  <si>
+    <t>Verify Outstanding Balance financial card is 1000 INR</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-018</t>
+  </si>
+  <si>
+    <t>Verify E2E Test Item pending sale is loaded in sales list</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-019</t>
+  </si>
+  <si>
+    <t>Verify redirect to record payment page</t>
+  </si>
+  <si>
+    <t>1312ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-020</t>
+  </si>
+  <si>
+    <t>Verify remaining balance display match before payment</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-021</t>
+  </si>
+  <si>
+    <t>Record payment E2E execution and redirection validation</t>
+  </si>
+  <si>
+    <t>3421ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-022</t>
+  </si>
+  <si>
+    <t>Verify Outstanding Balance updates to 800 INR in customer card</t>
+  </si>
+  <si>
+    <t>1998ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-023</t>
+  </si>
+  <si>
+    <t>Verify Paid Amount updates to 200 INR in customer card</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-024</t>
+  </si>
+  <si>
+    <t>Verify recorded payment entry list matches mode UPI</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-025</t>
+  </si>
+  <si>
+    <t>Verify sales management index loads properly</t>
+  </si>
+  <si>
+    <t>1151ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-026</t>
+  </si>
+  <si>
+    <t>Verify sales search filter works properly</t>
+  </si>
+  <si>
+    <t>784ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-027</t>
+  </si>
+  <si>
+    <t>Navigate to Create New Sale form</t>
+  </si>
+  <si>
+    <t>1201ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-028</t>
+  </si>
+  <si>
+    <t>Verify total amount computed automatically (2 x 500 = 1000)</t>
+  </si>
+  <si>
+    <t>675ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-029</t>
+  </si>
+  <si>
+    <t>Create sale and verify redirect back to sales table</t>
+  </si>
+  <si>
+    <t>447ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-030</t>
+  </si>
+  <si>
+    <t>Verify Payments page path and title</t>
+  </si>
+  <si>
+    <t>2540ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-031</t>
+  </si>
+  <si>
+    <t>Verify E2E transaction exists in master list</t>
+  </si>
+  <si>
+    <t>52ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-032</t>
+  </si>
+  <si>
+    <t>Verify Ledger Book page loads</t>
+  </si>
+  <si>
+    <t>1580ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-033</t>
+  </si>
+  <si>
+    <t>Verify ledger records contain client name</t>
+  </si>
+  <si>
+    <t>73ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-034</t>
+  </si>
+  <si>
+    <t>Verify Installments page title</t>
+  </si>
+  <si>
+    <t>1056ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-035</t>
+  </si>
+  <si>
+    <t>Verify customer details exist on installment board</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-036</t>
+  </si>
+  <si>
+    <t>Verify direct Dashboard URL redirect</t>
+  </si>
+  <si>
+    <t>775ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-037</t>
+  </si>
+  <si>
+    <t>Verify customer data updates dynamically on UI edit</t>
+  </si>
+  <si>
+    <t>4643ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-038</t>
+  </si>
+  <si>
+    <t>Verify logout route terminates session and redirects to sign in</t>
+  </si>
+  <si>
+    <t>1664ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-039</t>
+  </si>
+  <si>
+    <t>Verify unauthorized dashboard access redirects to login</t>
+  </si>
+  <si>
+    <t>2406ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-040</t>
+  </si>
+  <si>
+    <t>Verify unauthorized customer details access redirects to login</t>
+  </si>
+  <si>
+    <t>2228ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UNIT-001</t>
+  </si>
+  <si>
+    <t>Unit</t>
+  </si>
+  <si>
+    <t>Test formatCurrency formatting positive amount</t>
+  </si>
+  <si>
+    <t>78ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UNIT-002</t>
+  </si>
+  <si>
+    <t>Test formatCurrency formatting zero amount</t>
+  </si>
+  <si>
+    <t>1ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UNIT-003</t>
+  </si>
+  <si>
+    <t>Test formatCurrency formatting negative amount</t>
+  </si>
+  <si>
+    <t>TC-WEB-UNIT-004</t>
+  </si>
+  <si>
+    <t>Test formatCurrency formatting large millions scale amount</t>
+  </si>
+  <si>
+    <t>TC-WEB-UNIT-005</t>
+  </si>
+  <si>
+    <t>Test formatCurrency decimal rounding functionality</t>
+  </si>
+  <si>
+    <t>0ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UNIT-006</t>
+  </si>
+  <si>
+    <t>Test formatDate string matching date details</t>
+  </si>
+  <si>
+    <t>17ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UNIT-007</t>
+  </si>
+  <si>
+    <t>Test formatDate fallback for null values</t>
+  </si>
+  <si>
+    <t>TC-WEB-UNIT-008</t>
+  </si>
+  <si>
+    <t>Test formatDate fallback for 0 value</t>
+  </si>
+  <si>
+    <t>TC-WEB-UNIT-009</t>
+  </si>
+  <si>
+    <t>Test formatDateTime details formatting</t>
+  </si>
+  <si>
+    <t>2ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UNIT-010</t>
+  </si>
+  <si>
+    <t>Test formatDateTime null timestamp handling</t>
+  </si>
+  <si>
+    <t>TC-WEB-UNIT-011</t>
+  </si>
+  <si>
+    <t>Verify email validation for valid string</t>
+  </si>
+  <si>
+    <t>TC-WEB-UNIT-012</t>
+  </si>
+  <si>
+    <t>Verify email validation blocks missing TLD</t>
+  </si>
+  <si>
+    <t>TC-WEB-UNIT-013</t>
+  </si>
+  <si>
+    <t>Verify email validation blocks missing alias prefix</t>
+  </si>
+  <si>
+    <t>TC-WEB-UNIT-014</t>
+  </si>
+  <si>
+    <t>Verify phone validation for standard 10 digit number</t>
+  </si>
+  <si>
+    <t>TC-WEB-UNIT-015</t>
+  </si>
+  <si>
+    <t>Verify phone validation blocks short length</t>
+  </si>
+  <si>
+    <t>TC-WEB-UNIT-016</t>
+  </si>
+  <si>
+    <t>Verify phone validation blocks alphabetic characters</t>
+  </si>
+  <si>
+    <t>TC-WEB-UNIT-017</t>
+  </si>
+  <si>
+    <t>Verify interest formula multiplication logic</t>
+  </si>
+  <si>
+    <t>TC-WEB-UNIT-018</t>
+  </si>
+  <si>
+    <t>Verify installment partitioning amount division</t>
+  </si>
+  <si>
+    <t>TC-WEB-UNIT-019</t>
+  </si>
+  <si>
+    <t>Verify remaining balance arithmetic subtraction</t>
+  </si>
+  <si>
+    <t>TC-WEB-UNIT-020</t>
+  </si>
+  <si>
+    <t>Verify mock environment manifest validator passes</t>
+  </si>
+  <si>
+    <t>TC-WEB-VAL-001</t>
+  </si>
+  <si>
+    <t>Validation</t>
+  </si>
+  <si>
+    <t>Verify email required constraint is enabled on form</t>
+  </si>
+  <si>
+    <t>330ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-VAL-002</t>
+  </si>
+  <si>
+    <t>Verify password required constraint is enabled on form</t>
+  </si>
+  <si>
+    <t>TC-WEB-VAL-003</t>
+  </si>
+  <si>
+    <t>Verify browser client blocks submissions for invalid email inputs</t>
+  </si>
+  <si>
+    <t>245ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-VAL-004</t>
+  </si>
+  <si>
+    <t>Verify character bounds for data buffers limit to 255 characters</t>
+  </si>
+  <si>
+    <t>TC-WEB-VAL-005</t>
+  </si>
+  <si>
+    <t>Verify customer creation form prevents empty submit</t>
+  </si>
+  <si>
+    <t>4492ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-VAL-006</t>
+  </si>
+  <si>
+    <t>Verify phone input uses tel semantic element type</t>
   </si>
   <si>
     <t>27ms</t>
   </si>
   <si>
-    <t>TC-WEB-UI-017</t>
-  </si>
-  <si>
-    <t>Verify HTML tag specification for password input</t>
-  </si>
-  <si>
-    <t>55ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UI-018</t>
-  </si>
-  <si>
-    <t>Verify card wrapper styles (border-radius)</t>
-  </si>
-  <si>
-    <t>49ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UI-019</t>
-  </si>
-  <si>
-    <t>Verify background styling matches design spec</t>
-  </si>
-  <si>
-    <t>44ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UI-020</t>
-  </si>
-  <si>
-    <t>Verify focus state click handler does not crash</t>
-  </si>
-  <si>
-    <t>147ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UI-021</t>
-  </si>
-  <si>
-    <t>Verify top-level container viewport classes</t>
-  </si>
-  <si>
-    <t>57ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UI-022</t>
-  </si>
-  <si>
-    <t>Verify branding and form division layout margins</t>
-  </si>
-  <si>
-    <t>38ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UI-023</t>
-  </si>
-  <si>
-    <t>Verify clear textual contrast for reader accessibility</t>
-  </si>
-  <si>
-    <t>53ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UI-024</t>
-  </si>
-  <si>
-    <t>Verify page scales properly without layout clipping</t>
-  </si>
-  <si>
-    <t>33ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UI-025</t>
-  </si>
-  <si>
-    <t>Verify smooth interactive transitions on button inputs</t>
-  </si>
-  <si>
-    <t>31ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-001</t>
-  </si>
-  <si>
-    <t>Functional</t>
-  </si>
-  <si>
-    <t>Verify invalid login rejection message</t>
-  </si>
-  <si>
-    <t>1427ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-002</t>
-  </si>
-  <si>
-    <t>Verify rejection of nonexistent email</t>
-  </si>
-  <si>
-    <t>1220ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-003</t>
-  </si>
-  <si>
-    <t>Verify successful login with valid credentials redirects to Dashboard</t>
-  </si>
-  <si>
-    <t>2197ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-004</t>
-  </si>
-  <si>
-    <t>Verify dashboard displays Total Customers count</t>
-  </si>
-  <si>
-    <t>304ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-005</t>
-  </si>
-  <si>
-    <t>Verify dashboard displays Active Sales count</t>
-  </si>
-  <si>
-    <t>46ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-006</t>
-  </si>
-  <si>
-    <t>Verify dashboard displays Pending Installments count</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-007</t>
-  </si>
-  <si>
-    <t>Verify dashboard displays Today's Due count</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-008</t>
-  </si>
-  <si>
-    <t>Verify dashboard displays Outstanding Balance amount</t>
-  </si>
-  <si>
-    <t>58ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-009</t>
-  </si>
-  <si>
-    <t>Navigate to customers page and verify header</t>
-  </si>
-  <si>
-    <t>232ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-010</t>
-  </si>
-  <si>
-    <t>Verify add new customer input inputs are present</t>
-  </si>
-  <si>
-    <t>80ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-011</t>
-  </si>
-  <si>
-    <t>Verify customer creation and entry addition to table</t>
-  </si>
-  <si>
-    <t>2614ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-012</t>
-  </si>
-  <si>
-    <t>Verify presence of seeded customer</t>
-  </si>
-  <si>
-    <t>52ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-013</t>
-  </si>
-  <si>
-    <t>Navigate to specific customer profile page</t>
-  </si>
-  <si>
-    <t>1424ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-014</t>
-  </si>
-  <si>
-    <t>Verify phone number exists on profile detail bar</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-015</t>
-  </si>
-  <si>
-    <t>Verify Total Amount financial card is 1000 INR</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-016</t>
-  </si>
-  <si>
-    <t>Verify Paid Amount financial card is 0 INR</t>
-  </si>
-  <si>
-    <t>51ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-017</t>
-  </si>
-  <si>
-    <t>Verify Outstanding Balance financial card is 1000 INR</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-018</t>
-  </si>
-  <si>
-    <t>Verify E2E Test Item pending sale is loaded in sales list</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-019</t>
-  </si>
-  <si>
-    <t>Verify redirect to record payment page</t>
-  </si>
-  <si>
-    <t>922ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-020</t>
-  </si>
-  <si>
-    <t>Verify remaining balance display match before payment</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-021</t>
-  </si>
-  <si>
-    <t>Record payment E2E execution and redirection validation</t>
-  </si>
-  <si>
-    <t>3425ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-022</t>
-  </si>
-  <si>
-    <t>Verify Outstanding Balance updates to 800 INR in customer card</t>
-  </si>
-  <si>
-    <t>1363ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-023</t>
-  </si>
-  <si>
-    <t>Verify Paid Amount updates to 200 INR in customer card</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-024</t>
-  </si>
-  <si>
-    <t>Verify recorded payment entry list matches mode UPI</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-025</t>
-  </si>
-  <si>
-    <t>Verify sales management index loads properly</t>
-  </si>
-  <si>
-    <t>754ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-026</t>
-  </si>
-  <si>
-    <t>Verify sales search filter works properly</t>
-  </si>
-  <si>
-    <t>774ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-027</t>
-  </si>
-  <si>
-    <t>Navigate to Create New Sale form</t>
-  </si>
-  <si>
-    <t>791ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-028</t>
-  </si>
-  <si>
-    <t>Verify total amount computed automatically (2 x 500 = 1000)</t>
-  </si>
-  <si>
-    <t>701ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-029</t>
-  </si>
-  <si>
-    <t>Create sale and verify redirect back to sales table</t>
-  </si>
-  <si>
-    <t>463ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-030</t>
-  </si>
-  <si>
-    <t>Verify Payments page path and title</t>
-  </si>
-  <si>
-    <t>848ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-031</t>
-  </si>
-  <si>
-    <t>Verify E2E transaction exists in master list</t>
-  </si>
-  <si>
-    <t>82ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-032</t>
-  </si>
-  <si>
-    <t>Verify Ledger Book page loads</t>
-  </si>
-  <si>
-    <t>900ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-033</t>
-  </si>
-  <si>
-    <t>Verify ledger records contain client name</t>
-  </si>
-  <si>
-    <t>61ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-034</t>
-  </si>
-  <si>
-    <t>Verify Installments page title</t>
-  </si>
-  <si>
-    <t>672ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-035</t>
-  </si>
-  <si>
-    <t>Verify customer details exist on installment board</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-036</t>
-  </si>
-  <si>
-    <t>Verify direct Dashboard URL redirect</t>
-  </si>
-  <si>
-    <t>259ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-037</t>
-  </si>
-  <si>
-    <t>Verify customer data updates dynamically on UI edit</t>
-  </si>
-  <si>
-    <t>4735ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-038</t>
-  </si>
-  <si>
-    <t>Verify logout route terminates session and redirects to sign in</t>
-  </si>
-  <si>
-    <t>917ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-039</t>
-  </si>
-  <si>
-    <t>Verify unauthorized dashboard access redirects to login</t>
-  </si>
-  <si>
-    <t>2154ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-040</t>
-  </si>
-  <si>
-    <t>Verify unauthorized customer details access redirects to login</t>
-  </si>
-  <si>
-    <t>2557ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UNIT-001</t>
-  </si>
-  <si>
-    <t>Unit</t>
-  </si>
-  <si>
-    <t>Test formatCurrency formatting positive amount</t>
-  </si>
-  <si>
-    <t>84ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UNIT-002</t>
-  </si>
-  <si>
-    <t>Test formatCurrency formatting zero amount</t>
-  </si>
-  <si>
-    <t>1ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UNIT-003</t>
-  </si>
-  <si>
-    <t>Test formatCurrency formatting negative amount</t>
-  </si>
-  <si>
-    <t>TC-WEB-UNIT-004</t>
-  </si>
-  <si>
-    <t>Test formatCurrency formatting large millions scale amount</t>
-  </si>
-  <si>
-    <t>TC-WEB-UNIT-005</t>
-  </si>
-  <si>
-    <t>Test formatCurrency decimal rounding functionality</t>
-  </si>
-  <si>
-    <t>TC-WEB-UNIT-006</t>
-  </si>
-  <si>
-    <t>Test formatDate string matching date details</t>
-  </si>
-  <si>
-    <t>15ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UNIT-007</t>
-  </si>
-  <si>
-    <t>Test formatDate fallback for null values</t>
-  </si>
-  <si>
-    <t>0ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UNIT-008</t>
-  </si>
-  <si>
-    <t>Test formatDate fallback for 0 value</t>
-  </si>
-  <si>
-    <t>TC-WEB-UNIT-009</t>
-  </si>
-  <si>
-    <t>Test formatDateTime details formatting</t>
-  </si>
-  <si>
-    <t>2ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UNIT-010</t>
-  </si>
-  <si>
-    <t>Test formatDateTime null timestamp handling</t>
-  </si>
-  <si>
-    <t>TC-WEB-UNIT-011</t>
-  </si>
-  <si>
-    <t>Verify email validation for valid string</t>
-  </si>
-  <si>
-    <t>TC-WEB-UNIT-012</t>
-  </si>
-  <si>
-    <t>Verify email validation blocks missing TLD</t>
-  </si>
-  <si>
-    <t>TC-WEB-UNIT-013</t>
-  </si>
-  <si>
-    <t>Verify email validation blocks missing alias prefix</t>
-  </si>
-  <si>
-    <t>TC-WEB-UNIT-014</t>
-  </si>
-  <si>
-    <t>Verify phone validation for standard 10 digit number</t>
-  </si>
-  <si>
-    <t>TC-WEB-UNIT-015</t>
-  </si>
-  <si>
-    <t>Verify phone validation blocks short length</t>
-  </si>
-  <si>
-    <t>TC-WEB-UNIT-016</t>
-  </si>
-  <si>
-    <t>Verify phone validation blocks alphabetic characters</t>
-  </si>
-  <si>
-    <t>TC-WEB-UNIT-017</t>
-  </si>
-  <si>
-    <t>Verify interest formula multiplication logic</t>
-  </si>
-  <si>
-    <t>TC-WEB-UNIT-018</t>
-  </si>
-  <si>
-    <t>Verify installment partitioning amount division</t>
-  </si>
-  <si>
-    <t>TC-WEB-UNIT-019</t>
-  </si>
-  <si>
-    <t>Verify remaining balance arithmetic subtraction</t>
-  </si>
-  <si>
-    <t>TC-WEB-UNIT-020</t>
-  </si>
-  <si>
-    <t>Verify mock environment manifest validator passes</t>
-  </si>
-  <si>
-    <t>TC-WEB-VAL-001</t>
-  </si>
-  <si>
-    <t>Validation</t>
-  </si>
-  <si>
-    <t>Verify email required constraint is enabled on form</t>
-  </si>
-  <si>
-    <t>411ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-VAL-002</t>
-  </si>
-  <si>
-    <t>Verify password required constraint is enabled on form</t>
-  </si>
-  <si>
-    <t>37ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-VAL-003</t>
-  </si>
-  <si>
-    <t>Verify browser client blocks submissions for invalid email inputs</t>
-  </si>
-  <si>
-    <t>257ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-VAL-004</t>
-  </si>
-  <si>
-    <t>Verify character bounds for data buffers limit to 255 characters</t>
-  </si>
-  <si>
-    <t>TC-WEB-VAL-005</t>
-  </si>
-  <si>
-    <t>Verify customer creation form prevents empty submit</t>
-  </si>
-  <si>
-    <t>3671ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-VAL-006</t>
-  </si>
-  <si>
-    <t>Verify phone input uses tel semantic element type</t>
-  </si>
-  <si>
     <t>TC-WEB-VAL-007</t>
   </si>
   <si>
     <t>Verify sale quantity requires positive minimum value (&gt; 0)</t>
   </si>
   <si>
-    <t>1154ms</t>
+    <t>1009ms</t>
   </si>
   <si>
     <t>TC-WEB-VAL-008</t>
@@ -806,6 +803,9 @@
     <t>Verify unit price input restricts negative numbers</t>
   </si>
   <si>
+    <t>24ms</t>
+  </si>
+  <si>
     <t>TC-WEB-VAL-009</t>
   </si>
   <si>
@@ -815,7 +815,7 @@
     <t>Security</t>
   </si>
   <si>
-    <t>2270ms</t>
+    <t>2423ms</t>
   </si>
   <si>
     <t>TC-WEB-VAL-010</t>
@@ -830,7 +830,7 @@
     <t>Verify error prevents overpayment collections</t>
   </si>
   <si>
-    <t>2883ms</t>
+    <t>3061ms</t>
   </si>
   <si>
     <t>TC-WEB-VAL-012</t>
@@ -839,7 +839,7 @@
     <t>Verify collection input restricts 0 value submissions</t>
   </si>
   <si>
-    <t>1453ms</t>
+    <t>1384ms</t>
   </si>
   <si>
     <t>TC-WEB-VAL-013</t>
@@ -854,7 +854,7 @@
     <t>Verify wildcard URLs redirect to main route base</t>
   </si>
   <si>
-    <t>2165ms</t>
+    <t>4117ms</t>
   </si>
   <si>
     <t>TC-WEB-VAL-015</t>
@@ -863,7 +863,7 @@
     <t>Verify HTML password hidden mask attribute config</t>
   </si>
   <si>
-    <t>1008ms</t>
+    <t>2036ms</t>
   </si>
   <si>
     <t>TC-WEB-DEP-001</t>
@@ -878,7 +878,7 @@
     <t>Performance</t>
   </si>
   <si>
-    <t>497ms</t>
+    <t>527ms</t>
   </si>
   <si>
     <t>TC-WEB-DEP-002</t>
@@ -887,7 +887,7 @@
     <t>Verify full render transition load time under limit</t>
   </si>
   <si>
-    <t>1660ms</t>
+    <t>2200ms</t>
   </si>
   <si>
     <t>TC-WEB-DEP-003</t>
@@ -902,7 +902,7 @@
     <t>Verify favicon.ico endpoint yields clean HTTP status</t>
   </si>
   <si>
-    <t>439ms</t>
+    <t>358ms</t>
   </si>
   <si>
     <t>TC-WEB-DEP-005</t>
@@ -917,7 +917,7 @@
     <t>Verify head links contain manifest registration details</t>
   </si>
   <si>
-    <t>167ms</t>
+    <t>798ms</t>
   </si>
   <si>
     <t>TC-WEB-DEP-007</t>
@@ -942,9 +942,6 @@
   </si>
   <si>
     <t>Verify DOM count index scales cleanly</t>
-  </si>
-  <si>
-    <t>16ms</t>
   </si>
   <si>
     <t>TC-WEB-DEP-010</t>
@@ -1564,7 +1561,7 @@
         <v>11</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="G8" s="2" t="s">
         <v>13</v>
@@ -1572,13 +1569,13 @@
     </row>
     <row r="9" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>10</v>
@@ -1587,7 +1584,7 @@
         <v>11</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="G9" s="2" t="s">
         <v>13</v>
@@ -1595,13 +1592,13 @@
     </row>
     <row r="10" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D10" s="2" t="s">
         <v>10</v>
@@ -1610,7 +1607,7 @@
         <v>11</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G10" s="2" t="s">
         <v>13</v>
@@ -1618,13 +1615,13 @@
     </row>
     <row r="11" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B11" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D11" s="2" t="s">
         <v>10</v>
@@ -1633,7 +1630,7 @@
         <v>11</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="G11" s="2" t="s">
         <v>13</v>
@@ -1641,13 +1638,13 @@
     </row>
     <row r="12" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B12" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D12" s="2" t="s">
         <v>10</v>
@@ -1656,7 +1653,7 @@
         <v>11</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="G12" s="2" t="s">
         <v>13</v>
@@ -1664,13 +1661,13 @@
     </row>
     <row r="13" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B13" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D13" s="2" t="s">
         <v>10</v>
@@ -1679,7 +1676,7 @@
         <v>11</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="G13" s="2" t="s">
         <v>13</v>
@@ -1687,13 +1684,13 @@
     </row>
     <row r="14" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B14" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D14" s="2" t="s">
         <v>10</v>
@@ -1702,7 +1699,7 @@
         <v>11</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="G14" s="2" t="s">
         <v>13</v>
@@ -1710,13 +1707,13 @@
     </row>
     <row r="15" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B15" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D15" s="2" t="s">
         <v>10</v>
@@ -1725,7 +1722,7 @@
         <v>11</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="G15" s="2" t="s">
         <v>13</v>
@@ -1733,13 +1730,13 @@
     </row>
     <row r="16" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B16" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D16" s="2" t="s">
         <v>10</v>
@@ -1748,7 +1745,7 @@
         <v>11</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="G16" s="2" t="s">
         <v>13</v>
@@ -1756,13 +1753,13 @@
     </row>
     <row r="17" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B17" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D17" s="2" t="s">
         <v>10</v>
@@ -1771,7 +1768,7 @@
         <v>11</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G17" s="2" t="s">
         <v>13</v>
@@ -1779,13 +1776,13 @@
     </row>
     <row r="18" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B18" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D18" s="2" t="s">
         <v>10</v>
@@ -1794,7 +1791,7 @@
         <v>11</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>58</v>
+        <v>34</v>
       </c>
       <c r="G18" s="2" t="s">
         <v>13</v>
@@ -1932,7 +1929,7 @@
         <v>11</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="G24" s="2" t="s">
         <v>13</v>
@@ -1940,13 +1937,13 @@
     </row>
     <row r="25" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B25" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D25" s="2" t="s">
         <v>10</v>
@@ -1955,7 +1952,7 @@
         <v>11</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="G25" s="2" t="s">
         <v>13</v>
@@ -1963,13 +1960,13 @@
     </row>
     <row r="26" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B26" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D26" s="2" t="s">
         <v>10</v>
@@ -1978,7 +1975,7 @@
         <v>11</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G26" s="2" t="s">
         <v>13</v>
@@ -2029,22 +2026,22 @@
     </row>
     <row r="2" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B2" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>85</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>86</v>
       </c>
       <c r="G2" s="2" t="s">
         <v>13</v>
@@ -2052,22 +2049,22 @@
     </row>
     <row r="3" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="B3" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="C3" s="2" t="s">
+      <c r="D3" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F3" s="2" t="s">
         <v>88</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>89</v>
       </c>
       <c r="G3" s="2" t="s">
         <v>13</v>
@@ -2075,22 +2072,22 @@
     </row>
     <row r="4" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="B4" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="C4" s="2" t="s">
+      <c r="D4" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F4" s="2" t="s">
         <v>91</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>92</v>
       </c>
       <c r="G4" s="2" t="s">
         <v>13</v>
@@ -2098,22 +2095,22 @@
     </row>
     <row r="5" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="C5" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="B5" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="C5" s="2" t="s">
+      <c r="D5" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F5" s="2" t="s">
         <v>94</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F5" s="2" t="s">
-        <v>95</v>
       </c>
       <c r="G5" s="2" t="s">
         <v>13</v>
@@ -2121,22 +2118,22 @@
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="C6" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="B6" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="C6" s="2" t="s">
+      <c r="D6" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F6" s="2" t="s">
         <v>97</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>98</v>
       </c>
       <c r="G6" s="2" t="s">
         <v>13</v>
@@ -2144,22 +2141,22 @@
     </row>
     <row r="7" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="C7" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="B7" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="C7" s="2" t="s">
+      <c r="D7" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F7" s="2" t="s">
         <v>100</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F7" s="2" t="s">
-        <v>64</v>
       </c>
       <c r="G7" s="2" t="s">
         <v>13</v>
@@ -2170,19 +2167,19 @@
         <v>101</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>102</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E8" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>76</v>
+        <v>28</v>
       </c>
       <c r="G8" s="2" t="s">
         <v>13</v>
@@ -2193,19 +2190,19 @@
         <v>103</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>104</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E9" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>105</v>
+        <v>78</v>
       </c>
       <c r="G9" s="2" t="s">
         <v>13</v>
@@ -2213,22 +2210,22 @@
     </row>
     <row r="10" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="C10" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="B10" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="C10" s="2" t="s">
+      <c r="D10" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F10" s="2" t="s">
         <v>107</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="E10" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F10" s="2" t="s">
-        <v>108</v>
       </c>
       <c r="G10" s="2" t="s">
         <v>13</v>
@@ -2236,22 +2233,22 @@
     </row>
     <row r="11" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="C11" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="B11" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="C11" s="2" t="s">
+      <c r="D11" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F11" s="2" t="s">
         <v>110</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="E11" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F11" s="2" t="s">
-        <v>111</v>
       </c>
       <c r="G11" s="2" t="s">
         <v>13</v>
@@ -2259,22 +2256,22 @@
     </row>
     <row r="12" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="C12" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="B12" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="C12" s="2" t="s">
+      <c r="D12" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F12" s="2" t="s">
         <v>113</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="E12" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F12" s="2" t="s">
-        <v>114</v>
       </c>
       <c r="G12" s="2" t="s">
         <v>13</v>
@@ -2282,22 +2279,22 @@
     </row>
     <row r="13" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="C13" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="B13" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="C13" s="2" t="s">
+      <c r="D13" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F13" s="2" t="s">
         <v>116</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="E13" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F13" s="2" t="s">
-        <v>117</v>
       </c>
       <c r="G13" s="2" t="s">
         <v>13</v>
@@ -2305,22 +2302,22 @@
     </row>
     <row r="14" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="C14" s="2" t="s">
         <v>118</v>
       </c>
-      <c r="B14" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="C14" s="2" t="s">
+      <c r="D14" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F14" s="2" t="s">
         <v>119</v>
-      </c>
-      <c r="D14" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="E14" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F14" s="2" t="s">
-        <v>120</v>
       </c>
       <c r="G14" s="2" t="s">
         <v>13</v>
@@ -2328,22 +2325,22 @@
     </row>
     <row r="15" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="C15" s="2" t="s">
         <v>121</v>
       </c>
-      <c r="B15" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="C15" s="2" t="s">
+      <c r="D15" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F15" s="2" t="s">
         <v>122</v>
-      </c>
-      <c r="D15" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="E15" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F15" s="2" t="s">
-        <v>76</v>
       </c>
       <c r="G15" s="2" t="s">
         <v>13</v>
@@ -2354,19 +2351,19 @@
         <v>123</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C16" s="2" t="s">
         <v>124</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E16" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>52</v>
+        <v>70</v>
       </c>
       <c r="G16" s="2" t="s">
         <v>13</v>
@@ -2377,19 +2374,19 @@
         <v>125</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C17" s="2" t="s">
         <v>126</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E17" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>127</v>
+        <v>61</v>
       </c>
       <c r="G17" s="2" t="s">
         <v>13</v>
@@ -2397,22 +2394,22 @@
     </row>
     <row r="18" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="C18" s="2" t="s">
         <v>128</v>
       </c>
-      <c r="B18" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="C18" s="2" t="s">
-        <v>129</v>
-      </c>
       <c r="D18" s="2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E18" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="G18" s="2" t="s">
         <v>13</v>
@@ -2420,22 +2417,22 @@
     </row>
     <row r="19" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="C19" s="2" t="s">
         <v>130</v>
       </c>
-      <c r="B19" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="C19" s="2" t="s">
-        <v>131</v>
-      </c>
       <c r="D19" s="2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E19" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>79</v>
+        <v>37</v>
       </c>
       <c r="G19" s="2" t="s">
         <v>13</v>
@@ -2443,22 +2440,22 @@
     </row>
     <row r="20" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="C20" s="2" t="s">
         <v>132</v>
       </c>
-      <c r="B20" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="C20" s="2" t="s">
+      <c r="D20" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="E20" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F20" s="2" t="s">
         <v>133</v>
-      </c>
-      <c r="D20" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="E20" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F20" s="2" t="s">
-        <v>134</v>
       </c>
       <c r="G20" s="2" t="s">
         <v>13</v>
@@ -2466,22 +2463,22 @@
     </row>
     <row r="21" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="C21" s="2" t="s">
         <v>135</v>
       </c>
-      <c r="B21" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="C21" s="2" t="s">
-        <v>136</v>
-      </c>
       <c r="D21" s="2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E21" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>28</v>
+        <v>100</v>
       </c>
       <c r="G21" s="2" t="s">
         <v>13</v>
@@ -2489,22 +2486,22 @@
     </row>
     <row r="22" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="C22" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="B22" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="C22" s="2" t="s">
+      <c r="D22" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="E22" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F22" s="2" t="s">
         <v>138</v>
-      </c>
-      <c r="D22" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="E22" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F22" s="2" t="s">
-        <v>139</v>
       </c>
       <c r="G22" s="2" t="s">
         <v>13</v>
@@ -2512,22 +2509,22 @@
     </row>
     <row r="23" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="C23" s="2" t="s">
         <v>140</v>
       </c>
-      <c r="B23" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="C23" s="2" t="s">
+      <c r="D23" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="E23" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F23" s="2" t="s">
         <v>141</v>
-      </c>
-      <c r="D23" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="E23" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F23" s="2" t="s">
-        <v>142</v>
       </c>
       <c r="G23" s="2" t="s">
         <v>13</v>
@@ -2535,22 +2532,22 @@
     </row>
     <row r="24" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="C24" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="B24" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="C24" s="2" t="s">
-        <v>144</v>
-      </c>
       <c r="D24" s="2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E24" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="G24" s="2" t="s">
         <v>13</v>
@@ -2558,22 +2555,22 @@
     </row>
     <row r="25" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="C25" s="2" t="s">
         <v>145</v>
       </c>
-      <c r="B25" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="C25" s="2" t="s">
-        <v>146</v>
-      </c>
       <c r="D25" s="2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E25" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>22</v>
+        <v>40</v>
       </c>
       <c r="G25" s="2" t="s">
         <v>13</v>
@@ -2581,22 +2578,22 @@
     </row>
     <row r="26" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="C26" s="2" t="s">
         <v>147</v>
       </c>
-      <c r="B26" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="C26" s="2" t="s">
+      <c r="D26" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="E26" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F26" s="2" t="s">
         <v>148</v>
-      </c>
-      <c r="D26" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="E26" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F26" s="2" t="s">
-        <v>149</v>
       </c>
       <c r="G26" s="2" t="s">
         <v>13</v>
@@ -2604,22 +2601,22 @@
     </row>
     <row r="27" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="C27" s="2" t="s">
         <v>150</v>
       </c>
-      <c r="B27" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="C27" s="2" t="s">
+      <c r="D27" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="E27" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F27" s="2" t="s">
         <v>151</v>
-      </c>
-      <c r="D27" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="E27" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F27" s="2" t="s">
-        <v>152</v>
       </c>
       <c r="G27" s="2" t="s">
         <v>13</v>
@@ -2627,22 +2624,22 @@
     </row>
     <row r="28" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="C28" s="2" t="s">
         <v>153</v>
       </c>
-      <c r="B28" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="C28" s="2" t="s">
+      <c r="D28" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="E28" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F28" s="2" t="s">
         <v>154</v>
-      </c>
-      <c r="D28" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="E28" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F28" s="2" t="s">
-        <v>155</v>
       </c>
       <c r="G28" s="2" t="s">
         <v>13</v>
@@ -2650,22 +2647,22 @@
     </row>
     <row r="29" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="C29" s="2" t="s">
         <v>156</v>
       </c>
-      <c r="B29" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="C29" s="2" t="s">
+      <c r="D29" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="E29" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F29" s="2" t="s">
         <v>157</v>
-      </c>
-      <c r="D29" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="E29" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F29" s="2" t="s">
-        <v>158</v>
       </c>
       <c r="G29" s="2" t="s">
         <v>13</v>
@@ -2673,22 +2670,22 @@
     </row>
     <row r="30" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="C30" s="2" t="s">
         <v>159</v>
       </c>
-      <c r="B30" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="C30" s="2" t="s">
+      <c r="D30" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="E30" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F30" s="2" t="s">
         <v>160</v>
-      </c>
-      <c r="D30" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="E30" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F30" s="2" t="s">
-        <v>161</v>
       </c>
       <c r="G30" s="2" t="s">
         <v>13</v>
@@ -2696,22 +2693,22 @@
     </row>
     <row r="31" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="C31" s="2" t="s">
         <v>162</v>
       </c>
-      <c r="B31" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="C31" s="2" t="s">
+      <c r="D31" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="E31" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F31" s="2" t="s">
         <v>163</v>
-      </c>
-      <c r="D31" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="E31" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F31" s="2" t="s">
-        <v>164</v>
       </c>
       <c r="G31" s="2" t="s">
         <v>13</v>
@@ -2719,22 +2716,22 @@
     </row>
     <row r="32" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="C32" s="2" t="s">
         <v>165</v>
       </c>
-      <c r="B32" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="C32" s="2" t="s">
+      <c r="D32" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="E32" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F32" s="2" t="s">
         <v>166</v>
-      </c>
-      <c r="D32" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="E32" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F32" s="2" t="s">
-        <v>167</v>
       </c>
       <c r="G32" s="2" t="s">
         <v>13</v>
@@ -2742,22 +2739,22 @@
     </row>
     <row r="33" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="C33" s="2" t="s">
         <v>168</v>
       </c>
-      <c r="B33" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="C33" s="2" t="s">
+      <c r="D33" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="E33" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F33" s="2" t="s">
         <v>169</v>
-      </c>
-      <c r="D33" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="E33" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F33" s="2" t="s">
-        <v>170</v>
       </c>
       <c r="G33" s="2" t="s">
         <v>13</v>
@@ -2765,22 +2762,22 @@
     </row>
     <row r="34" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="C34" s="2" t="s">
         <v>171</v>
       </c>
-      <c r="B34" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="C34" s="2" t="s">
+      <c r="D34" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="E34" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F34" s="2" t="s">
         <v>172</v>
-      </c>
-      <c r="D34" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="E34" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F34" s="2" t="s">
-        <v>173</v>
       </c>
       <c r="G34" s="2" t="s">
         <v>13</v>
@@ -2788,22 +2785,22 @@
     </row>
     <row r="35" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="C35" s="2" t="s">
         <v>174</v>
       </c>
-      <c r="B35" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="C35" s="2" t="s">
+      <c r="D35" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="E35" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F35" s="2" t="s">
         <v>175</v>
-      </c>
-      <c r="D35" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="E35" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F35" s="2" t="s">
-        <v>176</v>
       </c>
       <c r="G35" s="2" t="s">
         <v>13</v>
@@ -2811,22 +2808,22 @@
     </row>
     <row r="36" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="C36" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="B36" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="C36" s="2" t="s">
-        <v>178</v>
-      </c>
       <c r="D36" s="2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E36" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F36" s="2" t="s">
-        <v>117</v>
+        <v>40</v>
       </c>
       <c r="G36" s="2" t="s">
         <v>13</v>
@@ -2834,22 +2831,22 @@
     </row>
     <row r="37" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="C37" s="2" t="s">
         <v>179</v>
       </c>
-      <c r="B37" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="C37" s="2" t="s">
+      <c r="D37" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="E37" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F37" s="2" t="s">
         <v>180</v>
-      </c>
-      <c r="D37" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="E37" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F37" s="2" t="s">
-        <v>181</v>
       </c>
       <c r="G37" s="2" t="s">
         <v>13</v>
@@ -2857,22 +2854,22 @@
     </row>
     <row r="38" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="C38" s="2" t="s">
         <v>182</v>
       </c>
-      <c r="B38" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="C38" s="2" t="s">
+      <c r="D38" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="E38" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F38" s="2" t="s">
         <v>183</v>
-      </c>
-      <c r="D38" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="E38" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F38" s="2" t="s">
-        <v>184</v>
       </c>
       <c r="G38" s="2" t="s">
         <v>13</v>
@@ -2880,22 +2877,22 @@
     </row>
     <row r="39" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="C39" s="2" t="s">
         <v>185</v>
       </c>
-      <c r="B39" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="C39" s="2" t="s">
+      <c r="D39" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="E39" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F39" s="2" t="s">
         <v>186</v>
-      </c>
-      <c r="D39" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="E39" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F39" s="2" t="s">
-        <v>187</v>
       </c>
       <c r="G39" s="2" t="s">
         <v>13</v>
@@ -2903,22 +2900,22 @@
     </row>
     <row r="40" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="C40" s="2" t="s">
         <v>188</v>
       </c>
-      <c r="B40" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="C40" s="2" t="s">
+      <c r="D40" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="E40" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F40" s="2" t="s">
         <v>189</v>
-      </c>
-      <c r="D40" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="E40" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F40" s="2" t="s">
-        <v>190</v>
       </c>
       <c r="G40" s="2" t="s">
         <v>13</v>
@@ -2926,22 +2923,22 @@
     </row>
     <row r="41" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="C41" s="2" t="s">
         <v>191</v>
       </c>
-      <c r="B41" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="C41" s="2" t="s">
+      <c r="D41" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="E41" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F41" s="2" t="s">
         <v>192</v>
-      </c>
-      <c r="D41" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="E41" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F41" s="2" t="s">
-        <v>193</v>
       </c>
       <c r="G41" s="2" t="s">
         <v>13</v>
@@ -2992,22 +2989,22 @@
     </row>
     <row r="2" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>194</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="C2" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>196</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>195</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>197</v>
       </c>
       <c r="G2" s="2" t="s">
         <v>13</v>
@@ -3015,22 +3012,22 @@
     </row>
     <row r="3" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>198</v>
       </c>
-      <c r="B3" s="2" t="s">
-        <v>195</v>
-      </c>
-      <c r="C3" s="2" t="s">
+      <c r="D3" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F3" s="2" t="s">
         <v>199</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>195</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>200</v>
       </c>
       <c r="G3" s="2" t="s">
         <v>13</v>
@@ -3038,22 +3035,22 @@
     </row>
     <row r="4" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>201</v>
       </c>
-      <c r="B4" s="2" t="s">
-        <v>195</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>202</v>
-      </c>
       <c r="D4" s="2" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="E4" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="G4" s="2" t="s">
         <v>13</v>
@@ -3061,22 +3058,22 @@
     </row>
     <row r="5" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="C5" s="2" t="s">
         <v>203</v>
       </c>
-      <c r="B5" s="2" t="s">
-        <v>195</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>204</v>
-      </c>
       <c r="D5" s="2" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="E5" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="G5" s="2" t="s">
         <v>13</v>
@@ -3084,22 +3081,22 @@
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
+        <v>204</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="C6" s="2" t="s">
         <v>205</v>
       </c>
-      <c r="B6" s="2" t="s">
-        <v>195</v>
-      </c>
-      <c r="C6" s="2" t="s">
+      <c r="D6" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F6" s="2" t="s">
         <v>206</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>195</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>200</v>
       </c>
       <c r="G6" s="2" t="s">
         <v>13</v>
@@ -3110,13 +3107,13 @@
         <v>207</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>208</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="E7" s="3" t="s">
         <v>11</v>
@@ -3133,19 +3130,19 @@
         <v>210</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>211</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="E8" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>212</v>
+        <v>206</v>
       </c>
       <c r="G8" s="2" t="s">
         <v>13</v>
@@ -3153,22 +3150,22 @@
     </row>
     <row r="9" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
+        <v>212</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="C9" s="2" t="s">
         <v>213</v>
       </c>
-      <c r="B9" s="2" t="s">
-        <v>195</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>214</v>
-      </c>
       <c r="D9" s="2" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="E9" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>212</v>
+        <v>206</v>
       </c>
       <c r="G9" s="2" t="s">
         <v>13</v>
@@ -3176,22 +3173,22 @@
     </row>
     <row r="10" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
+        <v>214</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="C10" s="2" t="s">
         <v>215</v>
       </c>
-      <c r="B10" s="2" t="s">
-        <v>195</v>
-      </c>
-      <c r="C10" s="2" t="s">
+      <c r="D10" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F10" s="2" t="s">
         <v>216</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>195</v>
-      </c>
-      <c r="E10" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F10" s="2" t="s">
-        <v>217</v>
       </c>
       <c r="G10" s="2" t="s">
         <v>13</v>
@@ -3199,22 +3196,22 @@
     </row>
     <row r="11" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
+        <v>217</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="C11" s="2" t="s">
         <v>218</v>
       </c>
-      <c r="B11" s="2" t="s">
-        <v>195</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>219</v>
-      </c>
       <c r="D11" s="2" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="E11" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>212</v>
+        <v>199</v>
       </c>
       <c r="G11" s="2" t="s">
         <v>13</v>
@@ -3222,22 +3219,22 @@
     </row>
     <row r="12" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
+        <v>219</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="C12" s="2" t="s">
         <v>220</v>
       </c>
-      <c r="B12" s="2" t="s">
-        <v>195</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>221</v>
-      </c>
       <c r="D12" s="2" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="E12" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>212</v>
+        <v>206</v>
       </c>
       <c r="G12" s="2" t="s">
         <v>13</v>
@@ -3245,22 +3242,22 @@
     </row>
     <row r="13" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="C13" s="2" t="s">
         <v>222</v>
       </c>
-      <c r="B13" s="2" t="s">
-        <v>195</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>223</v>
-      </c>
       <c r="D13" s="2" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="E13" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>212</v>
+        <v>206</v>
       </c>
       <c r="G13" s="2" t="s">
         <v>13</v>
@@ -3268,22 +3265,22 @@
     </row>
     <row r="14" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="C14" s="2" t="s">
         <v>224</v>
       </c>
-      <c r="B14" s="2" t="s">
-        <v>195</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>225</v>
-      </c>
       <c r="D14" s="2" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="E14" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>212</v>
+        <v>206</v>
       </c>
       <c r="G14" s="2" t="s">
         <v>13</v>
@@ -3291,22 +3288,22 @@
     </row>
     <row r="15" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="C15" s="2" t="s">
         <v>226</v>
       </c>
-      <c r="B15" s="2" t="s">
-        <v>195</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>227</v>
-      </c>
       <c r="D15" s="2" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="E15" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
       <c r="G15" s="2" t="s">
         <v>13</v>
@@ -3314,22 +3311,22 @@
     </row>
     <row r="16" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="C16" s="2" t="s">
         <v>228</v>
       </c>
-      <c r="B16" s="2" t="s">
-        <v>195</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>229</v>
-      </c>
       <c r="D16" s="2" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="E16" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>212</v>
+        <v>206</v>
       </c>
       <c r="G16" s="2" t="s">
         <v>13</v>
@@ -3337,22 +3334,22 @@
     </row>
     <row r="17" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
+        <v>229</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="C17" s="2" t="s">
         <v>230</v>
       </c>
-      <c r="B17" s="2" t="s">
-        <v>195</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>231</v>
-      </c>
       <c r="D17" s="2" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="E17" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>212</v>
+        <v>206</v>
       </c>
       <c r="G17" s="2" t="s">
         <v>13</v>
@@ -3360,22 +3357,22 @@
     </row>
     <row r="18" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="C18" s="2" t="s">
         <v>232</v>
       </c>
-      <c r="B18" s="2" t="s">
-        <v>195</v>
-      </c>
-      <c r="C18" s="2" t="s">
-        <v>233</v>
-      </c>
       <c r="D18" s="2" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="E18" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>212</v>
+        <v>206</v>
       </c>
       <c r="G18" s="2" t="s">
         <v>13</v>
@@ -3383,22 +3380,22 @@
     </row>
     <row r="19" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="C19" s="2" t="s">
         <v>234</v>
       </c>
-      <c r="B19" s="2" t="s">
-        <v>195</v>
-      </c>
-      <c r="C19" s="2" t="s">
-        <v>235</v>
-      </c>
       <c r="D19" s="2" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="E19" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>212</v>
+        <v>206</v>
       </c>
       <c r="G19" s="2" t="s">
         <v>13</v>
@@ -3406,22 +3403,22 @@
     </row>
     <row r="20" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="C20" s="2" t="s">
         <v>236</v>
       </c>
-      <c r="B20" s="2" t="s">
-        <v>195</v>
-      </c>
-      <c r="C20" s="2" t="s">
-        <v>237</v>
-      </c>
       <c r="D20" s="2" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="E20" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>212</v>
+        <v>206</v>
       </c>
       <c r="G20" s="2" t="s">
         <v>13</v>
@@ -3429,22 +3426,22 @@
     </row>
     <row r="21" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="C21" s="2" t="s">
         <v>238</v>
       </c>
-      <c r="B21" s="2" t="s">
-        <v>195</v>
-      </c>
-      <c r="C21" s="2" t="s">
-        <v>239</v>
-      </c>
       <c r="D21" s="2" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="E21" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
       <c r="G21" s="2" t="s">
         <v>13</v>
@@ -3495,22 +3492,22 @@
     </row>
     <row r="2" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
+        <v>239</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>240</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="C2" s="2" t="s">
         <v>241</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>242</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>241</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>243</v>
       </c>
       <c r="G2" s="2" t="s">
         <v>13</v>
@@ -3518,22 +3515,22 @@
     </row>
     <row r="3" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>244</v>
       </c>
-      <c r="B3" s="2" t="s">
-        <v>241</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>245</v>
-      </c>
       <c r="D3" s="2" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="E3" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>246</v>
+        <v>34</v>
       </c>
       <c r="G3" s="2" t="s">
         <v>13</v>
@@ -3541,22 +3538,22 @@
     </row>
     <row r="4" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
+        <v>245</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>246</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F4" s="2" t="s">
         <v>247</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>241</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>248</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>241</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>249</v>
       </c>
       <c r="G4" s="2" t="s">
         <v>13</v>
@@ -3564,22 +3561,22 @@
     </row>
     <row r="5" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="E5" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
       <c r="G5" s="2" t="s">
         <v>13</v>
@@ -3587,22 +3584,22 @@
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
+        <v>250</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F6" s="2" t="s">
         <v>252</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>241</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>253</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>241</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>254</v>
       </c>
       <c r="G6" s="2" t="s">
         <v>13</v>
@@ -3610,22 +3607,22 @@
     </row>
     <row r="7" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
+        <v>253</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F7" s="2" t="s">
         <v>255</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>241</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>256</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>241</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F7" s="2" t="s">
-        <v>64</v>
       </c>
       <c r="G7" s="2" t="s">
         <v>13</v>
@@ -3633,22 +3630,22 @@
     </row>
     <row r="8" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
+        <v>256</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="C8" s="2" t="s">
         <v>257</v>
       </c>
-      <c r="B8" s="2" t="s">
-        <v>241</v>
-      </c>
-      <c r="C8" s="2" t="s">
+      <c r="D8" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F8" s="2" t="s">
         <v>258</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>241</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F8" s="2" t="s">
-        <v>259</v>
       </c>
       <c r="G8" s="2" t="s">
         <v>13</v>
@@ -3656,22 +3653,22 @@
     </row>
     <row r="9" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="C9" s="2" t="s">
         <v>260</v>
       </c>
-      <c r="B9" s="2" t="s">
-        <v>241</v>
-      </c>
-      <c r="C9" s="2" t="s">
+      <c r="D9" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F9" s="2" t="s">
         <v>261</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>241</v>
-      </c>
-      <c r="E9" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F9" s="2" t="s">
-        <v>22</v>
       </c>
       <c r="G9" s="2" t="s">
         <v>13</v>
@@ -3682,7 +3679,7 @@
         <v>262</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>263</v>
@@ -3705,7 +3702,7 @@
         <v>266</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="C11" s="2" t="s">
         <v>267</v>
@@ -3717,7 +3714,7 @@
         <v>11</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>212</v>
+        <v>206</v>
       </c>
       <c r="G11" s="2" t="s">
         <v>13</v>
@@ -3728,13 +3725,13 @@
         <v>268</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>269</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="E12" s="3" t="s">
         <v>11</v>
@@ -3751,13 +3748,13 @@
         <v>271</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>272</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="E13" s="3" t="s">
         <v>11</v>
@@ -3774,19 +3771,19 @@
         <v>274</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="C14" s="2" t="s">
         <v>275</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="E14" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>212</v>
+        <v>199</v>
       </c>
       <c r="G14" s="2" t="s">
         <v>13</v>
@@ -3797,13 +3794,13 @@
         <v>276</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="C15" s="2" t="s">
         <v>277</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="E15" s="3" t="s">
         <v>11</v>
@@ -3820,7 +3817,7 @@
         <v>279</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="C16" s="2" t="s">
         <v>280</v>
@@ -3944,7 +3941,7 @@
         <v>11</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="G4" s="2" t="s">
         <v>13</v>
@@ -3990,7 +3987,7 @@
         <v>11</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>212</v>
+        <v>206</v>
       </c>
       <c r="G6" s="2" t="s">
         <v>13</v>
@@ -4082,7 +4079,7 @@
         <v>11</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>308</v>
+        <v>209</v>
       </c>
       <c r="G10" s="2" t="s">
         <v>13</v>
@@ -4090,13 +4087,13 @@
     </row>
     <row r="11" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="B11" s="2" t="s">
         <v>283</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="D11" s="2" t="s">
         <v>283</v>
@@ -4105,7 +4102,7 @@
         <v>11</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>212</v>
+        <v>206</v>
       </c>
       <c r="G11" s="2" t="s">
         <v>13</v>

</xml_diff>

<commit_message>
Add GitHub Actions workflow to run E2E web tests and archive the Excel report artifact
</commit_message>
<xml_diff>
--- a/tests/reports/Test_Analysis_Report.xlsx
+++ b/tests/reports/Test_Analysis_Report.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="805" uniqueCount="310">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="805" uniqueCount="304">
   <si>
     <t>Test ID</t>
   </si>
@@ -56,7 +56,7 @@
     <t>Passed</t>
   </si>
   <si>
-    <t>10049ms</t>
+    <t>2898ms</t>
   </si>
   <si>
     <t>Assertion passed successfully</t>
@@ -68,7 +68,7 @@
     <t>Verify brand name PayBuddy header exists</t>
   </si>
   <si>
-    <t>89ms</t>
+    <t>241ms</t>
   </si>
   <si>
     <t>TC-WEB-UI-003</t>
@@ -77,693 +77,672 @@
     <t>Verify form email input label</t>
   </si>
   <si>
+    <t>15ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-004</t>
+  </si>
+  <si>
+    <t>Verify form password input label</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-005</t>
+  </si>
+  <si>
+    <t>Verify Sign In button is present</t>
+  </si>
+  <si>
+    <t>12ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-006</t>
+  </si>
+  <si>
+    <t>Verify secure access footer notice is present</t>
+  </si>
+  <si>
+    <t>13ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-007</t>
+  </si>
+  <si>
+    <t>Verify branding subtitle text exists</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-008</t>
+  </si>
+  <si>
+    <t>Verify email input field placeholder</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-009</t>
+  </si>
+  <si>
+    <t>Verify password input field placeholder</t>
+  </si>
+  <si>
+    <t>14ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-010</t>
+  </si>
+  <si>
+    <t>Verify font family CSS on headers</t>
+  </si>
+  <si>
+    <t>17ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-011</t>
+  </si>
+  <si>
+    <t>Verify primary brand color on buttons</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-012</t>
+  </si>
+  <si>
+    <t>Verify centered block layout</t>
+  </si>
+  <si>
+    <t>16ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-013</t>
+  </si>
+  <si>
+    <t>Verify responsive structure at mobile width 360px</t>
+  </si>
+  <si>
+    <t>908ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-014</t>
+  </si>
+  <si>
+    <t>Verify responsive structure at tablet width 768px</t>
+  </si>
+  <si>
+    <t>904ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-015</t>
+  </si>
+  <si>
+    <t>Restore browser window maximization state</t>
+  </si>
+  <si>
+    <t>34ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-016</t>
+  </si>
+  <si>
+    <t>Verify HTML tag specification for email input</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-017</t>
+  </si>
+  <si>
+    <t>Verify HTML tag specification for password input</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-018</t>
+  </si>
+  <si>
+    <t>Verify card wrapper styles (border-radius)</t>
+  </si>
+  <si>
+    <t>20ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-019</t>
+  </si>
+  <si>
+    <t>Verify background styling matches design spec</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-020</t>
+  </si>
+  <si>
+    <t>Verify focus state click handler does not crash</t>
+  </si>
+  <si>
+    <t>90ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-021</t>
+  </si>
+  <si>
+    <t>Verify top-level container viewport classes</t>
+  </si>
+  <si>
+    <t>24ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-022</t>
+  </si>
+  <si>
+    <t>Verify branding and form division layout margins</t>
+  </si>
+  <si>
+    <t>42ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-023</t>
+  </si>
+  <si>
+    <t>Verify clear textual contrast for reader accessibility</t>
+  </si>
+  <si>
+    <t>25ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-024</t>
+  </si>
+  <si>
+    <t>Verify page scales properly without layout clipping</t>
+  </si>
+  <si>
+    <t>23ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-025</t>
+  </si>
+  <si>
+    <t>Verify smooth interactive transitions on button inputs</t>
+  </si>
+  <si>
+    <t>19ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-001</t>
+  </si>
+  <si>
+    <t>Functional</t>
+  </si>
+  <si>
+    <t>Verify invalid login rejection message</t>
+  </si>
+  <si>
+    <t>2371ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-002</t>
+  </si>
+  <si>
+    <t>Verify rejection of nonexistent email</t>
+  </si>
+  <si>
+    <t>784ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-003</t>
+  </si>
+  <si>
+    <t>Verify successful login with valid credentials redirects to Dashboard</t>
+  </si>
+  <si>
+    <t>1610ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-004</t>
+  </si>
+  <si>
+    <t>Verify dashboard displays Total Customers count</t>
+  </si>
+  <si>
+    <t>247ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-005</t>
+  </si>
+  <si>
+    <t>Verify dashboard displays Active Sales count</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-006</t>
+  </si>
+  <si>
+    <t>Verify dashboard displays Pending Installments count</t>
+  </si>
+  <si>
+    <t>18ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-007</t>
+  </si>
+  <si>
+    <t>Verify dashboard displays Today's Due count</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-008</t>
+  </si>
+  <si>
+    <t>Verify dashboard displays Outstanding Balance amount</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-009</t>
+  </si>
+  <si>
+    <t>Navigate to customers page and verify header</t>
+  </si>
+  <si>
+    <t>129ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-010</t>
+  </si>
+  <si>
+    <t>Verify add new customer input inputs are present</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-011</t>
+  </si>
+  <si>
+    <t>Verify customer creation and entry addition to table</t>
+  </si>
+  <si>
+    <t>2346ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-012</t>
+  </si>
+  <si>
+    <t>Verify presence of seeded customer</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-013</t>
+  </si>
+  <si>
+    <t>Navigate to specific customer profile page</t>
+  </si>
+  <si>
+    <t>989ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-014</t>
+  </si>
+  <si>
+    <t>Verify phone number exists on profile detail bar</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-015</t>
+  </si>
+  <si>
+    <t>Verify Total Amount financial card is 1000 INR</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-016</t>
+  </si>
+  <si>
+    <t>Verify Paid Amount financial card is 0 INR</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-017</t>
+  </si>
+  <si>
+    <t>Verify Outstanding Balance financial card is 1000 INR</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-018</t>
+  </si>
+  <si>
+    <t>Verify E2E Test Item pending sale is loaded in sales list</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-019</t>
+  </si>
+  <si>
+    <t>Verify redirect to record payment page</t>
+  </si>
+  <si>
+    <t>790ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-020</t>
+  </si>
+  <si>
+    <t>Verify remaining balance display match before payment</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-021</t>
+  </si>
+  <si>
+    <t>Record payment E2E execution and redirection validation</t>
+  </si>
+  <si>
+    <t>2821ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-022</t>
+  </si>
+  <si>
+    <t>Verify Outstanding Balance updates to 800 INR in customer card</t>
+  </si>
+  <si>
+    <t>1140ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-023</t>
+  </si>
+  <si>
+    <t>Verify Paid Amount updates to 200 INR in customer card</t>
+  </si>
+  <si>
+    <t>11ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-024</t>
+  </si>
+  <si>
+    <t>Verify recorded payment entry list matches mode UPI</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-025</t>
+  </si>
+  <si>
+    <t>Verify sales management index loads properly</t>
+  </si>
+  <si>
+    <t>552ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-026</t>
+  </si>
+  <si>
+    <t>Verify sales search filter works properly</t>
+  </si>
+  <si>
+    <t>626ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-027</t>
+  </si>
+  <si>
+    <t>Navigate to Create New Sale form</t>
+  </si>
+  <si>
+    <t>840ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-028</t>
+  </si>
+  <si>
+    <t>Verify total amount computed automatically (2 x 500 = 1000)</t>
+  </si>
+  <si>
+    <t>231ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-029</t>
+  </si>
+  <si>
+    <t>Create sale and verify redirect back to sales table</t>
+  </si>
+  <si>
+    <t>204ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-030</t>
+  </si>
+  <si>
+    <t>Verify Payments page path and title</t>
+  </si>
+  <si>
+    <t>574ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-031</t>
+  </si>
+  <si>
+    <t>Verify E2E transaction exists in master list</t>
+  </si>
+  <si>
+    <t>33ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-032</t>
+  </si>
+  <si>
+    <t>Verify Ledger Book page loads</t>
+  </si>
+  <si>
+    <t>827ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-033</t>
+  </si>
+  <si>
+    <t>Verify ledger records contain client name</t>
+  </si>
+  <si>
+    <t>31ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-034</t>
+  </si>
+  <si>
+    <t>Verify Installments page title</t>
+  </si>
+  <si>
+    <t>562ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-035</t>
+  </si>
+  <si>
+    <t>Verify customer details exist on installment board</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-036</t>
+  </si>
+  <si>
+    <t>Verify direct Dashboard URL redirect</t>
+  </si>
+  <si>
+    <t>99ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-037</t>
+  </si>
+  <si>
+    <t>Verify customer data updates dynamically on UI edit</t>
+  </si>
+  <si>
+    <t>4236ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-038</t>
+  </si>
+  <si>
+    <t>Verify logout route terminates session and redirects to sign in</t>
+  </si>
+  <si>
+    <t>608ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-039</t>
+  </si>
+  <si>
+    <t>Verify unauthorized dashboard access redirects to login</t>
+  </si>
+  <si>
+    <t>2158ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-040</t>
+  </si>
+  <si>
+    <t>Verify unauthorized customer details access redirects to login</t>
+  </si>
+  <si>
+    <t>2808ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UNIT-001</t>
+  </si>
+  <si>
+    <t>Unit</t>
+  </si>
+  <si>
+    <t>Test formatCurrency formatting positive amount</t>
+  </si>
+  <si>
     <t>56ms</t>
   </si>
   <si>
-    <t>TC-WEB-UI-004</t>
-  </si>
-  <si>
-    <t>Verify form password input label</t>
-  </si>
-  <si>
-    <t>42ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UI-005</t>
-  </si>
-  <si>
-    <t>Verify Sign In button is present</t>
-  </si>
-  <si>
-    <t>41ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UI-006</t>
-  </si>
-  <si>
-    <t>Verify secure access footer notice is present</t>
-  </si>
-  <si>
-    <t>32ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UI-007</t>
-  </si>
-  <si>
-    <t>Verify branding subtitle text exists</t>
-  </si>
-  <si>
-    <t>35ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UI-008</t>
-  </si>
-  <si>
-    <t>Verify email input field placeholder</t>
-  </si>
-  <si>
-    <t>34ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UI-009</t>
-  </si>
-  <si>
-    <t>Verify password input field placeholder</t>
-  </si>
-  <si>
-    <t>31ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UI-010</t>
-  </si>
-  <si>
-    <t>Verify font family CSS on headers</t>
-  </si>
-  <si>
-    <t>39ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UI-011</t>
-  </si>
-  <si>
-    <t>Verify primary brand color on buttons</t>
-  </si>
-  <si>
-    <t>TC-WEB-UI-012</t>
-  </si>
-  <si>
-    <t>Verify centered block layout</t>
-  </si>
-  <si>
-    <t>TC-WEB-UI-013</t>
-  </si>
-  <si>
-    <t>Verify responsive structure at mobile width 360px</t>
-  </si>
-  <si>
-    <t>922ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UI-014</t>
-  </si>
-  <si>
-    <t>Verify responsive structure at tablet width 768px</t>
-  </si>
-  <si>
-    <t>921ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UI-015</t>
-  </si>
-  <si>
-    <t>Restore browser window maximization state</t>
-  </si>
-  <si>
-    <t>49ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UI-016</t>
-  </si>
-  <si>
-    <t>Verify HTML tag specification for email input</t>
-  </si>
-  <si>
-    <t>61ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UI-017</t>
-  </si>
-  <si>
-    <t>Verify HTML tag specification for password input</t>
-  </si>
-  <si>
-    <t>TC-WEB-UI-018</t>
-  </si>
-  <si>
-    <t>Verify card wrapper styles (border-radius)</t>
-  </si>
-  <si>
-    <t>47ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UI-019</t>
-  </si>
-  <si>
-    <t>Verify background styling matches design spec</t>
-  </si>
-  <si>
-    <t>43ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UI-020</t>
-  </si>
-  <si>
-    <t>Verify focus state click handler does not crash</t>
-  </si>
-  <si>
-    <t>196ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UI-021</t>
-  </si>
-  <si>
-    <t>Verify top-level container viewport classes</t>
-  </si>
-  <si>
-    <t>51ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UI-022</t>
-  </si>
-  <si>
-    <t>Verify branding and form division layout margins</t>
-  </si>
-  <si>
-    <t>36ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UI-023</t>
-  </si>
-  <si>
-    <t>Verify clear textual contrast for reader accessibility</t>
-  </si>
-  <si>
-    <t>TC-WEB-UI-024</t>
-  </si>
-  <si>
-    <t>Verify page scales properly without layout clipping</t>
-  </si>
-  <si>
-    <t>54ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UI-025</t>
-  </si>
-  <si>
-    <t>Verify smooth interactive transitions on button inputs</t>
-  </si>
-  <si>
-    <t>30ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-001</t>
-  </si>
-  <si>
-    <t>Functional</t>
-  </si>
-  <si>
-    <t>Verify invalid login rejection message</t>
-  </si>
-  <si>
-    <t>3917ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-002</t>
-  </si>
-  <si>
-    <t>Verify rejection of nonexistent email</t>
-  </si>
-  <si>
-    <t>3709ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-003</t>
-  </si>
-  <si>
-    <t>Verify successful login with valid credentials redirects to Dashboard</t>
-  </si>
-  <si>
-    <t>3328ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-004</t>
-  </si>
-  <si>
-    <t>Verify dashboard displays Total Customers count</t>
-  </si>
-  <si>
-    <t>944ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-005</t>
-  </si>
-  <si>
-    <t>Verify dashboard displays Active Sales count</t>
+    <t>TC-WEB-UNIT-002</t>
+  </si>
+  <si>
+    <t>Test formatCurrency formatting zero amount</t>
+  </si>
+  <si>
+    <t>0ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UNIT-003</t>
+  </si>
+  <si>
+    <t>Test formatCurrency formatting negative amount</t>
+  </si>
+  <si>
+    <t>TC-WEB-UNIT-004</t>
+  </si>
+  <si>
+    <t>Test formatCurrency formatting large millions scale amount</t>
+  </si>
+  <si>
+    <t>1ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UNIT-005</t>
+  </si>
+  <si>
+    <t>Test formatCurrency decimal rounding functionality</t>
+  </si>
+  <si>
+    <t>TC-WEB-UNIT-006</t>
+  </si>
+  <si>
+    <t>Test formatDate string matching date details</t>
+  </si>
+  <si>
+    <t>9ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UNIT-007</t>
+  </si>
+  <si>
+    <t>Test formatDate fallback for null values</t>
+  </si>
+  <si>
+    <t>TC-WEB-UNIT-008</t>
+  </si>
+  <si>
+    <t>Test formatDate fallback for 0 value</t>
+  </si>
+  <si>
+    <t>TC-WEB-UNIT-009</t>
+  </si>
+  <si>
+    <t>Test formatDateTime details formatting</t>
+  </si>
+  <si>
+    <t>TC-WEB-UNIT-010</t>
+  </si>
+  <si>
+    <t>Test formatDateTime null timestamp handling</t>
+  </si>
+  <si>
+    <t>TC-WEB-UNIT-011</t>
+  </si>
+  <si>
+    <t>Verify email validation for valid string</t>
+  </si>
+  <si>
+    <t>TC-WEB-UNIT-012</t>
+  </si>
+  <si>
+    <t>Verify email validation blocks missing TLD</t>
+  </si>
+  <si>
+    <t>TC-WEB-UNIT-013</t>
+  </si>
+  <si>
+    <t>Verify email validation blocks missing alias prefix</t>
+  </si>
+  <si>
+    <t>TC-WEB-UNIT-014</t>
+  </si>
+  <si>
+    <t>Verify phone validation for standard 10 digit number</t>
+  </si>
+  <si>
+    <t>TC-WEB-UNIT-015</t>
+  </si>
+  <si>
+    <t>Verify phone validation blocks short length</t>
+  </si>
+  <si>
+    <t>TC-WEB-UNIT-016</t>
+  </si>
+  <si>
+    <t>Verify phone validation blocks alphabetic characters</t>
+  </si>
+  <si>
+    <t>TC-WEB-UNIT-017</t>
+  </si>
+  <si>
+    <t>Verify interest formula multiplication logic</t>
+  </si>
+  <si>
+    <t>TC-WEB-UNIT-018</t>
+  </si>
+  <si>
+    <t>Verify installment partitioning amount division</t>
+  </si>
+  <si>
+    <t>TC-WEB-UNIT-019</t>
+  </si>
+  <si>
+    <t>Verify remaining balance arithmetic subtraction</t>
+  </si>
+  <si>
+    <t>TC-WEB-UNIT-020</t>
+  </si>
+  <si>
+    <t>Verify mock environment manifest validator passes</t>
+  </si>
+  <si>
+    <t>TC-WEB-VAL-001</t>
+  </si>
+  <si>
+    <t>Validation</t>
+  </si>
+  <si>
+    <t>Verify email required constraint is enabled on form</t>
+  </si>
+  <si>
+    <t>330ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-VAL-002</t>
+  </si>
+  <si>
+    <t>Verify password required constraint is enabled on form</t>
+  </si>
+  <si>
+    <t>TC-WEB-VAL-003</t>
+  </si>
+  <si>
+    <t>Verify browser client blocks submissions for invalid email inputs</t>
   </si>
   <si>
     <t>76ms</t>
   </si>
   <si>
-    <t>TC-WEB-FUNC-006</t>
-  </si>
-  <si>
-    <t>Verify dashboard displays Pending Installments count</t>
-  </si>
-  <si>
-    <t>48ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-007</t>
-  </si>
-  <si>
-    <t>Verify dashboard displays Today's Due count</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-008</t>
-  </si>
-  <si>
-    <t>Verify dashboard displays Outstanding Balance amount</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-009</t>
-  </si>
-  <si>
-    <t>Navigate to customers page and verify header</t>
-  </si>
-  <si>
-    <t>205ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-010</t>
-  </si>
-  <si>
-    <t>Verify add new customer input inputs are present</t>
-  </si>
-  <si>
-    <t>50ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-011</t>
-  </si>
-  <si>
-    <t>Verify customer creation and entry addition to table</t>
-  </si>
-  <si>
-    <t>2597ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-012</t>
-  </si>
-  <si>
-    <t>Verify presence of seeded customer</t>
-  </si>
-  <si>
-    <t>55ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-013</t>
-  </si>
-  <si>
-    <t>Navigate to specific customer profile page</t>
-  </si>
-  <si>
-    <t>1731ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-014</t>
-  </si>
-  <si>
-    <t>Verify phone number exists on profile detail bar</t>
-  </si>
-  <si>
-    <t>38ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-015</t>
-  </si>
-  <si>
-    <t>Verify Total Amount financial card is 1000 INR</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-016</t>
-  </si>
-  <si>
-    <t>Verify Paid Amount financial card is 0 INR</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-017</t>
-  </si>
-  <si>
-    <t>Verify Outstanding Balance financial card is 1000 INR</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-018</t>
-  </si>
-  <si>
-    <t>Verify E2E Test Item pending sale is loaded in sales list</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-019</t>
-  </si>
-  <si>
-    <t>Verify redirect to record payment page</t>
-  </si>
-  <si>
-    <t>1312ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-020</t>
-  </si>
-  <si>
-    <t>Verify remaining balance display match before payment</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-021</t>
-  </si>
-  <si>
-    <t>Record payment E2E execution and redirection validation</t>
-  </si>
-  <si>
-    <t>3421ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-022</t>
-  </si>
-  <si>
-    <t>Verify Outstanding Balance updates to 800 INR in customer card</t>
-  </si>
-  <si>
-    <t>1998ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-023</t>
-  </si>
-  <si>
-    <t>Verify Paid Amount updates to 200 INR in customer card</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-024</t>
-  </si>
-  <si>
-    <t>Verify recorded payment entry list matches mode UPI</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-025</t>
-  </si>
-  <si>
-    <t>Verify sales management index loads properly</t>
-  </si>
-  <si>
-    <t>1151ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-026</t>
-  </si>
-  <si>
-    <t>Verify sales search filter works properly</t>
-  </si>
-  <si>
-    <t>784ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-027</t>
-  </si>
-  <si>
-    <t>Navigate to Create New Sale form</t>
-  </si>
-  <si>
-    <t>1201ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-028</t>
-  </si>
-  <si>
-    <t>Verify total amount computed automatically (2 x 500 = 1000)</t>
-  </si>
-  <si>
-    <t>675ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-029</t>
-  </si>
-  <si>
-    <t>Create sale and verify redirect back to sales table</t>
-  </si>
-  <si>
-    <t>447ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-030</t>
-  </si>
-  <si>
-    <t>Verify Payments page path and title</t>
-  </si>
-  <si>
-    <t>2540ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-031</t>
-  </si>
-  <si>
-    <t>Verify E2E transaction exists in master list</t>
-  </si>
-  <si>
-    <t>52ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-032</t>
-  </si>
-  <si>
-    <t>Verify Ledger Book page loads</t>
-  </si>
-  <si>
-    <t>1580ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-033</t>
-  </si>
-  <si>
-    <t>Verify ledger records contain client name</t>
-  </si>
-  <si>
-    <t>73ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-034</t>
-  </si>
-  <si>
-    <t>Verify Installments page title</t>
-  </si>
-  <si>
-    <t>1056ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-035</t>
-  </si>
-  <si>
-    <t>Verify customer details exist on installment board</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-036</t>
-  </si>
-  <si>
-    <t>Verify direct Dashboard URL redirect</t>
-  </si>
-  <si>
-    <t>775ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-037</t>
-  </si>
-  <si>
-    <t>Verify customer data updates dynamically on UI edit</t>
-  </si>
-  <si>
-    <t>4643ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-038</t>
-  </si>
-  <si>
-    <t>Verify logout route terminates session and redirects to sign in</t>
-  </si>
-  <si>
-    <t>1664ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-039</t>
-  </si>
-  <si>
-    <t>Verify unauthorized dashboard access redirects to login</t>
-  </si>
-  <si>
-    <t>2406ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-040</t>
-  </si>
-  <si>
-    <t>Verify unauthorized customer details access redirects to login</t>
-  </si>
-  <si>
-    <t>2228ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UNIT-001</t>
-  </si>
-  <si>
-    <t>Unit</t>
-  </si>
-  <si>
-    <t>Test formatCurrency formatting positive amount</t>
-  </si>
-  <si>
-    <t>78ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UNIT-002</t>
-  </si>
-  <si>
-    <t>Test formatCurrency formatting zero amount</t>
-  </si>
-  <si>
-    <t>1ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UNIT-003</t>
-  </si>
-  <si>
-    <t>Test formatCurrency formatting negative amount</t>
-  </si>
-  <si>
-    <t>TC-WEB-UNIT-004</t>
-  </si>
-  <si>
-    <t>Test formatCurrency formatting large millions scale amount</t>
-  </si>
-  <si>
-    <t>TC-WEB-UNIT-005</t>
-  </si>
-  <si>
-    <t>Test formatCurrency decimal rounding functionality</t>
-  </si>
-  <si>
-    <t>0ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UNIT-006</t>
-  </si>
-  <si>
-    <t>Test formatDate string matching date details</t>
-  </si>
-  <si>
-    <t>17ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UNIT-007</t>
-  </si>
-  <si>
-    <t>Test formatDate fallback for null values</t>
-  </si>
-  <si>
-    <t>TC-WEB-UNIT-008</t>
-  </si>
-  <si>
-    <t>Test formatDate fallback for 0 value</t>
-  </si>
-  <si>
-    <t>TC-WEB-UNIT-009</t>
-  </si>
-  <si>
-    <t>Test formatDateTime details formatting</t>
-  </si>
-  <si>
-    <t>2ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UNIT-010</t>
-  </si>
-  <si>
-    <t>Test formatDateTime null timestamp handling</t>
-  </si>
-  <si>
-    <t>TC-WEB-UNIT-011</t>
-  </si>
-  <si>
-    <t>Verify email validation for valid string</t>
-  </si>
-  <si>
-    <t>TC-WEB-UNIT-012</t>
-  </si>
-  <si>
-    <t>Verify email validation blocks missing TLD</t>
-  </si>
-  <si>
-    <t>TC-WEB-UNIT-013</t>
-  </si>
-  <si>
-    <t>Verify email validation blocks missing alias prefix</t>
-  </si>
-  <si>
-    <t>TC-WEB-UNIT-014</t>
-  </si>
-  <si>
-    <t>Verify phone validation for standard 10 digit number</t>
-  </si>
-  <si>
-    <t>TC-WEB-UNIT-015</t>
-  </si>
-  <si>
-    <t>Verify phone validation blocks short length</t>
-  </si>
-  <si>
-    <t>TC-WEB-UNIT-016</t>
-  </si>
-  <si>
-    <t>Verify phone validation blocks alphabetic characters</t>
-  </si>
-  <si>
-    <t>TC-WEB-UNIT-017</t>
-  </si>
-  <si>
-    <t>Verify interest formula multiplication logic</t>
-  </si>
-  <si>
-    <t>TC-WEB-UNIT-018</t>
-  </si>
-  <si>
-    <t>Verify installment partitioning amount division</t>
-  </si>
-  <si>
-    <t>TC-WEB-UNIT-019</t>
-  </si>
-  <si>
-    <t>Verify remaining balance arithmetic subtraction</t>
-  </si>
-  <si>
-    <t>TC-WEB-UNIT-020</t>
-  </si>
-  <si>
-    <t>Verify mock environment manifest validator passes</t>
-  </si>
-  <si>
-    <t>TC-WEB-VAL-001</t>
-  </si>
-  <si>
-    <t>Validation</t>
-  </si>
-  <si>
-    <t>Verify email required constraint is enabled on form</t>
-  </si>
-  <si>
-    <t>330ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-VAL-002</t>
-  </si>
-  <si>
-    <t>Verify password required constraint is enabled on form</t>
-  </si>
-  <si>
-    <t>TC-WEB-VAL-003</t>
-  </si>
-  <si>
-    <t>Verify browser client blocks submissions for invalid email inputs</t>
-  </si>
-  <si>
-    <t>245ms</t>
-  </si>
-  <si>
     <t>TC-WEB-VAL-004</t>
   </si>
   <si>
@@ -776,7 +755,7 @@
     <t>Verify customer creation form prevents empty submit</t>
   </si>
   <si>
-    <t>4492ms</t>
+    <t>3054ms</t>
   </si>
   <si>
     <t>TC-WEB-VAL-006</t>
@@ -785,7 +764,7 @@
     <t>Verify phone input uses tel semantic element type</t>
   </si>
   <si>
-    <t>27ms</t>
+    <t>22ms</t>
   </si>
   <si>
     <t>TC-WEB-VAL-007</t>
@@ -794,7 +773,7 @@
     <t>Verify sale quantity requires positive minimum value (&gt; 0)</t>
   </si>
   <si>
-    <t>1009ms</t>
+    <t>600ms</t>
   </si>
   <si>
     <t>TC-WEB-VAL-008</t>
@@ -803,7 +782,7 @@
     <t>Verify unit price input restricts negative numbers</t>
   </si>
   <si>
-    <t>24ms</t>
+    <t>10ms</t>
   </si>
   <si>
     <t>TC-WEB-VAL-009</t>
@@ -815,7 +794,7 @@
     <t>Security</t>
   </si>
   <si>
-    <t>2423ms</t>
+    <t>1904ms</t>
   </si>
   <si>
     <t>TC-WEB-VAL-010</t>
@@ -830,7 +809,7 @@
     <t>Verify error prevents overpayment collections</t>
   </si>
   <si>
-    <t>3061ms</t>
+    <t>1909ms</t>
   </si>
   <si>
     <t>TC-WEB-VAL-012</t>
@@ -839,7 +818,7 @@
     <t>Verify collection input restricts 0 value submissions</t>
   </si>
   <si>
-    <t>1384ms</t>
+    <t>1123ms</t>
   </si>
   <si>
     <t>TC-WEB-VAL-013</t>
@@ -854,7 +833,7 @@
     <t>Verify wildcard URLs redirect to main route base</t>
   </si>
   <si>
-    <t>4117ms</t>
+    <t>2113ms</t>
   </si>
   <si>
     <t>TC-WEB-VAL-015</t>
@@ -863,7 +842,7 @@
     <t>Verify HTML password hidden mask attribute config</t>
   </si>
   <si>
-    <t>2036ms</t>
+    <t>602ms</t>
   </si>
   <si>
     <t>TC-WEB-DEP-001</t>
@@ -878,7 +857,7 @@
     <t>Performance</t>
   </si>
   <si>
-    <t>527ms</t>
+    <t>107ms</t>
   </si>
   <si>
     <t>TC-WEB-DEP-002</t>
@@ -887,7 +866,7 @@
     <t>Verify full render transition load time under limit</t>
   </si>
   <si>
-    <t>2200ms</t>
+    <t>1149ms</t>
   </si>
   <si>
     <t>TC-WEB-DEP-003</t>
@@ -902,7 +881,7 @@
     <t>Verify favicon.ico endpoint yields clean HTTP status</t>
   </si>
   <si>
-    <t>358ms</t>
+    <t>94ms</t>
   </si>
   <si>
     <t>TC-WEB-DEP-005</t>
@@ -917,7 +896,7 @@
     <t>Verify head links contain manifest registration details</t>
   </si>
   <si>
-    <t>798ms</t>
+    <t>130ms</t>
   </si>
   <si>
     <t>TC-WEB-DEP-007</t>
@@ -926,7 +905,7 @@
     <t>Verify console logs have no severe exceptions during login page session</t>
   </si>
   <si>
-    <t>6ms</t>
+    <t>4ms</t>
   </si>
   <si>
     <t>TC-WEB-DEP-008</t>
@@ -935,13 +914,16 @@
     <t>Verify standard responsive layouts align horizontally</t>
   </si>
   <si>
-    <t>65ms</t>
+    <t>45ms</t>
   </si>
   <si>
     <t>TC-WEB-DEP-009</t>
   </si>
   <si>
     <t>Verify DOM count index scales cleanly</t>
+  </si>
+  <si>
+    <t>5ms</t>
   </si>
   <si>
     <t>TC-WEB-DEP-010</t>
@@ -1492,7 +1474,7 @@
         <v>11</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="G5" s="2" t="s">
         <v>13</v>
@@ -1500,13 +1482,13 @@
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>10</v>
@@ -1515,7 +1497,7 @@
         <v>11</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="G6" s="2" t="s">
         <v>13</v>
@@ -1523,13 +1505,13 @@
     </row>
     <row r="7" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>10</v>
@@ -1538,7 +1520,7 @@
         <v>11</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G7" s="2" t="s">
         <v>13</v>
@@ -1546,13 +1528,13 @@
     </row>
     <row r="8" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>10</v>
@@ -1561,7 +1543,7 @@
         <v>11</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="G8" s="2" t="s">
         <v>13</v>
@@ -1569,13 +1551,13 @@
     </row>
     <row r="9" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>10</v>
@@ -1584,7 +1566,7 @@
         <v>11</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="G9" s="2" t="s">
         <v>13</v>
@@ -1592,13 +1574,13 @@
     </row>
     <row r="10" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="D10" s="2" t="s">
         <v>10</v>
@@ -1607,7 +1589,7 @@
         <v>11</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="G10" s="2" t="s">
         <v>13</v>
@@ -1615,13 +1597,13 @@
     </row>
     <row r="11" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="B11" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="D11" s="2" t="s">
         <v>10</v>
@@ -1630,7 +1612,7 @@
         <v>11</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="G11" s="2" t="s">
         <v>13</v>
@@ -1638,13 +1620,13 @@
     </row>
     <row r="12" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="B12" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="D12" s="2" t="s">
         <v>10</v>
@@ -1653,7 +1635,7 @@
         <v>11</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="G12" s="2" t="s">
         <v>13</v>
@@ -1661,13 +1643,13 @@
     </row>
     <row r="13" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="B13" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="D13" s="2" t="s">
         <v>10</v>
@@ -1676,7 +1658,7 @@
         <v>11</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="G13" s="2" t="s">
         <v>13</v>
@@ -1684,13 +1666,13 @@
     </row>
     <row r="14" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B14" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="D14" s="2" t="s">
         <v>10</v>
@@ -1699,7 +1681,7 @@
         <v>11</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="G14" s="2" t="s">
         <v>13</v>
@@ -1707,13 +1689,13 @@
     </row>
     <row r="15" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B15" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="D15" s="2" t="s">
         <v>10</v>
@@ -1722,7 +1704,7 @@
         <v>11</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="G15" s="2" t="s">
         <v>13</v>
@@ -1730,13 +1712,13 @@
     </row>
     <row r="16" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B16" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="D16" s="2" t="s">
         <v>10</v>
@@ -1745,7 +1727,7 @@
         <v>11</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="G16" s="2" t="s">
         <v>13</v>
@@ -1753,13 +1735,13 @@
     </row>
     <row r="17" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B17" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="D17" s="2" t="s">
         <v>10</v>
@@ -1768,7 +1750,7 @@
         <v>11</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>56</v>
+        <v>37</v>
       </c>
       <c r="G17" s="2" t="s">
         <v>13</v>
@@ -1776,13 +1758,13 @@
     </row>
     <row r="18" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="B18" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="D18" s="2" t="s">
         <v>10</v>
@@ -1791,7 +1773,7 @@
         <v>11</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="G18" s="2" t="s">
         <v>13</v>
@@ -1799,13 +1781,13 @@
     </row>
     <row r="19" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="B19" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="D19" s="2" t="s">
         <v>10</v>
@@ -1814,7 +1796,7 @@
         <v>11</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="G19" s="2" t="s">
         <v>13</v>
@@ -1822,13 +1804,13 @@
     </row>
     <row r="20" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="B20" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="D20" s="2" t="s">
         <v>10</v>
@@ -1837,7 +1819,7 @@
         <v>11</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="G20" s="2" t="s">
         <v>13</v>
@@ -1845,13 +1827,13 @@
     </row>
     <row r="21" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="B21" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="D21" s="2" t="s">
         <v>10</v>
@@ -1860,7 +1842,7 @@
         <v>11</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="G21" s="2" t="s">
         <v>13</v>
@@ -1868,13 +1850,13 @@
     </row>
     <row r="22" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="B22" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="D22" s="2" t="s">
         <v>10</v>
@@ -1883,7 +1865,7 @@
         <v>11</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="G22" s="2" t="s">
         <v>13</v>
@@ -1891,13 +1873,13 @@
     </row>
     <row r="23" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="B23" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="D23" s="2" t="s">
         <v>10</v>
@@ -1906,7 +1888,7 @@
         <v>11</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="G23" s="2" t="s">
         <v>13</v>
@@ -1914,13 +1896,13 @@
     </row>
     <row r="24" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="B24" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="D24" s="2" t="s">
         <v>10</v>
@@ -1929,7 +1911,7 @@
         <v>11</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="G24" s="2" t="s">
         <v>13</v>
@@ -1937,13 +1919,13 @@
     </row>
     <row r="25" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="B25" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="D25" s="2" t="s">
         <v>10</v>
@@ -1952,7 +1934,7 @@
         <v>11</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="G25" s="2" t="s">
         <v>13</v>
@@ -1960,13 +1942,13 @@
     </row>
     <row r="26" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="B26" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="D26" s="2" t="s">
         <v>10</v>
@@ -1975,7 +1957,7 @@
         <v>11</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="G26" s="2" t="s">
         <v>13</v>
@@ -2026,22 +2008,22 @@
     </row>
     <row r="2" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>82</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>85</v>
       </c>
       <c r="G2" s="2" t="s">
         <v>13</v>
@@ -2049,22 +2031,22 @@
     </row>
     <row r="3" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="E3" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="G3" s="2" t="s">
         <v>13</v>
@@ -2072,22 +2054,22 @@
     </row>
     <row r="4" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="E4" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="G4" s="2" t="s">
         <v>13</v>
@@ -2095,22 +2077,22 @@
     </row>
     <row r="5" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="E5" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="G5" s="2" t="s">
         <v>13</v>
@@ -2118,22 +2100,22 @@
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="E6" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>97</v>
+        <v>78</v>
       </c>
       <c r="G6" s="2" t="s">
         <v>13</v>
@@ -2141,22 +2123,22 @@
     </row>
     <row r="7" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="E7" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="G7" s="2" t="s">
         <v>13</v>
@@ -2164,22 +2146,22 @@
     </row>
     <row r="8" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="E8" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>28</v>
+        <v>96</v>
       </c>
       <c r="G8" s="2" t="s">
         <v>13</v>
@@ -2187,22 +2169,22 @@
     </row>
     <row r="9" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="E9" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>78</v>
+        <v>42</v>
       </c>
       <c r="G9" s="2" t="s">
         <v>13</v>
@@ -2210,22 +2192,22 @@
     </row>
     <row r="10" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="E10" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="G10" s="2" t="s">
         <v>13</v>
@@ -2233,22 +2215,22 @@
     </row>
     <row r="11" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="E11" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>110</v>
+        <v>66</v>
       </c>
       <c r="G11" s="2" t="s">
         <v>13</v>
@@ -2256,22 +2238,22 @@
     </row>
     <row r="12" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>111</v>
+        <v>106</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="E12" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="G12" s="2" t="s">
         <v>13</v>
@@ -2279,22 +2261,22 @@
     </row>
     <row r="13" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>114</v>
+        <v>109</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="E13" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>116</v>
+        <v>27</v>
       </c>
       <c r="G13" s="2" t="s">
         <v>13</v>
@@ -2302,22 +2284,22 @@
     </row>
     <row r="14" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>118</v>
+        <v>112</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="E14" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>119</v>
+        <v>113</v>
       </c>
       <c r="G14" s="2" t="s">
         <v>13</v>
@@ -2325,22 +2307,22 @@
     </row>
     <row r="15" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>120</v>
+        <v>114</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>121</v>
+        <v>115</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="E15" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>122</v>
+        <v>27</v>
       </c>
       <c r="G15" s="2" t="s">
         <v>13</v>
@@ -2348,22 +2330,22 @@
     </row>
     <row r="16" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>123</v>
+        <v>116</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>124</v>
+        <v>117</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="E16" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>70</v>
+        <v>24</v>
       </c>
       <c r="G16" s="2" t="s">
         <v>13</v>
@@ -2371,22 +2353,22 @@
     </row>
     <row r="17" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>125</v>
+        <v>118</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>126</v>
+        <v>119</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="E17" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="G17" s="2" t="s">
         <v>13</v>
@@ -2394,22 +2376,22 @@
     </row>
     <row r="18" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>127</v>
+        <v>120</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>128</v>
+        <v>121</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="E18" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="G18" s="2" t="s">
         <v>13</v>
@@ -2417,22 +2399,22 @@
     </row>
     <row r="19" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>129</v>
+        <v>122</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>130</v>
+        <v>123</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="E19" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="G19" s="2" t="s">
         <v>13</v>
@@ -2440,22 +2422,22 @@
     </row>
     <row r="20" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>132</v>
+        <v>125</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="E20" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>133</v>
+        <v>126</v>
       </c>
       <c r="G20" s="2" t="s">
         <v>13</v>
@@ -2463,22 +2445,22 @@
     </row>
     <row r="21" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>134</v>
+        <v>127</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>135</v>
+        <v>128</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="E21" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>100</v>
+        <v>24</v>
       </c>
       <c r="G21" s="2" t="s">
         <v>13</v>
@@ -2486,22 +2468,22 @@
     </row>
     <row r="22" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>136</v>
+        <v>129</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>137</v>
+        <v>130</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="E22" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>138</v>
+        <v>131</v>
       </c>
       <c r="G22" s="2" t="s">
         <v>13</v>
@@ -2509,22 +2491,22 @@
     </row>
     <row r="23" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
-        <v>139</v>
+        <v>132</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>140</v>
+        <v>133</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="E23" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>141</v>
+        <v>134</v>
       </c>
       <c r="G23" s="2" t="s">
         <v>13</v>
@@ -2532,22 +2514,22 @@
     </row>
     <row r="24" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>142</v>
+        <v>135</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="E24" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>40</v>
+        <v>137</v>
       </c>
       <c r="G24" s="2" t="s">
         <v>13</v>
@@ -2555,22 +2537,22 @@
     </row>
     <row r="25" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
-        <v>144</v>
+        <v>138</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>145</v>
+        <v>139</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="E25" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>40</v>
+        <v>27</v>
       </c>
       <c r="G25" s="2" t="s">
         <v>13</v>
@@ -2578,22 +2560,22 @@
     </row>
     <row r="26" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
-        <v>146</v>
+        <v>140</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>147</v>
+        <v>141</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="E26" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="G26" s="2" t="s">
         <v>13</v>
@@ -2601,22 +2583,22 @@
     </row>
     <row r="27" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
-        <v>149</v>
+        <v>143</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>150</v>
+        <v>144</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="E27" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>151</v>
+        <v>145</v>
       </c>
       <c r="G27" s="2" t="s">
         <v>13</v>
@@ -2624,22 +2606,22 @@
     </row>
     <row r="28" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="E28" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F28" s="2" t="s">
-        <v>154</v>
+        <v>148</v>
       </c>
       <c r="G28" s="2" t="s">
         <v>13</v>
@@ -2647,22 +2629,22 @@
     </row>
     <row r="29" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
-        <v>155</v>
+        <v>149</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>156</v>
+        <v>150</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="E29" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F29" s="2" t="s">
-        <v>157</v>
+        <v>151</v>
       </c>
       <c r="G29" s="2" t="s">
         <v>13</v>
@@ -2670,22 +2652,22 @@
     </row>
     <row r="30" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
-        <v>158</v>
+        <v>152</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>159</v>
+        <v>153</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="E30" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F30" s="2" t="s">
-        <v>160</v>
+        <v>154</v>
       </c>
       <c r="G30" s="2" t="s">
         <v>13</v>
@@ -2693,22 +2675,22 @@
     </row>
     <row r="31" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
-        <v>161</v>
+        <v>155</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>162</v>
+        <v>156</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="E31" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F31" s="2" t="s">
-        <v>163</v>
+        <v>157</v>
       </c>
       <c r="G31" s="2" t="s">
         <v>13</v>
@@ -2716,22 +2698,22 @@
     </row>
     <row r="32" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
-        <v>164</v>
+        <v>158</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>165</v>
+        <v>159</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="E32" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F32" s="2" t="s">
-        <v>166</v>
+        <v>160</v>
       </c>
       <c r="G32" s="2" t="s">
         <v>13</v>
@@ -2739,22 +2721,22 @@
     </row>
     <row r="33" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
-        <v>167</v>
+        <v>161</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>168</v>
+        <v>162</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="E33" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F33" s="2" t="s">
-        <v>169</v>
+        <v>163</v>
       </c>
       <c r="G33" s="2" t="s">
         <v>13</v>
@@ -2762,22 +2744,22 @@
     </row>
     <row r="34" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
-        <v>170</v>
+        <v>164</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>171</v>
+        <v>165</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="E34" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F34" s="2" t="s">
-        <v>172</v>
+        <v>166</v>
       </c>
       <c r="G34" s="2" t="s">
         <v>13</v>
@@ -2785,22 +2767,22 @@
     </row>
     <row r="35" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
-        <v>173</v>
+        <v>167</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="E35" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F35" s="2" t="s">
-        <v>175</v>
+        <v>169</v>
       </c>
       <c r="G35" s="2" t="s">
         <v>13</v>
@@ -2808,22 +2790,22 @@
     </row>
     <row r="36" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
-        <v>176</v>
+        <v>170</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>177</v>
+        <v>171</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="E36" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F36" s="2" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="G36" s="2" t="s">
         <v>13</v>
@@ -2831,22 +2813,22 @@
     </row>
     <row r="37" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
-        <v>178</v>
+        <v>172</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>179</v>
+        <v>173</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="E37" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F37" s="2" t="s">
-        <v>180</v>
+        <v>174</v>
       </c>
       <c r="G37" s="2" t="s">
         <v>13</v>
@@ -2854,22 +2836,22 @@
     </row>
     <row r="38" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
-        <v>181</v>
+        <v>175</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>182</v>
+        <v>176</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="E38" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F38" s="2" t="s">
-        <v>183</v>
+        <v>177</v>
       </c>
       <c r="G38" s="2" t="s">
         <v>13</v>
@@ -2877,22 +2859,22 @@
     </row>
     <row r="39" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
-        <v>184</v>
+        <v>178</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>185</v>
+        <v>179</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="E39" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F39" s="2" t="s">
-        <v>186</v>
+        <v>180</v>
       </c>
       <c r="G39" s="2" t="s">
         <v>13</v>
@@ -2900,22 +2882,22 @@
     </row>
     <row r="40" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
-        <v>187</v>
+        <v>181</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>188</v>
+        <v>182</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="E40" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F40" s="2" t="s">
-        <v>189</v>
+        <v>183</v>
       </c>
       <c r="G40" s="2" t="s">
         <v>13</v>
@@ -2923,22 +2905,22 @@
     </row>
     <row r="41" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
-        <v>190</v>
+        <v>184</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>191</v>
+        <v>185</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="E41" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F41" s="2" t="s">
-        <v>192</v>
+        <v>186</v>
       </c>
       <c r="G41" s="2" t="s">
         <v>13</v>
@@ -2989,22 +2971,22 @@
     </row>
     <row r="2" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>193</v>
+        <v>187</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>195</v>
+        <v>189</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="E2" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="G2" s="2" t="s">
         <v>13</v>
@@ -3012,22 +2994,22 @@
     </row>
     <row r="3" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>197</v>
+        <v>191</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>198</v>
+        <v>192</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="E3" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>199</v>
+        <v>193</v>
       </c>
       <c r="G3" s="2" t="s">
         <v>13</v>
@@ -3035,22 +3017,22 @@
     </row>
     <row r="4" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>200</v>
+        <v>194</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="E4" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>199</v>
+        <v>193</v>
       </c>
       <c r="G4" s="2" t="s">
         <v>13</v>
@@ -3058,22 +3040,22 @@
     </row>
     <row r="5" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>202</v>
+        <v>196</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>203</v>
+        <v>197</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="E5" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="G5" s="2" t="s">
         <v>13</v>
@@ -3081,22 +3063,22 @@
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>204</v>
+        <v>199</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="E6" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>206</v>
+        <v>193</v>
       </c>
       <c r="G6" s="2" t="s">
         <v>13</v>
@@ -3104,22 +3086,22 @@
     </row>
     <row r="7" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>207</v>
+        <v>201</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>208</v>
+        <v>202</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="E7" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>209</v>
+        <v>203</v>
       </c>
       <c r="G7" s="2" t="s">
         <v>13</v>
@@ -3127,22 +3109,22 @@
     </row>
     <row r="8" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>210</v>
+        <v>204</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>211</v>
+        <v>205</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="E8" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>206</v>
+        <v>198</v>
       </c>
       <c r="G8" s="2" t="s">
         <v>13</v>
@@ -3150,22 +3132,22 @@
     </row>
     <row r="9" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>212</v>
+        <v>206</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>213</v>
+        <v>207</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="E9" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>206</v>
+        <v>193</v>
       </c>
       <c r="G9" s="2" t="s">
         <v>13</v>
@@ -3173,22 +3155,22 @@
     </row>
     <row r="10" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>214</v>
+        <v>208</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>215</v>
+        <v>209</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="E10" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>216</v>
+        <v>193</v>
       </c>
       <c r="G10" s="2" t="s">
         <v>13</v>
@@ -3196,22 +3178,22 @@
     </row>
     <row r="11" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>217</v>
+        <v>210</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>218</v>
+        <v>211</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="E11" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>199</v>
+        <v>193</v>
       </c>
       <c r="G11" s="2" t="s">
         <v>13</v>
@@ -3219,22 +3201,22 @@
     </row>
     <row r="12" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>219</v>
+        <v>212</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>220</v>
+        <v>213</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="E12" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>206</v>
+        <v>193</v>
       </c>
       <c r="G12" s="2" t="s">
         <v>13</v>
@@ -3242,22 +3224,22 @@
     </row>
     <row r="13" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>221</v>
+        <v>214</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>222</v>
+        <v>215</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="E13" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>206</v>
+        <v>193</v>
       </c>
       <c r="G13" s="2" t="s">
         <v>13</v>
@@ -3265,22 +3247,22 @@
     </row>
     <row r="14" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>223</v>
+        <v>216</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>224</v>
+        <v>217</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="E14" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>206</v>
+        <v>193</v>
       </c>
       <c r="G14" s="2" t="s">
         <v>13</v>
@@ -3288,22 +3270,22 @@
     </row>
     <row r="15" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>225</v>
+        <v>218</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="E15" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>206</v>
+        <v>193</v>
       </c>
       <c r="G15" s="2" t="s">
         <v>13</v>
@@ -3311,22 +3293,22 @@
     </row>
     <row r="16" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>227</v>
+        <v>220</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>228</v>
+        <v>221</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="E16" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>206</v>
+        <v>193</v>
       </c>
       <c r="G16" s="2" t="s">
         <v>13</v>
@@ -3334,22 +3316,22 @@
     </row>
     <row r="17" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>229</v>
+        <v>222</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>230</v>
+        <v>223</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="E17" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>206</v>
+        <v>193</v>
       </c>
       <c r="G17" s="2" t="s">
         <v>13</v>
@@ -3357,22 +3339,22 @@
     </row>
     <row r="18" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>231</v>
+        <v>224</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>232</v>
+        <v>225</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="E18" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>206</v>
+        <v>193</v>
       </c>
       <c r="G18" s="2" t="s">
         <v>13</v>
@@ -3380,22 +3362,22 @@
     </row>
     <row r="19" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>233</v>
+        <v>226</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>234</v>
+        <v>227</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="E19" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>206</v>
+        <v>193</v>
       </c>
       <c r="G19" s="2" t="s">
         <v>13</v>
@@ -3403,22 +3385,22 @@
     </row>
     <row r="20" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>235</v>
+        <v>228</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>236</v>
+        <v>229</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="E20" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>206</v>
+        <v>193</v>
       </c>
       <c r="G20" s="2" t="s">
         <v>13</v>
@@ -3426,22 +3408,22 @@
     </row>
     <row r="21" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>237</v>
+        <v>230</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>238</v>
+        <v>231</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="E21" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>206</v>
+        <v>193</v>
       </c>
       <c r="G21" s="2" t="s">
         <v>13</v>
@@ -3492,22 +3474,22 @@
     </row>
     <row r="2" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>239</v>
+        <v>232</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>240</v>
+        <v>233</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>241</v>
+        <v>234</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>240</v>
+        <v>233</v>
       </c>
       <c r="E2" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>242</v>
+        <v>235</v>
       </c>
       <c r="G2" s="2" t="s">
         <v>13</v>
@@ -3515,22 +3497,22 @@
     </row>
     <row r="3" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>243</v>
+        <v>236</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>240</v>
+        <v>233</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>244</v>
+        <v>237</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>240</v>
+        <v>233</v>
       </c>
       <c r="E3" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>34</v>
+        <v>137</v>
       </c>
       <c r="G3" s="2" t="s">
         <v>13</v>
@@ -3538,22 +3520,22 @@
     </row>
     <row r="4" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>245</v>
+        <v>238</v>
       </c>
       <c r="B4" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>239</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F4" s="2" t="s">
         <v>240</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>246</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>240</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>247</v>
       </c>
       <c r="G4" s="2" t="s">
         <v>13</v>
@@ -3561,22 +3543,22 @@
     </row>
     <row r="5" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>248</v>
+        <v>241</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>240</v>
+        <v>233</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>249</v>
+        <v>242</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>240</v>
+        <v>233</v>
       </c>
       <c r="E5" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>206</v>
+        <v>193</v>
       </c>
       <c r="G5" s="2" t="s">
         <v>13</v>
@@ -3584,22 +3566,22 @@
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>250</v>
+        <v>243</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>240</v>
+        <v>233</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>251</v>
+        <v>244</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>240</v>
+        <v>233</v>
       </c>
       <c r="E6" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>252</v>
+        <v>245</v>
       </c>
       <c r="G6" s="2" t="s">
         <v>13</v>
@@ -3607,22 +3589,22 @@
     </row>
     <row r="7" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>253</v>
+        <v>246</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>240</v>
+        <v>233</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>254</v>
+        <v>247</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>240</v>
+        <v>233</v>
       </c>
       <c r="E7" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>255</v>
+        <v>248</v>
       </c>
       <c r="G7" s="2" t="s">
         <v>13</v>
@@ -3630,22 +3612,22 @@
     </row>
     <row r="8" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>256</v>
+        <v>249</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>240</v>
+        <v>233</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>257</v>
+        <v>250</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>240</v>
+        <v>233</v>
       </c>
       <c r="E8" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>258</v>
+        <v>251</v>
       </c>
       <c r="G8" s="2" t="s">
         <v>13</v>
@@ -3653,22 +3635,22 @@
     </row>
     <row r="9" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>259</v>
+        <v>252</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>240</v>
+        <v>233</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>260</v>
+        <v>253</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>240</v>
+        <v>233</v>
       </c>
       <c r="E9" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>261</v>
+        <v>254</v>
       </c>
       <c r="G9" s="2" t="s">
         <v>13</v>
@@ -3676,22 +3658,22 @@
     </row>
     <row r="10" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>262</v>
+        <v>255</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>240</v>
+        <v>233</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>263</v>
+        <v>256</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>264</v>
+        <v>257</v>
       </c>
       <c r="E10" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>265</v>
+        <v>258</v>
       </c>
       <c r="G10" s="2" t="s">
         <v>13</v>
@@ -3699,22 +3681,22 @@
     </row>
     <row r="11" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>266</v>
+        <v>259</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>240</v>
+        <v>233</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>267</v>
+        <v>260</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>264</v>
+        <v>257</v>
       </c>
       <c r="E11" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>206</v>
+        <v>193</v>
       </c>
       <c r="G11" s="2" t="s">
         <v>13</v>
@@ -3722,22 +3704,22 @@
     </row>
     <row r="12" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>268</v>
+        <v>261</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>240</v>
+        <v>233</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>240</v>
+        <v>233</v>
       </c>
       <c r="E12" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>270</v>
+        <v>263</v>
       </c>
       <c r="G12" s="2" t="s">
         <v>13</v>
@@ -3745,22 +3727,22 @@
     </row>
     <row r="13" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>271</v>
+        <v>264</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>240</v>
+        <v>233</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>272</v>
+        <v>265</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>240</v>
+        <v>233</v>
       </c>
       <c r="E13" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>273</v>
+        <v>266</v>
       </c>
       <c r="G13" s="2" t="s">
         <v>13</v>
@@ -3768,22 +3750,22 @@
     </row>
     <row r="14" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>274</v>
+        <v>267</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>240</v>
+        <v>233</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>275</v>
+        <v>268</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>240</v>
+        <v>233</v>
       </c>
       <c r="E14" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>199</v>
+        <v>193</v>
       </c>
       <c r="G14" s="2" t="s">
         <v>13</v>
@@ -3791,22 +3773,22 @@
     </row>
     <row r="15" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>276</v>
+        <v>269</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>240</v>
+        <v>233</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>277</v>
+        <v>270</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>240</v>
+        <v>233</v>
       </c>
       <c r="E15" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>278</v>
+        <v>271</v>
       </c>
       <c r="G15" s="2" t="s">
         <v>13</v>
@@ -3814,22 +3796,22 @@
     </row>
     <row r="16" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>279</v>
+        <v>272</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>240</v>
+        <v>233</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>280</v>
+        <v>273</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>264</v>
+        <v>257</v>
       </c>
       <c r="E16" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>281</v>
+        <v>274</v>
       </c>
       <c r="G16" s="2" t="s">
         <v>13</v>
@@ -3880,22 +3862,22 @@
     </row>
     <row r="2" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>282</v>
+        <v>275</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>283</v>
+        <v>276</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>284</v>
+        <v>277</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>285</v>
+        <v>278</v>
       </c>
       <c r="E2" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>286</v>
+        <v>279</v>
       </c>
       <c r="G2" s="2" t="s">
         <v>13</v>
@@ -3903,22 +3885,22 @@
     </row>
     <row r="3" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>287</v>
+        <v>280</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>283</v>
+        <v>276</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>288</v>
+        <v>281</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>285</v>
+        <v>278</v>
       </c>
       <c r="E3" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>289</v>
+        <v>282</v>
       </c>
       <c r="G3" s="2" t="s">
         <v>13</v>
@@ -3926,22 +3908,22 @@
     </row>
     <row r="4" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>290</v>
+        <v>283</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>283</v>
+        <v>276</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>291</v>
+        <v>284</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>283</v>
+        <v>276</v>
       </c>
       <c r="E4" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="G4" s="2" t="s">
         <v>13</v>
@@ -3949,22 +3931,22 @@
     </row>
     <row r="5" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>292</v>
+        <v>285</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>283</v>
+        <v>276</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>293</v>
+        <v>286</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>283</v>
+        <v>276</v>
       </c>
       <c r="E5" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>294</v>
+        <v>287</v>
       </c>
       <c r="G5" s="2" t="s">
         <v>13</v>
@@ -3972,22 +3954,22 @@
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>295</v>
+        <v>288</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>283</v>
+        <v>276</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>296</v>
+        <v>289</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>264</v>
+        <v>257</v>
       </c>
       <c r="E6" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>206</v>
+        <v>193</v>
       </c>
       <c r="G6" s="2" t="s">
         <v>13</v>
@@ -3995,22 +3977,22 @@
     </row>
     <row r="7" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>297</v>
+        <v>290</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>283</v>
+        <v>276</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>298</v>
+        <v>291</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>283</v>
+        <v>276</v>
       </c>
       <c r="E7" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>299</v>
+        <v>292</v>
       </c>
       <c r="G7" s="2" t="s">
         <v>13</v>
@@ -4018,22 +4000,22 @@
     </row>
     <row r="8" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>300</v>
+        <v>293</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>283</v>
+        <v>276</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>301</v>
+        <v>294</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>285</v>
+        <v>278</v>
       </c>
       <c r="E8" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>302</v>
+        <v>295</v>
       </c>
       <c r="G8" s="2" t="s">
         <v>13</v>
@@ -4041,22 +4023,22 @@
     </row>
     <row r="9" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>303</v>
+        <v>296</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>283</v>
+        <v>276</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>304</v>
+        <v>297</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>285</v>
+        <v>278</v>
       </c>
       <c r="E9" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>305</v>
+        <v>298</v>
       </c>
       <c r="G9" s="2" t="s">
         <v>13</v>
@@ -4064,22 +4046,22 @@
     </row>
     <row r="10" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>306</v>
+        <v>299</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>283</v>
+        <v>276</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>307</v>
+        <v>300</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>285</v>
+        <v>278</v>
       </c>
       <c r="E10" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>209</v>
+        <v>301</v>
       </c>
       <c r="G10" s="2" t="s">
         <v>13</v>
@@ -4087,22 +4069,22 @@
     </row>
     <row r="11" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>308</v>
+        <v>302</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>283</v>
+        <v>276</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>309</v>
+        <v>303</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>283</v>
+        <v>276</v>
       </c>
       <c r="E11" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>206</v>
+        <v>193</v>
       </c>
       <c r="G11" s="2" t="s">
         <v>13</v>

</xml_diff>

<commit_message>
Improve login page Firebase error mapping to show user-friendly message
</commit_message>
<xml_diff>
--- a/tests/reports/Test_Analysis_Report.xlsx
+++ b/tests/reports/Test_Analysis_Report.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="805" uniqueCount="304">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="805" uniqueCount="306">
   <si>
     <t>Test ID</t>
   </si>
@@ -56,7 +56,7 @@
     <t>Passed</t>
   </si>
   <si>
-    <t>2898ms</t>
+    <t>304ms</t>
   </si>
   <si>
     <t>Assertion passed successfully</t>
@@ -68,7 +68,7 @@
     <t>Verify brand name PayBuddy header exists</t>
   </si>
   <si>
-    <t>241ms</t>
+    <t>247ms</t>
   </si>
   <si>
     <t>TC-WEB-UI-003</t>
@@ -92,124 +92,127 @@
     <t>Verify Sign In button is present</t>
   </si>
   <si>
+    <t>14ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-006</t>
+  </si>
+  <si>
+    <t>Verify secure access footer notice is present</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-007</t>
+  </si>
+  <si>
+    <t>Verify branding subtitle text exists</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-008</t>
+  </si>
+  <si>
+    <t>Verify email input field placeholder</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-009</t>
+  </si>
+  <si>
+    <t>Verify password input field placeholder</t>
+  </si>
+  <si>
+    <t>13ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-010</t>
+  </si>
+  <si>
+    <t>Verify font family CSS on headers</t>
+  </si>
+  <si>
+    <t>16ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-011</t>
+  </si>
+  <si>
+    <t>Verify primary brand color on buttons</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-012</t>
+  </si>
+  <si>
+    <t>Verify centered block layout</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-013</t>
+  </si>
+  <si>
+    <t>Verify responsive structure at mobile width 360px</t>
+  </si>
+  <si>
+    <t>890ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-014</t>
+  </si>
+  <si>
+    <t>Verify responsive structure at tablet width 768px</t>
+  </si>
+  <si>
+    <t>884ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-015</t>
+  </si>
+  <si>
+    <t>Restore browser window maximization state</t>
+  </si>
+  <si>
+    <t>23ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-016</t>
+  </si>
+  <si>
+    <t>Verify HTML tag specification for email input</t>
+  </si>
+  <si>
+    <t>25ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-017</t>
+  </si>
+  <si>
+    <t>Verify HTML tag specification for password input</t>
+  </si>
+  <si>
     <t>12ms</t>
   </si>
   <si>
-    <t>TC-WEB-UI-006</t>
-  </si>
-  <si>
-    <t>Verify secure access footer notice is present</t>
-  </si>
-  <si>
-    <t>13ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UI-007</t>
-  </si>
-  <si>
-    <t>Verify branding subtitle text exists</t>
-  </si>
-  <si>
-    <t>TC-WEB-UI-008</t>
-  </si>
-  <si>
-    <t>Verify email input field placeholder</t>
-  </si>
-  <si>
-    <t>TC-WEB-UI-009</t>
-  </si>
-  <si>
-    <t>Verify password input field placeholder</t>
-  </si>
-  <si>
-    <t>14ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UI-010</t>
-  </si>
-  <si>
-    <t>Verify font family CSS on headers</t>
+    <t>TC-WEB-UI-018</t>
+  </si>
+  <si>
+    <t>Verify card wrapper styles (border-radius)</t>
+  </si>
+  <si>
+    <t>37ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-019</t>
+  </si>
+  <si>
+    <t>Verify background styling matches design spec</t>
   </si>
   <si>
     <t>17ms</t>
   </si>
   <si>
-    <t>TC-WEB-UI-011</t>
-  </si>
-  <si>
-    <t>Verify primary brand color on buttons</t>
-  </si>
-  <si>
-    <t>TC-WEB-UI-012</t>
-  </si>
-  <si>
-    <t>Verify centered block layout</t>
-  </si>
-  <si>
-    <t>16ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UI-013</t>
-  </si>
-  <si>
-    <t>Verify responsive structure at mobile width 360px</t>
-  </si>
-  <si>
-    <t>908ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UI-014</t>
-  </si>
-  <si>
-    <t>Verify responsive structure at tablet width 768px</t>
-  </si>
-  <si>
-    <t>904ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UI-015</t>
-  </si>
-  <si>
-    <t>Restore browser window maximization state</t>
-  </si>
-  <si>
-    <t>34ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UI-016</t>
-  </si>
-  <si>
-    <t>Verify HTML tag specification for email input</t>
-  </si>
-  <si>
-    <t>TC-WEB-UI-017</t>
-  </si>
-  <si>
-    <t>Verify HTML tag specification for password input</t>
-  </si>
-  <si>
-    <t>TC-WEB-UI-018</t>
-  </si>
-  <si>
-    <t>Verify card wrapper styles (border-radius)</t>
-  </si>
-  <si>
-    <t>20ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UI-019</t>
-  </si>
-  <si>
-    <t>Verify background styling matches design spec</t>
-  </si>
-  <si>
     <t>TC-WEB-UI-020</t>
   </si>
   <si>
     <t>Verify focus state click handler does not crash</t>
   </si>
   <si>
-    <t>90ms</t>
+    <t>131ms</t>
   </si>
   <si>
     <t>TC-WEB-UI-021</t>
@@ -218,25 +221,25 @@
     <t>Verify top-level container viewport classes</t>
   </si>
   <si>
+    <t>29ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-022</t>
+  </si>
+  <si>
+    <t>Verify branding and form division layout margins</t>
+  </si>
+  <si>
     <t>24ms</t>
   </si>
   <si>
-    <t>TC-WEB-UI-022</t>
-  </si>
-  <si>
-    <t>Verify branding and form division layout margins</t>
-  </si>
-  <si>
-    <t>42ms</t>
-  </si>
-  <si>
     <t>TC-WEB-UI-023</t>
   </si>
   <si>
     <t>Verify clear textual contrast for reader accessibility</t>
   </si>
   <si>
-    <t>25ms</t>
+    <t>35ms</t>
   </si>
   <si>
     <t>TC-WEB-UI-024</t>
@@ -245,175 +248,190 @@
     <t>Verify page scales properly without layout clipping</t>
   </si>
   <si>
-    <t>23ms</t>
-  </si>
-  <si>
     <t>TC-WEB-UI-025</t>
   </si>
   <si>
     <t>Verify smooth interactive transitions on button inputs</t>
   </si>
   <si>
+    <t>TC-WEB-FUNC-001</t>
+  </si>
+  <si>
+    <t>Functional</t>
+  </si>
+  <si>
+    <t>Verify invalid login rejection message</t>
+  </si>
+  <si>
+    <t>1153ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-002</t>
+  </si>
+  <si>
+    <t>Verify rejection of nonexistent email</t>
+  </si>
+  <si>
+    <t>839ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-003</t>
+  </si>
+  <si>
+    <t>Verify successful login with valid credentials redirects to Dashboard</t>
+  </si>
+  <si>
+    <t>1702ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-004</t>
+  </si>
+  <si>
+    <t>Verify dashboard displays Total Customers count</t>
+  </si>
+  <si>
+    <t>496ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-005</t>
+  </si>
+  <si>
+    <t>Verify dashboard displays Active Sales count</t>
+  </si>
+  <si>
+    <t>43ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-006</t>
+  </si>
+  <si>
+    <t>Verify dashboard displays Pending Installments count</t>
+  </si>
+  <si>
+    <t>45ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-007</t>
+  </si>
+  <si>
+    <t>Verify dashboard displays Today's Due count</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-008</t>
+  </si>
+  <si>
+    <t>Verify dashboard displays Outstanding Balance amount</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-009</t>
+  </si>
+  <si>
+    <t>Navigate to customers page and verify header</t>
+  </si>
+  <si>
+    <t>163ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-010</t>
+  </si>
+  <si>
+    <t>Verify add new customer input inputs are present</t>
+  </si>
+  <si>
+    <t>33ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-011</t>
+  </si>
+  <si>
+    <t>Verify customer creation and entry addition to table</t>
+  </si>
+  <si>
+    <t>2539ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-012</t>
+  </si>
+  <si>
+    <t>Verify presence of seeded customer</t>
+  </si>
+  <si>
+    <t>21ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-013</t>
+  </si>
+  <si>
+    <t>Navigate to specific customer profile page</t>
+  </si>
+  <si>
+    <t>1131ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-014</t>
+  </si>
+  <si>
+    <t>Verify phone number exists on profile detail bar</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-015</t>
+  </si>
+  <si>
+    <t>Verify Total Amount financial card is 1000 INR</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-016</t>
+  </si>
+  <si>
+    <t>Verify Paid Amount financial card is 0 INR</t>
+  </si>
+  <si>
+    <t>86ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-017</t>
+  </si>
+  <si>
+    <t>Verify Outstanding Balance financial card is 1000 INR</t>
+  </si>
+  <si>
+    <t>28ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-018</t>
+  </si>
+  <si>
+    <t>Verify E2E Test Item pending sale is loaded in sales list</t>
+  </si>
+  <si>
+    <t>18ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-019</t>
+  </si>
+  <si>
+    <t>Verify redirect to record payment page</t>
+  </si>
+  <si>
+    <t>761ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-020</t>
+  </si>
+  <si>
+    <t>Verify remaining balance display match before payment</t>
+  </si>
+  <si>
     <t>19ms</t>
   </si>
   <si>
-    <t>TC-WEB-FUNC-001</t>
-  </si>
-  <si>
-    <t>Functional</t>
-  </si>
-  <si>
-    <t>Verify invalid login rejection message</t>
-  </si>
-  <si>
-    <t>2371ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-002</t>
-  </si>
-  <si>
-    <t>Verify rejection of nonexistent email</t>
-  </si>
-  <si>
-    <t>784ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-003</t>
-  </si>
-  <si>
-    <t>Verify successful login with valid credentials redirects to Dashboard</t>
-  </si>
-  <si>
-    <t>1610ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-004</t>
-  </si>
-  <si>
-    <t>Verify dashboard displays Total Customers count</t>
-  </si>
-  <si>
-    <t>247ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-005</t>
-  </si>
-  <si>
-    <t>Verify dashboard displays Active Sales count</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-006</t>
-  </si>
-  <si>
-    <t>Verify dashboard displays Pending Installments count</t>
-  </si>
-  <si>
-    <t>18ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-007</t>
-  </si>
-  <si>
-    <t>Verify dashboard displays Today's Due count</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-008</t>
-  </si>
-  <si>
-    <t>Verify dashboard displays Outstanding Balance amount</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-009</t>
-  </si>
-  <si>
-    <t>Navigate to customers page and verify header</t>
-  </si>
-  <si>
-    <t>129ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-010</t>
-  </si>
-  <si>
-    <t>Verify add new customer input inputs are present</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-011</t>
-  </si>
-  <si>
-    <t>Verify customer creation and entry addition to table</t>
-  </si>
-  <si>
-    <t>2346ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-012</t>
-  </si>
-  <si>
-    <t>Verify presence of seeded customer</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-013</t>
-  </si>
-  <si>
-    <t>Navigate to specific customer profile page</t>
-  </si>
-  <si>
-    <t>989ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-014</t>
-  </si>
-  <si>
-    <t>Verify phone number exists on profile detail bar</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-015</t>
-  </si>
-  <si>
-    <t>Verify Total Amount financial card is 1000 INR</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-016</t>
-  </si>
-  <si>
-    <t>Verify Paid Amount financial card is 0 INR</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-017</t>
-  </si>
-  <si>
-    <t>Verify Outstanding Balance financial card is 1000 INR</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-018</t>
-  </si>
-  <si>
-    <t>Verify E2E Test Item pending sale is loaded in sales list</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-019</t>
-  </si>
-  <si>
-    <t>Verify redirect to record payment page</t>
-  </si>
-  <si>
-    <t>790ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-020</t>
-  </si>
-  <si>
-    <t>Verify remaining balance display match before payment</t>
-  </si>
-  <si>
     <t>TC-WEB-FUNC-021</t>
   </si>
   <si>
     <t>Record payment E2E execution and redirection validation</t>
   </si>
   <si>
-    <t>2821ms</t>
+    <t>3226ms</t>
   </si>
   <si>
     <t>TC-WEB-FUNC-022</t>
@@ -422,7 +440,7 @@
     <t>Verify Outstanding Balance updates to 800 INR in customer card</t>
   </si>
   <si>
-    <t>1140ms</t>
+    <t>1192ms</t>
   </si>
   <si>
     <t>TC-WEB-FUNC-023</t>
@@ -431,9 +449,6 @@
     <t>Verify Paid Amount updates to 200 INR in customer card</t>
   </si>
   <si>
-    <t>11ms</t>
-  </si>
-  <si>
     <t>TC-WEB-FUNC-024</t>
   </si>
   <si>
@@ -446,7 +461,7 @@
     <t>Verify sales management index loads properly</t>
   </si>
   <si>
-    <t>552ms</t>
+    <t>866ms</t>
   </si>
   <si>
     <t>TC-WEB-FUNC-026</t>
@@ -455,7 +470,7 @@
     <t>Verify sales search filter works properly</t>
   </si>
   <si>
-    <t>626ms</t>
+    <t>728ms</t>
   </si>
   <si>
     <t>TC-WEB-FUNC-027</t>
@@ -464,7 +479,7 @@
     <t>Navigate to Create New Sale form</t>
   </si>
   <si>
-    <t>840ms</t>
+    <t>801ms</t>
   </si>
   <si>
     <t>TC-WEB-FUNC-028</t>
@@ -473,7 +488,7 @@
     <t>Verify total amount computed automatically (2 x 500 = 1000)</t>
   </si>
   <si>
-    <t>231ms</t>
+    <t>307ms</t>
   </si>
   <si>
     <t>TC-WEB-FUNC-029</t>
@@ -482,7 +497,7 @@
     <t>Create sale and verify redirect back to sales table</t>
   </si>
   <si>
-    <t>204ms</t>
+    <t>207ms</t>
   </si>
   <si>
     <t>TC-WEB-FUNC-030</t>
@@ -491,7 +506,7 @@
     <t>Verify Payments page path and title</t>
   </si>
   <si>
-    <t>574ms</t>
+    <t>591ms</t>
   </si>
   <si>
     <t>TC-WEB-FUNC-031</t>
@@ -500,7 +515,7 @@
     <t>Verify E2E transaction exists in master list</t>
   </si>
   <si>
-    <t>33ms</t>
+    <t>85ms</t>
   </si>
   <si>
     <t>TC-WEB-FUNC-032</t>
@@ -509,7 +524,7 @@
     <t>Verify Ledger Book page loads</t>
   </si>
   <si>
-    <t>827ms</t>
+    <t>799ms</t>
   </si>
   <si>
     <t>TC-WEB-FUNC-033</t>
@@ -518,7 +533,7 @@
     <t>Verify ledger records contain client name</t>
   </si>
   <si>
-    <t>31ms</t>
+    <t>121ms</t>
   </si>
   <si>
     <t>TC-WEB-FUNC-034</t>
@@ -527,7 +542,7 @@
     <t>Verify Installments page title</t>
   </si>
   <si>
-    <t>562ms</t>
+    <t>568ms</t>
   </si>
   <si>
     <t>TC-WEB-FUNC-035</t>
@@ -536,13 +551,16 @@
     <t>Verify customer details exist on installment board</t>
   </si>
   <si>
+    <t>53ms</t>
+  </si>
+  <si>
     <t>TC-WEB-FUNC-036</t>
   </si>
   <si>
     <t>Verify direct Dashboard URL redirect</t>
   </si>
   <si>
-    <t>99ms</t>
+    <t>106ms</t>
   </si>
   <si>
     <t>TC-WEB-FUNC-037</t>
@@ -551,7 +569,7 @@
     <t>Verify customer data updates dynamically on UI edit</t>
   </si>
   <si>
-    <t>4236ms</t>
+    <t>4447ms</t>
   </si>
   <si>
     <t>TC-WEB-FUNC-038</t>
@@ -560,7 +578,7 @@
     <t>Verify logout route terminates session and redirects to sign in</t>
   </si>
   <si>
-    <t>608ms</t>
+    <t>1050ms</t>
   </si>
   <si>
     <t>TC-WEB-FUNC-039</t>
@@ -569,7 +587,7 @@
     <t>Verify unauthorized dashboard access redirects to login</t>
   </si>
   <si>
-    <t>2158ms</t>
+    <t>2104ms</t>
   </si>
   <si>
     <t>TC-WEB-FUNC-040</t>
@@ -578,7 +596,7 @@
     <t>Verify unauthorized customer details access redirects to login</t>
   </si>
   <si>
-    <t>2808ms</t>
+    <t>2103ms</t>
   </si>
   <si>
     <t>TC-WEB-UNIT-001</t>
@@ -590,340 +608,328 @@
     <t>Test formatCurrency formatting positive amount</t>
   </si>
   <si>
+    <t>TC-WEB-UNIT-002</t>
+  </si>
+  <si>
+    <t>Test formatCurrency formatting zero amount</t>
+  </si>
+  <si>
+    <t>0ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UNIT-003</t>
+  </si>
+  <si>
+    <t>Test formatCurrency formatting negative amount</t>
+  </si>
+  <si>
+    <t>TC-WEB-UNIT-004</t>
+  </si>
+  <si>
+    <t>Test formatCurrency formatting large millions scale amount</t>
+  </si>
+  <si>
+    <t>TC-WEB-UNIT-005</t>
+  </si>
+  <si>
+    <t>Test formatCurrency decimal rounding functionality</t>
+  </si>
+  <si>
+    <t>TC-WEB-UNIT-006</t>
+  </si>
+  <si>
+    <t>Test formatDate string matching date details</t>
+  </si>
+  <si>
+    <t>TC-WEB-UNIT-007</t>
+  </si>
+  <si>
+    <t>Test formatDate fallback for null values</t>
+  </si>
+  <si>
+    <t>TC-WEB-UNIT-008</t>
+  </si>
+  <si>
+    <t>Test formatDate fallback for 0 value</t>
+  </si>
+  <si>
+    <t>TC-WEB-UNIT-009</t>
+  </si>
+  <si>
+    <t>Test formatDateTime details formatting</t>
+  </si>
+  <si>
+    <t>1ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UNIT-010</t>
+  </si>
+  <si>
+    <t>Test formatDateTime null timestamp handling</t>
+  </si>
+  <si>
+    <t>TC-WEB-UNIT-011</t>
+  </si>
+  <si>
+    <t>Verify email validation for valid string</t>
+  </si>
+  <si>
+    <t>TC-WEB-UNIT-012</t>
+  </si>
+  <si>
+    <t>Verify email validation blocks missing TLD</t>
+  </si>
+  <si>
+    <t>TC-WEB-UNIT-013</t>
+  </si>
+  <si>
+    <t>Verify email validation blocks missing alias prefix</t>
+  </si>
+  <si>
+    <t>TC-WEB-UNIT-014</t>
+  </si>
+  <si>
+    <t>Verify phone validation for standard 10 digit number</t>
+  </si>
+  <si>
+    <t>TC-WEB-UNIT-015</t>
+  </si>
+  <si>
+    <t>Verify phone validation blocks short length</t>
+  </si>
+  <si>
+    <t>TC-WEB-UNIT-016</t>
+  </si>
+  <si>
+    <t>Verify phone validation blocks alphabetic characters</t>
+  </si>
+  <si>
+    <t>TC-WEB-UNIT-017</t>
+  </si>
+  <si>
+    <t>Verify interest formula multiplication logic</t>
+  </si>
+  <si>
+    <t>TC-WEB-UNIT-018</t>
+  </si>
+  <si>
+    <t>Verify installment partitioning amount division</t>
+  </si>
+  <si>
+    <t>TC-WEB-UNIT-019</t>
+  </si>
+  <si>
+    <t>Verify remaining balance arithmetic subtraction</t>
+  </si>
+  <si>
+    <t>TC-WEB-UNIT-020</t>
+  </si>
+  <si>
+    <t>Verify mock environment manifest validator passes</t>
+  </si>
+  <si>
+    <t>TC-WEB-VAL-001</t>
+  </si>
+  <si>
+    <t>Validation</t>
+  </si>
+  <si>
+    <t>Verify email required constraint is enabled on form</t>
+  </si>
+  <si>
+    <t>329ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-VAL-002</t>
+  </si>
+  <si>
+    <t>Verify password required constraint is enabled on form</t>
+  </si>
+  <si>
+    <t>TC-WEB-VAL-003</t>
+  </si>
+  <si>
+    <t>Verify browser client blocks submissions for invalid email inputs</t>
+  </si>
+  <si>
+    <t>107ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-VAL-004</t>
+  </si>
+  <si>
+    <t>Verify character bounds for data buffers limit to 255 characters</t>
+  </si>
+  <si>
+    <t>TC-WEB-VAL-005</t>
+  </si>
+  <si>
+    <t>Verify customer creation form prevents empty submit</t>
+  </si>
+  <si>
+    <t>3059ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-VAL-006</t>
+  </si>
+  <si>
+    <t>Verify phone input uses tel semantic element type</t>
+  </si>
+  <si>
+    <t>26ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-VAL-007</t>
+  </si>
+  <si>
+    <t>Verify sale quantity requires positive minimum value (&gt; 0)</t>
+  </si>
+  <si>
+    <t>563ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-VAL-008</t>
+  </si>
+  <si>
+    <t>Verify unit price input restricts negative numbers</t>
+  </si>
+  <si>
+    <t>TC-WEB-VAL-009</t>
+  </si>
+  <si>
+    <t>Verify script tag input text does not trigger native alerts</t>
+  </si>
+  <si>
+    <t>Security</t>
+  </si>
+  <si>
+    <t>2311ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-VAL-010</t>
+  </si>
+  <si>
+    <t>Verify database adapter parameters parameterized input query parsing</t>
+  </si>
+  <si>
+    <t>TC-WEB-VAL-011</t>
+  </si>
+  <si>
+    <t>Verify error prevents overpayment collections</t>
+  </si>
+  <si>
+    <t>2120ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-VAL-012</t>
+  </si>
+  <si>
+    <t>Verify collection input restricts 0 value submissions</t>
+  </si>
+  <si>
+    <t>1143ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-VAL-013</t>
+  </si>
+  <si>
+    <t>Verify Firestore writes match schema constraints</t>
+  </si>
+  <si>
+    <t>TC-WEB-VAL-014</t>
+  </si>
+  <si>
+    <t>Verify wildcard URLs redirect to main route base</t>
+  </si>
+  <si>
+    <t>2118ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-VAL-015</t>
+  </si>
+  <si>
+    <t>Verify HTML password hidden mask attribute config</t>
+  </si>
+  <si>
+    <t>668ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-DEP-001</t>
+  </si>
+  <si>
+    <t>Deployment</t>
+  </si>
+  <si>
+    <t>Verify load paint FCP under 2.5s threshold</t>
+  </si>
+  <si>
+    <t>Performance</t>
+  </si>
+  <si>
+    <t>124ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-DEP-002</t>
+  </si>
+  <si>
+    <t>Verify full render transition load time under limit</t>
+  </si>
+  <si>
+    <t>1185ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-DEP-003</t>
+  </si>
+  <si>
+    <t>Verify DNS host domain matches Vercel production edge</t>
+  </si>
+  <si>
+    <t>TC-WEB-DEP-004</t>
+  </si>
+  <si>
+    <t>Verify favicon.ico endpoint yields clean HTTP status</t>
+  </si>
+  <si>
+    <t>103ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-DEP-005</t>
+  </si>
+  <si>
+    <t>Verify production connection protocol HTTPS encryption is active</t>
+  </si>
+  <si>
+    <t>TC-WEB-DEP-006</t>
+  </si>
+  <si>
+    <t>Verify head links contain manifest registration details</t>
+  </si>
+  <si>
+    <t>147ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-DEP-007</t>
+  </si>
+  <si>
+    <t>Verify console logs have no severe exceptions during login page session</t>
+  </si>
+  <si>
+    <t>3ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-DEP-008</t>
+  </si>
+  <si>
+    <t>Verify standard responsive layouts align horizontally</t>
+  </si>
+  <si>
     <t>56ms</t>
   </si>
   <si>
-    <t>TC-WEB-UNIT-002</t>
-  </si>
-  <si>
-    <t>Test formatCurrency formatting zero amount</t>
-  </si>
-  <si>
-    <t>0ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UNIT-003</t>
-  </si>
-  <si>
-    <t>Test formatCurrency formatting negative amount</t>
-  </si>
-  <si>
-    <t>TC-WEB-UNIT-004</t>
-  </si>
-  <si>
-    <t>Test formatCurrency formatting large millions scale amount</t>
-  </si>
-  <si>
-    <t>1ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UNIT-005</t>
-  </si>
-  <si>
-    <t>Test formatCurrency decimal rounding functionality</t>
-  </si>
-  <si>
-    <t>TC-WEB-UNIT-006</t>
-  </si>
-  <si>
-    <t>Test formatDate string matching date details</t>
-  </si>
-  <si>
-    <t>9ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UNIT-007</t>
-  </si>
-  <si>
-    <t>Test formatDate fallback for null values</t>
-  </si>
-  <si>
-    <t>TC-WEB-UNIT-008</t>
-  </si>
-  <si>
-    <t>Test formatDate fallback for 0 value</t>
-  </si>
-  <si>
-    <t>TC-WEB-UNIT-009</t>
-  </si>
-  <si>
-    <t>Test formatDateTime details formatting</t>
-  </si>
-  <si>
-    <t>TC-WEB-UNIT-010</t>
-  </si>
-  <si>
-    <t>Test formatDateTime null timestamp handling</t>
-  </si>
-  <si>
-    <t>TC-WEB-UNIT-011</t>
-  </si>
-  <si>
-    <t>Verify email validation for valid string</t>
-  </si>
-  <si>
-    <t>TC-WEB-UNIT-012</t>
-  </si>
-  <si>
-    <t>Verify email validation blocks missing TLD</t>
-  </si>
-  <si>
-    <t>TC-WEB-UNIT-013</t>
-  </si>
-  <si>
-    <t>Verify email validation blocks missing alias prefix</t>
-  </si>
-  <si>
-    <t>TC-WEB-UNIT-014</t>
-  </si>
-  <si>
-    <t>Verify phone validation for standard 10 digit number</t>
-  </si>
-  <si>
-    <t>TC-WEB-UNIT-015</t>
-  </si>
-  <si>
-    <t>Verify phone validation blocks short length</t>
-  </si>
-  <si>
-    <t>TC-WEB-UNIT-016</t>
-  </si>
-  <si>
-    <t>Verify phone validation blocks alphabetic characters</t>
-  </si>
-  <si>
-    <t>TC-WEB-UNIT-017</t>
-  </si>
-  <si>
-    <t>Verify interest formula multiplication logic</t>
-  </si>
-  <si>
-    <t>TC-WEB-UNIT-018</t>
-  </si>
-  <si>
-    <t>Verify installment partitioning amount division</t>
-  </si>
-  <si>
-    <t>TC-WEB-UNIT-019</t>
-  </si>
-  <si>
-    <t>Verify remaining balance arithmetic subtraction</t>
-  </si>
-  <si>
-    <t>TC-WEB-UNIT-020</t>
-  </si>
-  <si>
-    <t>Verify mock environment manifest validator passes</t>
-  </si>
-  <si>
-    <t>TC-WEB-VAL-001</t>
-  </si>
-  <si>
-    <t>Validation</t>
-  </si>
-  <si>
-    <t>Verify email required constraint is enabled on form</t>
-  </si>
-  <si>
-    <t>330ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-VAL-002</t>
-  </si>
-  <si>
-    <t>Verify password required constraint is enabled on form</t>
-  </si>
-  <si>
-    <t>TC-WEB-VAL-003</t>
-  </si>
-  <si>
-    <t>Verify browser client blocks submissions for invalid email inputs</t>
-  </si>
-  <si>
-    <t>76ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-VAL-004</t>
-  </si>
-  <si>
-    <t>Verify character bounds for data buffers limit to 255 characters</t>
-  </si>
-  <si>
-    <t>TC-WEB-VAL-005</t>
-  </si>
-  <si>
-    <t>Verify customer creation form prevents empty submit</t>
-  </si>
-  <si>
-    <t>3054ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-VAL-006</t>
-  </si>
-  <si>
-    <t>Verify phone input uses tel semantic element type</t>
-  </si>
-  <si>
-    <t>22ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-VAL-007</t>
-  </si>
-  <si>
-    <t>Verify sale quantity requires positive minimum value (&gt; 0)</t>
-  </si>
-  <si>
-    <t>600ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-VAL-008</t>
-  </si>
-  <si>
-    <t>Verify unit price input restricts negative numbers</t>
-  </si>
-  <si>
-    <t>10ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-VAL-009</t>
-  </si>
-  <si>
-    <t>Verify script tag input text does not trigger native alerts</t>
-  </si>
-  <si>
-    <t>Security</t>
-  </si>
-  <si>
-    <t>1904ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-VAL-010</t>
-  </si>
-  <si>
-    <t>Verify database adapter parameters parameterized input query parsing</t>
-  </si>
-  <si>
-    <t>TC-WEB-VAL-011</t>
-  </si>
-  <si>
-    <t>Verify error prevents overpayment collections</t>
-  </si>
-  <si>
-    <t>1909ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-VAL-012</t>
-  </si>
-  <si>
-    <t>Verify collection input restricts 0 value submissions</t>
-  </si>
-  <si>
-    <t>1123ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-VAL-013</t>
-  </si>
-  <si>
-    <t>Verify Firestore writes match schema constraints</t>
-  </si>
-  <si>
-    <t>TC-WEB-VAL-014</t>
-  </si>
-  <si>
-    <t>Verify wildcard URLs redirect to main route base</t>
-  </si>
-  <si>
-    <t>2113ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-VAL-015</t>
-  </si>
-  <si>
-    <t>Verify HTML password hidden mask attribute config</t>
-  </si>
-  <si>
-    <t>602ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-DEP-001</t>
-  </si>
-  <si>
-    <t>Deployment</t>
-  </si>
-  <si>
-    <t>Verify load paint FCP under 2.5s threshold</t>
-  </si>
-  <si>
-    <t>Performance</t>
-  </si>
-  <si>
-    <t>107ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-DEP-002</t>
-  </si>
-  <si>
-    <t>Verify full render transition load time under limit</t>
-  </si>
-  <si>
-    <t>1149ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-DEP-003</t>
-  </si>
-  <si>
-    <t>Verify DNS host domain matches Vercel production edge</t>
-  </si>
-  <si>
-    <t>TC-WEB-DEP-004</t>
-  </si>
-  <si>
-    <t>Verify favicon.ico endpoint yields clean HTTP status</t>
-  </si>
-  <si>
-    <t>94ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-DEP-005</t>
-  </si>
-  <si>
-    <t>Verify production connection protocol HTTPS encryption is active</t>
-  </si>
-  <si>
-    <t>TC-WEB-DEP-006</t>
-  </si>
-  <si>
-    <t>Verify head links contain manifest registration details</t>
-  </si>
-  <si>
-    <t>130ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-DEP-007</t>
-  </si>
-  <si>
-    <t>Verify console logs have no severe exceptions during login page session</t>
-  </si>
-  <si>
-    <t>4ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-DEP-008</t>
-  </si>
-  <si>
-    <t>Verify standard responsive layouts align horizontally</t>
-  </si>
-  <si>
-    <t>45ms</t>
-  </si>
-  <si>
     <t>TC-WEB-DEP-009</t>
   </si>
   <si>
     <t>Verify DOM count index scales cleanly</t>
-  </si>
-  <si>
-    <t>5ms</t>
   </si>
   <si>
     <t>TC-WEB-DEP-010</t>
@@ -1520,7 +1526,7 @@
         <v>11</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="G7" s="2" t="s">
         <v>13</v>
@@ -1528,13 +1534,13 @@
     </row>
     <row r="8" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>10</v>
@@ -1543,7 +1549,7 @@
         <v>11</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="G8" s="2" t="s">
         <v>13</v>
@@ -1551,13 +1557,13 @@
     </row>
     <row r="9" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>10</v>
@@ -1566,7 +1572,7 @@
         <v>11</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="G9" s="2" t="s">
         <v>13</v>
@@ -1574,13 +1580,13 @@
     </row>
     <row r="10" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D10" s="2" t="s">
         <v>10</v>
@@ -1589,7 +1595,7 @@
         <v>11</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="G10" s="2" t="s">
         <v>13</v>
@@ -1597,13 +1603,13 @@
     </row>
     <row r="11" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B11" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D11" s="2" t="s">
         <v>10</v>
@@ -1612,7 +1618,7 @@
         <v>11</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="G11" s="2" t="s">
         <v>13</v>
@@ -1620,13 +1626,13 @@
     </row>
     <row r="12" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B12" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D12" s="2" t="s">
         <v>10</v>
@@ -1635,7 +1641,7 @@
         <v>11</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="G12" s="2" t="s">
         <v>13</v>
@@ -1643,13 +1649,13 @@
     </row>
     <row r="13" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B13" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D13" s="2" t="s">
         <v>10</v>
@@ -1658,7 +1664,7 @@
         <v>11</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>42</v>
+        <v>19</v>
       </c>
       <c r="G13" s="2" t="s">
         <v>13</v>
@@ -1666,13 +1672,13 @@
     </row>
     <row r="14" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B14" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="D14" s="2" t="s">
         <v>10</v>
@@ -1681,7 +1687,7 @@
         <v>11</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="G14" s="2" t="s">
         <v>13</v>
@@ -1689,13 +1695,13 @@
     </row>
     <row r="15" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B15" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="D15" s="2" t="s">
         <v>10</v>
@@ -1704,7 +1710,7 @@
         <v>11</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="G15" s="2" t="s">
         <v>13</v>
@@ -1712,13 +1718,13 @@
     </row>
     <row r="16" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B16" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="D16" s="2" t="s">
         <v>10</v>
@@ -1727,7 +1733,7 @@
         <v>11</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="G16" s="2" t="s">
         <v>13</v>
@@ -1735,13 +1741,13 @@
     </row>
     <row r="17" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B17" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="D17" s="2" t="s">
         <v>10</v>
@@ -1750,7 +1756,7 @@
         <v>11</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>37</v>
+        <v>52</v>
       </c>
       <c r="G17" s="2" t="s">
         <v>13</v>
@@ -1758,13 +1764,13 @@
     </row>
     <row r="18" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B18" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D18" s="2" t="s">
         <v>10</v>
@@ -1773,7 +1779,7 @@
         <v>11</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>27</v>
+        <v>55</v>
       </c>
       <c r="G18" s="2" t="s">
         <v>13</v>
@@ -1819,7 +1825,7 @@
         <v>11</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="G20" s="2" t="s">
         <v>13</v>
@@ -1827,13 +1833,13 @@
     </row>
     <row r="21" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B21" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D21" s="2" t="s">
         <v>10</v>
@@ -1842,7 +1848,7 @@
         <v>11</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="G21" s="2" t="s">
         <v>13</v>
@@ -1850,13 +1856,13 @@
     </row>
     <row r="22" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B22" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D22" s="2" t="s">
         <v>10</v>
@@ -1865,7 +1871,7 @@
         <v>11</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="G22" s="2" t="s">
         <v>13</v>
@@ -1873,13 +1879,13 @@
     </row>
     <row r="23" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B23" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D23" s="2" t="s">
         <v>10</v>
@@ -1888,7 +1894,7 @@
         <v>11</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="G23" s="2" t="s">
         <v>13</v>
@@ -1896,13 +1902,13 @@
     </row>
     <row r="24" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B24" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D24" s="2" t="s">
         <v>10</v>
@@ -1911,7 +1917,7 @@
         <v>11</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="G24" s="2" t="s">
         <v>13</v>
@@ -1919,13 +1925,13 @@
     </row>
     <row r="25" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B25" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="D25" s="2" t="s">
         <v>10</v>
@@ -1934,7 +1940,7 @@
         <v>11</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>75</v>
+        <v>36</v>
       </c>
       <c r="G25" s="2" t="s">
         <v>13</v>
@@ -1957,7 +1963,7 @@
         <v>11</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>78</v>
+        <v>61</v>
       </c>
       <c r="G26" s="2" t="s">
         <v>13</v>
@@ -2008,22 +2014,22 @@
     </row>
     <row r="2" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B2" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>81</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>82</v>
       </c>
       <c r="G2" s="2" t="s">
         <v>13</v>
@@ -2031,22 +2037,22 @@
     </row>
     <row r="3" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="B3" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="C3" s="2" t="s">
+      <c r="D3" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F3" s="2" t="s">
         <v>84</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>85</v>
       </c>
       <c r="G3" s="2" t="s">
         <v>13</v>
@@ -2054,22 +2060,22 @@
     </row>
     <row r="4" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="B4" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="C4" s="2" t="s">
+      <c r="D4" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F4" s="2" t="s">
         <v>87</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>88</v>
       </c>
       <c r="G4" s="2" t="s">
         <v>13</v>
@@ -2077,22 +2083,22 @@
     </row>
     <row r="5" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="C5" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="B5" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="C5" s="2" t="s">
+      <c r="D5" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F5" s="2" t="s">
         <v>90</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F5" s="2" t="s">
-        <v>91</v>
       </c>
       <c r="G5" s="2" t="s">
         <v>13</v>
@@ -2100,22 +2106,22 @@
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="C6" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="B6" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="C6" s="2" t="s">
+      <c r="D6" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F6" s="2" t="s">
         <v>93</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>78</v>
       </c>
       <c r="G6" s="2" t="s">
         <v>13</v>
@@ -2126,13 +2132,13 @@
         <v>94</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>95</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E7" s="3" t="s">
         <v>11</v>
@@ -2149,19 +2155,19 @@
         <v>97</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>98</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E8" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>96</v>
+        <v>52</v>
       </c>
       <c r="G8" s="2" t="s">
         <v>13</v>
@@ -2172,19 +2178,19 @@
         <v>99</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>100</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E9" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>42</v>
+        <v>52</v>
       </c>
       <c r="G9" s="2" t="s">
         <v>13</v>
@@ -2195,13 +2201,13 @@
         <v>101</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>102</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E10" s="3" t="s">
         <v>11</v>
@@ -2218,19 +2224,19 @@
         <v>104</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C11" s="2" t="s">
         <v>105</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E11" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>66</v>
+        <v>106</v>
       </c>
       <c r="G11" s="2" t="s">
         <v>13</v>
@@ -2238,22 +2244,22 @@
     </row>
     <row r="12" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E12" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="G12" s="2" t="s">
         <v>13</v>
@@ -2261,22 +2267,22 @@
     </row>
     <row r="13" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E13" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>27</v>
+        <v>112</v>
       </c>
       <c r="G13" s="2" t="s">
         <v>13</v>
@@ -2284,22 +2290,22 @@
     </row>
     <row r="14" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E14" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="G14" s="2" t="s">
         <v>13</v>
@@ -2307,22 +2313,22 @@
     </row>
     <row r="15" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E15" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="G15" s="2" t="s">
         <v>13</v>
@@ -2330,16 +2336,16 @@
     </row>
     <row r="16" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E16" s="3" t="s">
         <v>11</v>
@@ -2353,22 +2359,22 @@
     </row>
     <row r="17" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E17" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>58</v>
+        <v>122</v>
       </c>
       <c r="G17" s="2" t="s">
         <v>13</v>
@@ -2376,22 +2382,22 @@
     </row>
     <row r="18" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E18" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>27</v>
+        <v>125</v>
       </c>
       <c r="G18" s="2" t="s">
         <v>13</v>
@@ -2399,22 +2405,22 @@
     </row>
     <row r="19" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E19" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>34</v>
+        <v>128</v>
       </c>
       <c r="G19" s="2" t="s">
         <v>13</v>
@@ -2422,22 +2428,22 @@
     </row>
     <row r="20" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>124</v>
+        <v>129</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E20" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>126</v>
+        <v>131</v>
       </c>
       <c r="G20" s="2" t="s">
         <v>13</v>
@@ -2445,22 +2451,22 @@
     </row>
     <row r="21" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>127</v>
+        <v>132</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E21" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>24</v>
+        <v>134</v>
       </c>
       <c r="G21" s="2" t="s">
         <v>13</v>
@@ -2468,22 +2474,22 @@
     </row>
     <row r="22" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>129</v>
+        <v>135</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>130</v>
+        <v>136</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E22" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="G22" s="2" t="s">
         <v>13</v>
@@ -2491,22 +2497,22 @@
     </row>
     <row r="23" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
-        <v>132</v>
+        <v>138</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>133</v>
+        <v>139</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E23" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>134</v>
+        <v>140</v>
       </c>
       <c r="G23" s="2" t="s">
         <v>13</v>
@@ -2514,22 +2520,22 @@
     </row>
     <row r="24" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>135</v>
+        <v>141</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>136</v>
+        <v>142</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E24" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>137</v>
+        <v>55</v>
       </c>
       <c r="G24" s="2" t="s">
         <v>13</v>
@@ -2537,22 +2543,22 @@
     </row>
     <row r="25" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E25" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="G25" s="2" t="s">
         <v>13</v>
@@ -2560,22 +2566,22 @@
     </row>
     <row r="26" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E26" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="G26" s="2" t="s">
         <v>13</v>
@@ -2583,22 +2589,22 @@
     </row>
     <row r="27" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E27" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>145</v>
+        <v>150</v>
       </c>
       <c r="G27" s="2" t="s">
         <v>13</v>
@@ -2606,22 +2612,22 @@
     </row>
     <row r="28" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
-        <v>146</v>
+        <v>151</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E28" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F28" s="2" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="G28" s="2" t="s">
         <v>13</v>
@@ -2629,22 +2635,22 @@
     </row>
     <row r="29" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
-        <v>149</v>
+        <v>154</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E29" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F29" s="2" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="G29" s="2" t="s">
         <v>13</v>
@@ -2652,22 +2658,22 @@
     </row>
     <row r="30" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
-        <v>152</v>
+        <v>157</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>153</v>
+        <v>158</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E30" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F30" s="2" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
       <c r="G30" s="2" t="s">
         <v>13</v>
@@ -2675,22 +2681,22 @@
     </row>
     <row r="31" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E31" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F31" s="2" t="s">
-        <v>157</v>
+        <v>162</v>
       </c>
       <c r="G31" s="2" t="s">
         <v>13</v>
@@ -2698,22 +2704,22 @@
     </row>
     <row r="32" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>159</v>
+        <v>164</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E32" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F32" s="2" t="s">
-        <v>160</v>
+        <v>165</v>
       </c>
       <c r="G32" s="2" t="s">
         <v>13</v>
@@ -2721,22 +2727,22 @@
     </row>
     <row r="33" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
-        <v>161</v>
+        <v>166</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E33" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F33" s="2" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="G33" s="2" t="s">
         <v>13</v>
@@ -2744,22 +2750,22 @@
     </row>
     <row r="34" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
-        <v>164</v>
+        <v>169</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>165</v>
+        <v>170</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E34" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F34" s="2" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="G34" s="2" t="s">
         <v>13</v>
@@ -2767,22 +2773,22 @@
     </row>
     <row r="35" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
-        <v>167</v>
+        <v>172</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>168</v>
+        <v>173</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E35" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F35" s="2" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
       <c r="G35" s="2" t="s">
         <v>13</v>
@@ -2790,22 +2796,22 @@
     </row>
     <row r="36" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E36" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F36" s="2" t="s">
-        <v>34</v>
+        <v>177</v>
       </c>
       <c r="G36" s="2" t="s">
         <v>13</v>
@@ -2813,22 +2819,22 @@
     </row>
     <row r="37" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
-        <v>172</v>
+        <v>178</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E37" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F37" s="2" t="s">
-        <v>174</v>
+        <v>180</v>
       </c>
       <c r="G37" s="2" t="s">
         <v>13</v>
@@ -2836,22 +2842,22 @@
     </row>
     <row r="38" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
-        <v>175</v>
+        <v>181</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>176</v>
+        <v>182</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E38" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F38" s="2" t="s">
-        <v>177</v>
+        <v>183</v>
       </c>
       <c r="G38" s="2" t="s">
         <v>13</v>
@@ -2859,22 +2865,22 @@
     </row>
     <row r="39" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
-        <v>178</v>
+        <v>184</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>179</v>
+        <v>185</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E39" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F39" s="2" t="s">
-        <v>180</v>
+        <v>186</v>
       </c>
       <c r="G39" s="2" t="s">
         <v>13</v>
@@ -2882,22 +2888,22 @@
     </row>
     <row r="40" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
-        <v>181</v>
+        <v>187</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>182</v>
+        <v>188</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E40" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F40" s="2" t="s">
-        <v>183</v>
+        <v>189</v>
       </c>
       <c r="G40" s="2" t="s">
         <v>13</v>
@@ -2905,22 +2911,22 @@
     </row>
     <row r="41" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>185</v>
+        <v>191</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E41" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F41" s="2" t="s">
-        <v>186</v>
+        <v>192</v>
       </c>
       <c r="G41" s="2" t="s">
         <v>13</v>
@@ -2971,22 +2977,22 @@
     </row>
     <row r="2" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>187</v>
+        <v>193</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>188</v>
+        <v>194</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>189</v>
+        <v>195</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>188</v>
+        <v>194</v>
       </c>
       <c r="E2" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>190</v>
+        <v>52</v>
       </c>
       <c r="G2" s="2" t="s">
         <v>13</v>
@@ -2994,22 +3000,22 @@
     </row>
     <row r="3" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>191</v>
+        <v>196</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>188</v>
+        <v>194</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>192</v>
+        <v>197</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>188</v>
+        <v>194</v>
       </c>
       <c r="E3" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>193</v>
+        <v>198</v>
       </c>
       <c r="G3" s="2" t="s">
         <v>13</v>
@@ -3017,22 +3023,22 @@
     </row>
     <row r="4" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="B4" s="2" t="s">
         <v>194</v>
       </c>
-      <c r="B4" s="2" t="s">
-        <v>188</v>
-      </c>
       <c r="C4" s="2" t="s">
-        <v>195</v>
+        <v>200</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>188</v>
+        <v>194</v>
       </c>
       <c r="E4" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>193</v>
+        <v>198</v>
       </c>
       <c r="G4" s="2" t="s">
         <v>13</v>
@@ -3040,16 +3046,16 @@
     </row>
     <row r="5" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>196</v>
+        <v>201</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>188</v>
+        <v>194</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>197</v>
+        <v>202</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>188</v>
+        <v>194</v>
       </c>
       <c r="E5" s="3" t="s">
         <v>11</v>
@@ -3063,22 +3069,22 @@
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>199</v>
+        <v>203</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>188</v>
+        <v>194</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>200</v>
+        <v>204</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>188</v>
+        <v>194</v>
       </c>
       <c r="E6" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>193</v>
+        <v>198</v>
       </c>
       <c r="G6" s="2" t="s">
         <v>13</v>
@@ -3086,22 +3092,22 @@
     </row>
     <row r="7" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>201</v>
+        <v>205</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>188</v>
+        <v>194</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>188</v>
+        <v>194</v>
       </c>
       <c r="E7" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>203</v>
+        <v>33</v>
       </c>
       <c r="G7" s="2" t="s">
         <v>13</v>
@@ -3109,16 +3115,16 @@
     </row>
     <row r="8" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>188</v>
+        <v>194</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>188</v>
+        <v>194</v>
       </c>
       <c r="E8" s="3" t="s">
         <v>11</v>
@@ -3132,22 +3138,22 @@
     </row>
     <row r="9" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>188</v>
+        <v>194</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>188</v>
+        <v>194</v>
       </c>
       <c r="E9" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>193</v>
+        <v>198</v>
       </c>
       <c r="G9" s="2" t="s">
         <v>13</v>
@@ -3155,22 +3161,22 @@
     </row>
     <row r="10" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>188</v>
+        <v>194</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>188</v>
+        <v>194</v>
       </c>
       <c r="E10" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>193</v>
+        <v>213</v>
       </c>
       <c r="G10" s="2" t="s">
         <v>13</v>
@@ -3178,22 +3184,22 @@
     </row>
     <row r="11" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>210</v>
+        <v>214</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>188</v>
+        <v>194</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>188</v>
+        <v>194</v>
       </c>
       <c r="E11" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>193</v>
+        <v>198</v>
       </c>
       <c r="G11" s="2" t="s">
         <v>13</v>
@@ -3201,22 +3207,22 @@
     </row>
     <row r="12" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>212</v>
+        <v>216</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>188</v>
+        <v>194</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>188</v>
+        <v>194</v>
       </c>
       <c r="E12" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>193</v>
+        <v>198</v>
       </c>
       <c r="G12" s="2" t="s">
         <v>13</v>
@@ -3224,22 +3230,22 @@
     </row>
     <row r="13" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>188</v>
+        <v>194</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>215</v>
+        <v>219</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>188</v>
+        <v>194</v>
       </c>
       <c r="E13" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>193</v>
+        <v>198</v>
       </c>
       <c r="G13" s="2" t="s">
         <v>13</v>
@@ -3247,22 +3253,22 @@
     </row>
     <row r="14" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>188</v>
+        <v>194</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>217</v>
+        <v>221</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>188</v>
+        <v>194</v>
       </c>
       <c r="E14" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>193</v>
+        <v>198</v>
       </c>
       <c r="G14" s="2" t="s">
         <v>13</v>
@@ -3270,22 +3276,22 @@
     </row>
     <row r="15" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>188</v>
+        <v>194</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>188</v>
+        <v>194</v>
       </c>
       <c r="E15" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>193</v>
+        <v>198</v>
       </c>
       <c r="G15" s="2" t="s">
         <v>13</v>
@@ -3293,22 +3299,22 @@
     </row>
     <row r="16" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>220</v>
+        <v>224</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>188</v>
+        <v>194</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>188</v>
+        <v>194</v>
       </c>
       <c r="E16" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>193</v>
+        <v>198</v>
       </c>
       <c r="G16" s="2" t="s">
         <v>13</v>
@@ -3316,22 +3322,22 @@
     </row>
     <row r="17" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>188</v>
+        <v>194</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>223</v>
+        <v>227</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>188</v>
+        <v>194</v>
       </c>
       <c r="E17" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>193</v>
+        <v>198</v>
       </c>
       <c r="G17" s="2" t="s">
         <v>13</v>
@@ -3339,22 +3345,22 @@
     </row>
     <row r="18" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>188</v>
+        <v>194</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>225</v>
+        <v>229</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>188</v>
+        <v>194</v>
       </c>
       <c r="E18" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>193</v>
+        <v>198</v>
       </c>
       <c r="G18" s="2" t="s">
         <v>13</v>
@@ -3362,22 +3368,22 @@
     </row>
     <row r="19" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>188</v>
+        <v>194</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>188</v>
+        <v>194</v>
       </c>
       <c r="E19" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>193</v>
+        <v>198</v>
       </c>
       <c r="G19" s="2" t="s">
         <v>13</v>
@@ -3385,22 +3391,22 @@
     </row>
     <row r="20" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>228</v>
+        <v>232</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>188</v>
+        <v>194</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>229</v>
+        <v>233</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>188</v>
+        <v>194</v>
       </c>
       <c r="E20" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>193</v>
+        <v>198</v>
       </c>
       <c r="G20" s="2" t="s">
         <v>13</v>
@@ -3408,22 +3414,22 @@
     </row>
     <row r="21" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>230</v>
+        <v>234</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>188</v>
+        <v>194</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>231</v>
+        <v>235</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>188</v>
+        <v>194</v>
       </c>
       <c r="E21" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>193</v>
+        <v>198</v>
       </c>
       <c r="G21" s="2" t="s">
         <v>13</v>
@@ -3474,22 +3480,22 @@
     </row>
     <row r="2" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>234</v>
+        <v>238</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="E2" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="G2" s="2" t="s">
         <v>13</v>
@@ -3497,22 +3503,22 @@
     </row>
     <row r="3" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>236</v>
+        <v>240</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="C3" s="2" t="s">
+        <v>241</v>
+      </c>
+      <c r="D3" s="2" t="s">
         <v>237</v>
       </c>
-      <c r="D3" s="2" t="s">
-        <v>233</v>
-      </c>
       <c r="E3" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>137</v>
+        <v>55</v>
       </c>
       <c r="G3" s="2" t="s">
         <v>13</v>
@@ -3520,22 +3526,22 @@
     </row>
     <row r="4" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>239</v>
+        <v>243</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="E4" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>240</v>
+        <v>244</v>
       </c>
       <c r="G4" s="2" t="s">
         <v>13</v>
@@ -3543,22 +3549,22 @@
     </row>
     <row r="5" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>242</v>
+        <v>246</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="E5" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>193</v>
+        <v>198</v>
       </c>
       <c r="G5" s="2" t="s">
         <v>13</v>
@@ -3566,22 +3572,22 @@
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>243</v>
+        <v>247</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>244</v>
+        <v>248</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="E6" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
       <c r="G6" s="2" t="s">
         <v>13</v>
@@ -3589,22 +3595,22 @@
     </row>
     <row r="7" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="E7" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>248</v>
+        <v>252</v>
       </c>
       <c r="G7" s="2" t="s">
         <v>13</v>
@@ -3612,22 +3618,22 @@
     </row>
     <row r="8" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>249</v>
+        <v>253</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>250</v>
+        <v>254</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="E8" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>251</v>
+        <v>255</v>
       </c>
       <c r="G8" s="2" t="s">
         <v>13</v>
@@ -3635,22 +3641,22 @@
     </row>
     <row r="9" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>252</v>
+        <v>256</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>253</v>
+        <v>257</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="E9" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>254</v>
+        <v>33</v>
       </c>
       <c r="G9" s="2" t="s">
         <v>13</v>
@@ -3658,22 +3664,22 @@
     </row>
     <row r="10" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="E10" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
       <c r="G10" s="2" t="s">
         <v>13</v>
@@ -3681,22 +3687,22 @@
     </row>
     <row r="11" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="C11" s="2" t="s">
+        <v>263</v>
+      </c>
+      <c r="D11" s="2" t="s">
         <v>260</v>
       </c>
-      <c r="D11" s="2" t="s">
-        <v>257</v>
-      </c>
       <c r="E11" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>193</v>
+        <v>198</v>
       </c>
       <c r="G11" s="2" t="s">
         <v>13</v>
@@ -3704,22 +3710,22 @@
     </row>
     <row r="12" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>262</v>
+        <v>265</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="E12" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>263</v>
+        <v>266</v>
       </c>
       <c r="G12" s="2" t="s">
         <v>13</v>
@@ -3727,22 +3733,22 @@
     </row>
     <row r="13" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>264</v>
+        <v>267</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>265</v>
+        <v>268</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="E13" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>266</v>
+        <v>269</v>
       </c>
       <c r="G13" s="2" t="s">
         <v>13</v>
@@ -3750,22 +3756,22 @@
     </row>
     <row r="14" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>268</v>
+        <v>271</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="E14" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>193</v>
+        <v>198</v>
       </c>
       <c r="G14" s="2" t="s">
         <v>13</v>
@@ -3773,22 +3779,22 @@
     </row>
     <row r="15" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>269</v>
+        <v>272</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="E15" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>271</v>
+        <v>274</v>
       </c>
       <c r="G15" s="2" t="s">
         <v>13</v>
@@ -3796,22 +3802,22 @@
     </row>
     <row r="16" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>272</v>
+        <v>275</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>273</v>
+        <v>276</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="E16" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
       <c r="G16" s="2" t="s">
         <v>13</v>
@@ -3862,22 +3868,22 @@
     </row>
     <row r="2" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>275</v>
+        <v>278</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>277</v>
+        <v>280</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
       <c r="E2" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
       <c r="G2" s="2" t="s">
         <v>13</v>
@@ -3885,22 +3891,22 @@
     </row>
     <row r="3" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>280</v>
+        <v>283</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="C3" s="2" t="s">
+        <v>284</v>
+      </c>
+      <c r="D3" s="2" t="s">
         <v>281</v>
       </c>
-      <c r="D3" s="2" t="s">
-        <v>278</v>
-      </c>
       <c r="E3" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
       <c r="G3" s="2" t="s">
         <v>13</v>
@@ -3908,16 +3914,16 @@
     </row>
     <row r="4" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>283</v>
+        <v>286</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>284</v>
+        <v>287</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="E4" s="3" t="s">
         <v>11</v>
@@ -3931,22 +3937,22 @@
     </row>
     <row r="5" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>285</v>
+        <v>288</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>286</v>
+        <v>289</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="E5" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="G5" s="2" t="s">
         <v>13</v>
@@ -3954,22 +3960,22 @@
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="E6" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>193</v>
+        <v>198</v>
       </c>
       <c r="G6" s="2" t="s">
         <v>13</v>
@@ -3977,22 +3983,22 @@
     </row>
     <row r="7" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>291</v>
+        <v>294</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="E7" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>292</v>
+        <v>295</v>
       </c>
       <c r="G7" s="2" t="s">
         <v>13</v>
@@ -4000,22 +4006,22 @@
     </row>
     <row r="8" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>293</v>
+        <v>296</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>294</v>
+        <v>297</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
       <c r="E8" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="G8" s="2" t="s">
         <v>13</v>
@@ -4023,22 +4029,22 @@
     </row>
     <row r="9" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>296</v>
+        <v>299</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>297</v>
+        <v>300</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
       <c r="E9" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
       <c r="G9" s="2" t="s">
         <v>13</v>
@@ -4046,22 +4052,22 @@
     </row>
     <row r="10" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>299</v>
+        <v>302</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>300</v>
+        <v>303</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
       <c r="E10" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>301</v>
+        <v>134</v>
       </c>
       <c r="G10" s="2" t="s">
         <v>13</v>
@@ -4069,22 +4075,22 @@
     </row>
     <row r="11" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="E11" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>193</v>
+        <v>198</v>
       </c>
       <c r="G11" s="2" t="s">
         <v>13</v>

</xml_diff>

<commit_message>
Implement registration flow, onboarding screen, and repository updates, and synchronize E2E test suite
</commit_message>
<xml_diff>
--- a/tests/reports/Test_Analysis_Report.xlsx
+++ b/tests/reports/Test_Analysis_Report.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="805" uniqueCount="306">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="805" uniqueCount="309">
   <si>
     <t>Test ID</t>
   </si>
@@ -56,7 +56,7 @@
     <t>Passed</t>
   </si>
   <si>
-    <t>304ms</t>
+    <t>2239ms</t>
   </si>
   <si>
     <t>Assertion passed successfully</t>
@@ -68,7 +68,7 @@
     <t>Verify brand name PayBuddy header exists</t>
   </si>
   <si>
-    <t>247ms</t>
+    <t>322ms</t>
   </si>
   <si>
     <t>TC-WEB-UI-003</t>
@@ -77,7 +77,7 @@
     <t>Verify form email input label</t>
   </si>
   <si>
-    <t>15ms</t>
+    <t>53ms</t>
   </si>
   <si>
     <t>TC-WEB-UI-004</t>
@@ -86,850 +86,859 @@
     <t>Verify form password input label</t>
   </si>
   <si>
+    <t>54ms</t>
+  </si>
+  <si>
     <t>TC-WEB-UI-005</t>
   </si>
   <si>
     <t>Verify Sign In button is present</t>
   </si>
   <si>
+    <t>44ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-006</t>
+  </si>
+  <si>
+    <t>Verify secure access footer notice is present</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-007</t>
+  </si>
+  <si>
+    <t>Verify branding subtitle text exists</t>
+  </si>
+  <si>
+    <t>52ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-008</t>
+  </si>
+  <si>
+    <t>Verify email input field placeholder</t>
+  </si>
+  <si>
+    <t>49ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-009</t>
+  </si>
+  <si>
+    <t>Verify password input field placeholder</t>
+  </si>
+  <si>
+    <t>51ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-010</t>
+  </si>
+  <si>
+    <t>Verify font family CSS on headers</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-011</t>
+  </si>
+  <si>
+    <t>Verify primary brand color on buttons</t>
+  </si>
+  <si>
+    <t>47ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-012</t>
+  </si>
+  <si>
+    <t>Verify centered block layout</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-013</t>
+  </si>
+  <si>
+    <t>Verify responsive structure at mobile width 360px</t>
+  </si>
+  <si>
+    <t>945ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-014</t>
+  </si>
+  <si>
+    <t>Verify responsive structure at tablet width 768px</t>
+  </si>
+  <si>
+    <t>942ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-015</t>
+  </si>
+  <si>
+    <t>Restore browser window maximization state</t>
+  </si>
+  <si>
+    <t>59ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-016</t>
+  </si>
+  <si>
+    <t>Verify HTML tag specification for email input</t>
+  </si>
+  <si>
+    <t>67ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-017</t>
+  </si>
+  <si>
+    <t>Verify HTML tag specification for password input</t>
+  </si>
+  <si>
+    <t>50ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-018</t>
+  </si>
+  <si>
+    <t>Verify card wrapper styles (border-radius)</t>
+  </si>
+  <si>
+    <t>110ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-019</t>
+  </si>
+  <si>
+    <t>Verify background styling matches design spec</t>
+  </si>
+  <si>
+    <t>45ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-020</t>
+  </si>
+  <si>
+    <t>Verify focus state click handler does not crash</t>
+  </si>
+  <si>
+    <t>156ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-021</t>
+  </si>
+  <si>
+    <t>Verify top-level container viewport classes</t>
+  </si>
+  <si>
+    <t>64ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-022</t>
+  </si>
+  <si>
+    <t>Verify branding and form division layout margins</t>
+  </si>
+  <si>
+    <t>61ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-023</t>
+  </si>
+  <si>
+    <t>Verify clear textual contrast for reader accessibility</t>
+  </si>
+  <si>
+    <t>56ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-024</t>
+  </si>
+  <si>
+    <t>Verify page scales properly without layout clipping</t>
+  </si>
+  <si>
+    <t>38ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-025</t>
+  </si>
+  <si>
+    <t>Verify smooth interactive transitions on button inputs</t>
+  </si>
+  <si>
+    <t>33ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-001</t>
+  </si>
+  <si>
+    <t>Functional</t>
+  </si>
+  <si>
+    <t>Verify invalid login rejection message</t>
+  </si>
+  <si>
+    <t>1912ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-002</t>
+  </si>
+  <si>
+    <t>Verify rejection of nonexistent email</t>
+  </si>
+  <si>
+    <t>1667ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-003</t>
+  </si>
+  <si>
+    <t>Verify successful login with valid credentials redirects to Dashboard</t>
+  </si>
+  <si>
+    <t>2080ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-004</t>
+  </si>
+  <si>
+    <t>Verify dashboard displays Total Customers count</t>
+  </si>
+  <si>
+    <t>281ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-005</t>
+  </si>
+  <si>
+    <t>Verify dashboard displays Active Sales count</t>
+  </si>
+  <si>
+    <t>60ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-006</t>
+  </si>
+  <si>
+    <t>Verify dashboard displays Pending Installments count</t>
+  </si>
+  <si>
+    <t>35ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-007</t>
+  </si>
+  <si>
+    <t>Verify dashboard displays Today's Due count</t>
+  </si>
+  <si>
+    <t>36ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-008</t>
+  </si>
+  <si>
+    <t>Verify dashboard displays Outstanding Balance amount</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-009</t>
+  </si>
+  <si>
+    <t>Navigate to customers page and verify header</t>
+  </si>
+  <si>
+    <t>393ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-010</t>
+  </si>
+  <si>
+    <t>Verify add new customer input inputs are present</t>
+  </si>
+  <si>
+    <t>57ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-011</t>
+  </si>
+  <si>
+    <t>Verify customer creation and entry addition to table</t>
+  </si>
+  <si>
+    <t>3044ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-012</t>
+  </si>
+  <si>
+    <t>Verify presence of seeded customer</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-013</t>
+  </si>
+  <si>
+    <t>Navigate to specific customer profile page</t>
+  </si>
+  <si>
+    <t>1425ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-014</t>
+  </si>
+  <si>
+    <t>Verify phone number exists on profile detail bar</t>
+  </si>
+  <si>
+    <t>39ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-015</t>
+  </si>
+  <si>
+    <t>Verify Total Amount financial card is 1000 INR</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-016</t>
+  </si>
+  <si>
+    <t>Verify Paid Amount financial card is 0 INR</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-017</t>
+  </si>
+  <si>
+    <t>Verify Outstanding Balance financial card is 1000 INR</t>
+  </si>
+  <si>
+    <t>41ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-018</t>
+  </si>
+  <si>
+    <t>Verify E2E Test Item pending sale is loaded in sales list</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-019</t>
+  </si>
+  <si>
+    <t>Verify redirect to record payment page</t>
+  </si>
+  <si>
+    <t>1096ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-020</t>
+  </si>
+  <si>
+    <t>Verify remaining balance display match before payment</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-021</t>
+  </si>
+  <si>
+    <t>Record payment E2E execution and redirection validation</t>
+  </si>
+  <si>
+    <t>3240ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-022</t>
+  </si>
+  <si>
+    <t>Verify Outstanding Balance updates to 800 INR in customer card</t>
+  </si>
+  <si>
+    <t>1228ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-023</t>
+  </si>
+  <si>
+    <t>Verify Paid Amount updates to 200 INR in customer card</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-024</t>
+  </si>
+  <si>
+    <t>Verify recorded payment entry list matches mode UPI</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-025</t>
+  </si>
+  <si>
+    <t>Verify sales management index loads properly</t>
+  </si>
+  <si>
+    <t>728ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-026</t>
+  </si>
+  <si>
+    <t>Verify sales search filter works properly</t>
+  </si>
+  <si>
+    <t>794ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-027</t>
+  </si>
+  <si>
+    <t>Navigate to Create New Sale form</t>
+  </si>
+  <si>
+    <t>666ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-028</t>
+  </si>
+  <si>
+    <t>Verify total amount computed automatically (2 x 500 = 1000)</t>
+  </si>
+  <si>
+    <t>655ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-029</t>
+  </si>
+  <si>
+    <t>Create sale and verify redirect back to sales table</t>
+  </si>
+  <si>
+    <t>500ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-030</t>
+  </si>
+  <si>
+    <t>Verify Payments page path and title</t>
+  </si>
+  <si>
+    <t>662ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-031</t>
+  </si>
+  <si>
+    <t>Verify E2E transaction exists in master list</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-032</t>
+  </si>
+  <si>
+    <t>Verify Ledger Book page loads</t>
+  </si>
+  <si>
+    <t>743ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-033</t>
+  </si>
+  <si>
+    <t>Verify ledger records contain client name</t>
+  </si>
+  <si>
+    <t>71ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-034</t>
+  </si>
+  <si>
+    <t>Verify Installments page title</t>
+  </si>
+  <si>
+    <t>648ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-035</t>
+  </si>
+  <si>
+    <t>Verify customer details exist on installment board</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-036</t>
+  </si>
+  <si>
+    <t>Verify direct Dashboard URL redirect</t>
+  </si>
+  <si>
+    <t>123ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-037</t>
+  </si>
+  <si>
+    <t>Verify customer data updates dynamically on UI edit</t>
+  </si>
+  <si>
+    <t>4674ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-038</t>
+  </si>
+  <si>
+    <t>Verify logout route terminates session and redirects to sign in</t>
+  </si>
+  <si>
+    <t>809ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-039</t>
+  </si>
+  <si>
+    <t>Verify unauthorized dashboard access redirects to login</t>
+  </si>
+  <si>
+    <t>2153ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-040</t>
+  </si>
+  <si>
+    <t>Verify unauthorized customer details access redirects to login</t>
+  </si>
+  <si>
+    <t>TC-WEB-UNIT-001</t>
+  </si>
+  <si>
+    <t>Unit</t>
+  </si>
+  <si>
+    <t>Test formatCurrency formatting positive amount</t>
+  </si>
+  <si>
+    <t>79ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UNIT-002</t>
+  </si>
+  <si>
+    <t>Test formatCurrency formatting zero amount</t>
+  </si>
+  <si>
+    <t>1ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UNIT-003</t>
+  </si>
+  <si>
+    <t>Test formatCurrency formatting negative amount</t>
+  </si>
+  <si>
+    <t>2ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UNIT-004</t>
+  </si>
+  <si>
+    <t>Test formatCurrency formatting large millions scale amount</t>
+  </si>
+  <si>
+    <t>0ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UNIT-005</t>
+  </si>
+  <si>
+    <t>Test formatCurrency decimal rounding functionality</t>
+  </si>
+  <si>
+    <t>TC-WEB-UNIT-006</t>
+  </si>
+  <si>
+    <t>Test formatDate string matching date details</t>
+  </si>
+  <si>
+    <t>22ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UNIT-007</t>
+  </si>
+  <si>
+    <t>Test formatDate fallback for null values</t>
+  </si>
+  <si>
+    <t>TC-WEB-UNIT-008</t>
+  </si>
+  <si>
+    <t>Test formatDate fallback for 0 value</t>
+  </si>
+  <si>
+    <t>TC-WEB-UNIT-009</t>
+  </si>
+  <si>
+    <t>Test formatDateTime details formatting</t>
+  </si>
+  <si>
+    <t>TC-WEB-UNIT-010</t>
+  </si>
+  <si>
+    <t>Test formatDateTime null timestamp handling</t>
+  </si>
+  <si>
+    <t>TC-WEB-UNIT-011</t>
+  </si>
+  <si>
+    <t>Verify email validation for valid string</t>
+  </si>
+  <si>
+    <t>TC-WEB-UNIT-012</t>
+  </si>
+  <si>
+    <t>Verify email validation blocks missing TLD</t>
+  </si>
+  <si>
+    <t>TC-WEB-UNIT-013</t>
+  </si>
+  <si>
+    <t>Verify email validation blocks missing alias prefix</t>
+  </si>
+  <si>
+    <t>TC-WEB-UNIT-014</t>
+  </si>
+  <si>
+    <t>Verify phone validation for standard 10 digit number</t>
+  </si>
+  <si>
+    <t>TC-WEB-UNIT-015</t>
+  </si>
+  <si>
+    <t>Verify phone validation blocks short length</t>
+  </si>
+  <si>
+    <t>TC-WEB-UNIT-016</t>
+  </si>
+  <si>
+    <t>Verify phone validation blocks alphabetic characters</t>
+  </si>
+  <si>
+    <t>TC-WEB-UNIT-017</t>
+  </si>
+  <si>
+    <t>Verify interest formula multiplication logic</t>
+  </si>
+  <si>
+    <t>TC-WEB-UNIT-018</t>
+  </si>
+  <si>
+    <t>Verify installment partitioning amount division</t>
+  </si>
+  <si>
+    <t>TC-WEB-UNIT-019</t>
+  </si>
+  <si>
+    <t>Verify remaining balance arithmetic subtraction</t>
+  </si>
+  <si>
+    <t>TC-WEB-UNIT-020</t>
+  </si>
+  <si>
+    <t>Verify mock environment manifest validator passes</t>
+  </si>
+  <si>
+    <t>TC-WEB-VAL-001</t>
+  </si>
+  <si>
+    <t>Validation</t>
+  </si>
+  <si>
+    <t>Verify email required constraint is enabled on form</t>
+  </si>
+  <si>
+    <t>191ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-VAL-002</t>
+  </si>
+  <si>
+    <t>Verify password required constraint is enabled on form</t>
+  </si>
+  <si>
+    <t>TC-WEB-VAL-003</t>
+  </si>
+  <si>
+    <t>Verify browser client blocks submissions for invalid email inputs</t>
+  </si>
+  <si>
+    <t>253ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-VAL-004</t>
+  </si>
+  <si>
+    <t>Verify character bounds for data buffers limit to 255 characters</t>
+  </si>
+  <si>
+    <t>TC-WEB-VAL-005</t>
+  </si>
+  <si>
+    <t>Verify customer creation form prevents empty submit</t>
+  </si>
+  <si>
+    <t>3184ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-VAL-006</t>
+  </si>
+  <si>
+    <t>Verify phone input uses tel semantic element type</t>
+  </si>
+  <si>
+    <t>TC-WEB-VAL-007</t>
+  </si>
+  <si>
+    <t>Verify sale quantity requires positive minimum value (&gt; 0)</t>
+  </si>
+  <si>
+    <t>624ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-VAL-008</t>
+  </si>
+  <si>
+    <t>Verify unit price input restricts negative numbers</t>
+  </si>
+  <si>
+    <t>37ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-VAL-009</t>
+  </si>
+  <si>
+    <t>Verify script tag input text does not trigger native alerts</t>
+  </si>
+  <si>
+    <t>Security</t>
+  </si>
+  <si>
+    <t>2472ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-VAL-010</t>
+  </si>
+  <si>
+    <t>Verify database adapter parameters parameterized input query parsing</t>
+  </si>
+  <si>
+    <t>TC-WEB-VAL-011</t>
+  </si>
+  <si>
+    <t>Verify error prevents overpayment collections</t>
+  </si>
+  <si>
+    <t>1936ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-VAL-012</t>
+  </si>
+  <si>
+    <t>Verify collection input restricts 0 value submissions</t>
+  </si>
+  <si>
+    <t>1437ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-VAL-013</t>
+  </si>
+  <si>
+    <t>Verify Firestore writes match schema constraints</t>
+  </si>
+  <si>
+    <t>TC-WEB-VAL-014</t>
+  </si>
+  <si>
+    <t>Verify wildcard URLs redirect to main route base</t>
+  </si>
+  <si>
+    <t>2128ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-VAL-015</t>
+  </si>
+  <si>
+    <t>Verify HTML password hidden mask attribute config</t>
+  </si>
+  <si>
+    <t>844ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-DEP-001</t>
+  </si>
+  <si>
+    <t>Deployment</t>
+  </si>
+  <si>
+    <t>Verify load paint FCP under 2.5s threshold</t>
+  </si>
+  <si>
+    <t>Performance</t>
+  </si>
+  <si>
+    <t>152ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-DEP-002</t>
+  </si>
+  <si>
+    <t>Verify full render transition load time under limit</t>
+  </si>
+  <si>
+    <t>1451ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-DEP-003</t>
+  </si>
+  <si>
+    <t>Verify DNS host domain matches Vercel production edge</t>
+  </si>
+  <si>
+    <t>TC-WEB-DEP-004</t>
+  </si>
+  <si>
+    <t>Verify favicon.ico endpoint yields clean HTTP status</t>
+  </si>
+  <si>
+    <t>127ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-DEP-005</t>
+  </si>
+  <si>
+    <t>Verify production connection protocol HTTPS encryption is active</t>
+  </si>
+  <si>
+    <t>TC-WEB-DEP-006</t>
+  </si>
+  <si>
+    <t>Verify head links contain manifest registration details</t>
+  </si>
+  <si>
+    <t>184ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-DEP-007</t>
+  </si>
+  <si>
+    <t>Verify console logs have no severe exceptions during login page session</t>
+  </si>
+  <si>
+    <t>8ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-DEP-008</t>
+  </si>
+  <si>
+    <t>Verify standard responsive layouts align horizontally</t>
+  </si>
+  <si>
+    <t>TC-WEB-DEP-009</t>
+  </si>
+  <si>
+    <t>Verify DOM count index scales cleanly</t>
+  </si>
+  <si>
     <t>14ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UI-006</t>
-  </si>
-  <si>
-    <t>Verify secure access footer notice is present</t>
-  </si>
-  <si>
-    <t>TC-WEB-UI-007</t>
-  </si>
-  <si>
-    <t>Verify branding subtitle text exists</t>
-  </si>
-  <si>
-    <t>TC-WEB-UI-008</t>
-  </si>
-  <si>
-    <t>Verify email input field placeholder</t>
-  </si>
-  <si>
-    <t>TC-WEB-UI-009</t>
-  </si>
-  <si>
-    <t>Verify password input field placeholder</t>
-  </si>
-  <si>
-    <t>13ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UI-010</t>
-  </si>
-  <si>
-    <t>Verify font family CSS on headers</t>
-  </si>
-  <si>
-    <t>16ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UI-011</t>
-  </si>
-  <si>
-    <t>Verify primary brand color on buttons</t>
-  </si>
-  <si>
-    <t>TC-WEB-UI-012</t>
-  </si>
-  <si>
-    <t>Verify centered block layout</t>
-  </si>
-  <si>
-    <t>TC-WEB-UI-013</t>
-  </si>
-  <si>
-    <t>Verify responsive structure at mobile width 360px</t>
-  </si>
-  <si>
-    <t>890ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UI-014</t>
-  </si>
-  <si>
-    <t>Verify responsive structure at tablet width 768px</t>
-  </si>
-  <si>
-    <t>884ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UI-015</t>
-  </si>
-  <si>
-    <t>Restore browser window maximization state</t>
-  </si>
-  <si>
-    <t>23ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UI-016</t>
-  </si>
-  <si>
-    <t>Verify HTML tag specification for email input</t>
-  </si>
-  <si>
-    <t>25ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UI-017</t>
-  </si>
-  <si>
-    <t>Verify HTML tag specification for password input</t>
-  </si>
-  <si>
-    <t>12ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UI-018</t>
-  </si>
-  <si>
-    <t>Verify card wrapper styles (border-radius)</t>
-  </si>
-  <si>
-    <t>37ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UI-019</t>
-  </si>
-  <si>
-    <t>Verify background styling matches design spec</t>
-  </si>
-  <si>
-    <t>17ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UI-020</t>
-  </si>
-  <si>
-    <t>Verify focus state click handler does not crash</t>
-  </si>
-  <si>
-    <t>131ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UI-021</t>
-  </si>
-  <si>
-    <t>Verify top-level container viewport classes</t>
-  </si>
-  <si>
-    <t>29ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UI-022</t>
-  </si>
-  <si>
-    <t>Verify branding and form division layout margins</t>
-  </si>
-  <si>
-    <t>24ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UI-023</t>
-  </si>
-  <si>
-    <t>Verify clear textual contrast for reader accessibility</t>
-  </si>
-  <si>
-    <t>35ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UI-024</t>
-  </si>
-  <si>
-    <t>Verify page scales properly without layout clipping</t>
-  </si>
-  <si>
-    <t>TC-WEB-UI-025</t>
-  </si>
-  <si>
-    <t>Verify smooth interactive transitions on button inputs</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-001</t>
-  </si>
-  <si>
-    <t>Functional</t>
-  </si>
-  <si>
-    <t>Verify invalid login rejection message</t>
-  </si>
-  <si>
-    <t>1153ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-002</t>
-  </si>
-  <si>
-    <t>Verify rejection of nonexistent email</t>
-  </si>
-  <si>
-    <t>839ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-003</t>
-  </si>
-  <si>
-    <t>Verify successful login with valid credentials redirects to Dashboard</t>
-  </si>
-  <si>
-    <t>1702ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-004</t>
-  </si>
-  <si>
-    <t>Verify dashboard displays Total Customers count</t>
-  </si>
-  <si>
-    <t>496ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-005</t>
-  </si>
-  <si>
-    <t>Verify dashboard displays Active Sales count</t>
-  </si>
-  <si>
-    <t>43ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-006</t>
-  </si>
-  <si>
-    <t>Verify dashboard displays Pending Installments count</t>
-  </si>
-  <si>
-    <t>45ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-007</t>
-  </si>
-  <si>
-    <t>Verify dashboard displays Today's Due count</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-008</t>
-  </si>
-  <si>
-    <t>Verify dashboard displays Outstanding Balance amount</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-009</t>
-  </si>
-  <si>
-    <t>Navigate to customers page and verify header</t>
-  </si>
-  <si>
-    <t>163ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-010</t>
-  </si>
-  <si>
-    <t>Verify add new customer input inputs are present</t>
-  </si>
-  <si>
-    <t>33ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-011</t>
-  </si>
-  <si>
-    <t>Verify customer creation and entry addition to table</t>
-  </si>
-  <si>
-    <t>2539ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-012</t>
-  </si>
-  <si>
-    <t>Verify presence of seeded customer</t>
-  </si>
-  <si>
-    <t>21ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-013</t>
-  </si>
-  <si>
-    <t>Navigate to specific customer profile page</t>
-  </si>
-  <si>
-    <t>1131ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-014</t>
-  </si>
-  <si>
-    <t>Verify phone number exists on profile detail bar</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-015</t>
-  </si>
-  <si>
-    <t>Verify Total Amount financial card is 1000 INR</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-016</t>
-  </si>
-  <si>
-    <t>Verify Paid Amount financial card is 0 INR</t>
-  </si>
-  <si>
-    <t>86ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-017</t>
-  </si>
-  <si>
-    <t>Verify Outstanding Balance financial card is 1000 INR</t>
-  </si>
-  <si>
-    <t>28ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-018</t>
-  </si>
-  <si>
-    <t>Verify E2E Test Item pending sale is loaded in sales list</t>
-  </si>
-  <si>
-    <t>18ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-019</t>
-  </si>
-  <si>
-    <t>Verify redirect to record payment page</t>
-  </si>
-  <si>
-    <t>761ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-020</t>
-  </si>
-  <si>
-    <t>Verify remaining balance display match before payment</t>
-  </si>
-  <si>
-    <t>19ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-021</t>
-  </si>
-  <si>
-    <t>Record payment E2E execution and redirection validation</t>
-  </si>
-  <si>
-    <t>3226ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-022</t>
-  </si>
-  <si>
-    <t>Verify Outstanding Balance updates to 800 INR in customer card</t>
-  </si>
-  <si>
-    <t>1192ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-023</t>
-  </si>
-  <si>
-    <t>Verify Paid Amount updates to 200 INR in customer card</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-024</t>
-  </si>
-  <si>
-    <t>Verify recorded payment entry list matches mode UPI</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-025</t>
-  </si>
-  <si>
-    <t>Verify sales management index loads properly</t>
-  </si>
-  <si>
-    <t>866ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-026</t>
-  </si>
-  <si>
-    <t>Verify sales search filter works properly</t>
-  </si>
-  <si>
-    <t>728ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-027</t>
-  </si>
-  <si>
-    <t>Navigate to Create New Sale form</t>
-  </si>
-  <si>
-    <t>801ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-028</t>
-  </si>
-  <si>
-    <t>Verify total amount computed automatically (2 x 500 = 1000)</t>
-  </si>
-  <si>
-    <t>307ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-029</t>
-  </si>
-  <si>
-    <t>Create sale and verify redirect back to sales table</t>
-  </si>
-  <si>
-    <t>207ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-030</t>
-  </si>
-  <si>
-    <t>Verify Payments page path and title</t>
-  </si>
-  <si>
-    <t>591ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-031</t>
-  </si>
-  <si>
-    <t>Verify E2E transaction exists in master list</t>
-  </si>
-  <si>
-    <t>85ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-032</t>
-  </si>
-  <si>
-    <t>Verify Ledger Book page loads</t>
-  </si>
-  <si>
-    <t>799ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-033</t>
-  </si>
-  <si>
-    <t>Verify ledger records contain client name</t>
-  </si>
-  <si>
-    <t>121ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-034</t>
-  </si>
-  <si>
-    <t>Verify Installments page title</t>
-  </si>
-  <si>
-    <t>568ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-035</t>
-  </si>
-  <si>
-    <t>Verify customer details exist on installment board</t>
-  </si>
-  <si>
-    <t>53ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-036</t>
-  </si>
-  <si>
-    <t>Verify direct Dashboard URL redirect</t>
-  </si>
-  <si>
-    <t>106ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-037</t>
-  </si>
-  <si>
-    <t>Verify customer data updates dynamically on UI edit</t>
-  </si>
-  <si>
-    <t>4447ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-038</t>
-  </si>
-  <si>
-    <t>Verify logout route terminates session and redirects to sign in</t>
-  </si>
-  <si>
-    <t>1050ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-039</t>
-  </si>
-  <si>
-    <t>Verify unauthorized dashboard access redirects to login</t>
-  </si>
-  <si>
-    <t>2104ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-040</t>
-  </si>
-  <si>
-    <t>Verify unauthorized customer details access redirects to login</t>
-  </si>
-  <si>
-    <t>2103ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UNIT-001</t>
-  </si>
-  <si>
-    <t>Unit</t>
-  </si>
-  <si>
-    <t>Test formatCurrency formatting positive amount</t>
-  </si>
-  <si>
-    <t>TC-WEB-UNIT-002</t>
-  </si>
-  <si>
-    <t>Test formatCurrency formatting zero amount</t>
-  </si>
-  <si>
-    <t>0ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UNIT-003</t>
-  </si>
-  <si>
-    <t>Test formatCurrency formatting negative amount</t>
-  </si>
-  <si>
-    <t>TC-WEB-UNIT-004</t>
-  </si>
-  <si>
-    <t>Test formatCurrency formatting large millions scale amount</t>
-  </si>
-  <si>
-    <t>TC-WEB-UNIT-005</t>
-  </si>
-  <si>
-    <t>Test formatCurrency decimal rounding functionality</t>
-  </si>
-  <si>
-    <t>TC-WEB-UNIT-006</t>
-  </si>
-  <si>
-    <t>Test formatDate string matching date details</t>
-  </si>
-  <si>
-    <t>TC-WEB-UNIT-007</t>
-  </si>
-  <si>
-    <t>Test formatDate fallback for null values</t>
-  </si>
-  <si>
-    <t>TC-WEB-UNIT-008</t>
-  </si>
-  <si>
-    <t>Test formatDate fallback for 0 value</t>
-  </si>
-  <si>
-    <t>TC-WEB-UNIT-009</t>
-  </si>
-  <si>
-    <t>Test formatDateTime details formatting</t>
-  </si>
-  <si>
-    <t>1ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UNIT-010</t>
-  </si>
-  <si>
-    <t>Test formatDateTime null timestamp handling</t>
-  </si>
-  <si>
-    <t>TC-WEB-UNIT-011</t>
-  </si>
-  <si>
-    <t>Verify email validation for valid string</t>
-  </si>
-  <si>
-    <t>TC-WEB-UNIT-012</t>
-  </si>
-  <si>
-    <t>Verify email validation blocks missing TLD</t>
-  </si>
-  <si>
-    <t>TC-WEB-UNIT-013</t>
-  </si>
-  <si>
-    <t>Verify email validation blocks missing alias prefix</t>
-  </si>
-  <si>
-    <t>TC-WEB-UNIT-014</t>
-  </si>
-  <si>
-    <t>Verify phone validation for standard 10 digit number</t>
-  </si>
-  <si>
-    <t>TC-WEB-UNIT-015</t>
-  </si>
-  <si>
-    <t>Verify phone validation blocks short length</t>
-  </si>
-  <si>
-    <t>TC-WEB-UNIT-016</t>
-  </si>
-  <si>
-    <t>Verify phone validation blocks alphabetic characters</t>
-  </si>
-  <si>
-    <t>TC-WEB-UNIT-017</t>
-  </si>
-  <si>
-    <t>Verify interest formula multiplication logic</t>
-  </si>
-  <si>
-    <t>TC-WEB-UNIT-018</t>
-  </si>
-  <si>
-    <t>Verify installment partitioning amount division</t>
-  </si>
-  <si>
-    <t>TC-WEB-UNIT-019</t>
-  </si>
-  <si>
-    <t>Verify remaining balance arithmetic subtraction</t>
-  </si>
-  <si>
-    <t>TC-WEB-UNIT-020</t>
-  </si>
-  <si>
-    <t>Verify mock environment manifest validator passes</t>
-  </si>
-  <si>
-    <t>TC-WEB-VAL-001</t>
-  </si>
-  <si>
-    <t>Validation</t>
-  </si>
-  <si>
-    <t>Verify email required constraint is enabled on form</t>
-  </si>
-  <si>
-    <t>329ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-VAL-002</t>
-  </si>
-  <si>
-    <t>Verify password required constraint is enabled on form</t>
-  </si>
-  <si>
-    <t>TC-WEB-VAL-003</t>
-  </si>
-  <si>
-    <t>Verify browser client blocks submissions for invalid email inputs</t>
-  </si>
-  <si>
-    <t>107ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-VAL-004</t>
-  </si>
-  <si>
-    <t>Verify character bounds for data buffers limit to 255 characters</t>
-  </si>
-  <si>
-    <t>TC-WEB-VAL-005</t>
-  </si>
-  <si>
-    <t>Verify customer creation form prevents empty submit</t>
-  </si>
-  <si>
-    <t>3059ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-VAL-006</t>
-  </si>
-  <si>
-    <t>Verify phone input uses tel semantic element type</t>
-  </si>
-  <si>
-    <t>26ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-VAL-007</t>
-  </si>
-  <si>
-    <t>Verify sale quantity requires positive minimum value (&gt; 0)</t>
-  </si>
-  <si>
-    <t>563ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-VAL-008</t>
-  </si>
-  <si>
-    <t>Verify unit price input restricts negative numbers</t>
-  </si>
-  <si>
-    <t>TC-WEB-VAL-009</t>
-  </si>
-  <si>
-    <t>Verify script tag input text does not trigger native alerts</t>
-  </si>
-  <si>
-    <t>Security</t>
-  </si>
-  <si>
-    <t>2311ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-VAL-010</t>
-  </si>
-  <si>
-    <t>Verify database adapter parameters parameterized input query parsing</t>
-  </si>
-  <si>
-    <t>TC-WEB-VAL-011</t>
-  </si>
-  <si>
-    <t>Verify error prevents overpayment collections</t>
-  </si>
-  <si>
-    <t>2120ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-VAL-012</t>
-  </si>
-  <si>
-    <t>Verify collection input restricts 0 value submissions</t>
-  </si>
-  <si>
-    <t>1143ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-VAL-013</t>
-  </si>
-  <si>
-    <t>Verify Firestore writes match schema constraints</t>
-  </si>
-  <si>
-    <t>TC-WEB-VAL-014</t>
-  </si>
-  <si>
-    <t>Verify wildcard URLs redirect to main route base</t>
-  </si>
-  <si>
-    <t>2118ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-VAL-015</t>
-  </si>
-  <si>
-    <t>Verify HTML password hidden mask attribute config</t>
-  </si>
-  <si>
-    <t>668ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-DEP-001</t>
-  </si>
-  <si>
-    <t>Deployment</t>
-  </si>
-  <si>
-    <t>Verify load paint FCP under 2.5s threshold</t>
-  </si>
-  <si>
-    <t>Performance</t>
-  </si>
-  <si>
-    <t>124ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-DEP-002</t>
-  </si>
-  <si>
-    <t>Verify full render transition load time under limit</t>
-  </si>
-  <si>
-    <t>1185ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-DEP-003</t>
-  </si>
-  <si>
-    <t>Verify DNS host domain matches Vercel production edge</t>
-  </si>
-  <si>
-    <t>TC-WEB-DEP-004</t>
-  </si>
-  <si>
-    <t>Verify favicon.ico endpoint yields clean HTTP status</t>
-  </si>
-  <si>
-    <t>103ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-DEP-005</t>
-  </si>
-  <si>
-    <t>Verify production connection protocol HTTPS encryption is active</t>
-  </si>
-  <si>
-    <t>TC-WEB-DEP-006</t>
-  </si>
-  <si>
-    <t>Verify head links contain manifest registration details</t>
-  </si>
-  <si>
-    <t>147ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-DEP-007</t>
-  </si>
-  <si>
-    <t>Verify console logs have no severe exceptions during login page session</t>
-  </si>
-  <si>
-    <t>3ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-DEP-008</t>
-  </si>
-  <si>
-    <t>Verify standard responsive layouts align horizontally</t>
-  </si>
-  <si>
-    <t>56ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-DEP-009</t>
-  </si>
-  <si>
-    <t>Verify DOM count index scales cleanly</t>
   </si>
   <si>
     <t>TC-WEB-DEP-010</t>
@@ -1480,7 +1489,7 @@
         <v>11</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="G5" s="2" t="s">
         <v>13</v>
@@ -1488,13 +1497,13 @@
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>10</v>
@@ -1503,7 +1512,7 @@
         <v>11</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G6" s="2" t="s">
         <v>13</v>
@@ -1511,13 +1520,13 @@
     </row>
     <row r="7" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>10</v>
@@ -1526,7 +1535,7 @@
         <v>11</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="G7" s="2" t="s">
         <v>13</v>
@@ -1534,13 +1543,13 @@
     </row>
     <row r="8" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>10</v>
@@ -1549,7 +1558,7 @@
         <v>11</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="G8" s="2" t="s">
         <v>13</v>
@@ -1557,13 +1566,13 @@
     </row>
     <row r="9" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>10</v>
@@ -1572,7 +1581,7 @@
         <v>11</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>24</v>
+        <v>33</v>
       </c>
       <c r="G9" s="2" t="s">
         <v>13</v>
@@ -1580,13 +1589,13 @@
     </row>
     <row r="10" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="D10" s="2" t="s">
         <v>10</v>
@@ -1595,7 +1604,7 @@
         <v>11</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="G10" s="2" t="s">
         <v>13</v>
@@ -1603,13 +1612,13 @@
     </row>
     <row r="11" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="B11" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="D11" s="2" t="s">
         <v>10</v>
@@ -1618,7 +1627,7 @@
         <v>11</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>36</v>
+        <v>22</v>
       </c>
       <c r="G11" s="2" t="s">
         <v>13</v>
@@ -1626,13 +1635,13 @@
     </row>
     <row r="12" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B12" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="D12" s="2" t="s">
         <v>10</v>
@@ -1641,7 +1650,7 @@
         <v>11</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>33</v>
+        <v>41</v>
       </c>
       <c r="G12" s="2" t="s">
         <v>13</v>
@@ -1649,13 +1658,13 @@
     </row>
     <row r="13" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="B13" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="D13" s="2" t="s">
         <v>10</v>
@@ -1664,7 +1673,7 @@
         <v>11</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="G13" s="2" t="s">
         <v>13</v>
@@ -1672,13 +1681,13 @@
     </row>
     <row r="14" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="B14" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="D14" s="2" t="s">
         <v>10</v>
@@ -1687,7 +1696,7 @@
         <v>11</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="G14" s="2" t="s">
         <v>13</v>
@@ -1695,13 +1704,13 @@
     </row>
     <row r="15" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="B15" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="D15" s="2" t="s">
         <v>10</v>
@@ -1710,7 +1719,7 @@
         <v>11</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="G15" s="2" t="s">
         <v>13</v>
@@ -1718,13 +1727,13 @@
     </row>
     <row r="16" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="B16" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="D16" s="2" t="s">
         <v>10</v>
@@ -1733,7 +1742,7 @@
         <v>11</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="G16" s="2" t="s">
         <v>13</v>
@@ -1741,13 +1750,13 @@
     </row>
     <row r="17" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="B17" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="D17" s="2" t="s">
         <v>10</v>
@@ -1756,7 +1765,7 @@
         <v>11</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="G17" s="2" t="s">
         <v>13</v>
@@ -1764,13 +1773,13 @@
     </row>
     <row r="18" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="B18" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="D18" s="2" t="s">
         <v>10</v>
@@ -1779,7 +1788,7 @@
         <v>11</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="G18" s="2" t="s">
         <v>13</v>
@@ -1787,13 +1796,13 @@
     </row>
     <row r="19" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="B19" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="D19" s="2" t="s">
         <v>10</v>
@@ -1802,7 +1811,7 @@
         <v>11</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="G19" s="2" t="s">
         <v>13</v>
@@ -1810,13 +1819,13 @@
     </row>
     <row r="20" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="B20" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="D20" s="2" t="s">
         <v>10</v>
@@ -1825,7 +1834,7 @@
         <v>11</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="G20" s="2" t="s">
         <v>13</v>
@@ -1833,13 +1842,13 @@
     </row>
     <row r="21" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="B21" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="D21" s="2" t="s">
         <v>10</v>
@@ -1848,7 +1857,7 @@
         <v>11</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="G21" s="2" t="s">
         <v>13</v>
@@ -1856,13 +1865,13 @@
     </row>
     <row r="22" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="B22" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="D22" s="2" t="s">
         <v>10</v>
@@ -1871,7 +1880,7 @@
         <v>11</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="G22" s="2" t="s">
         <v>13</v>
@@ -1879,13 +1888,13 @@
     </row>
     <row r="23" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="B23" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="D23" s="2" t="s">
         <v>10</v>
@@ -1894,7 +1903,7 @@
         <v>11</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="G23" s="2" t="s">
         <v>13</v>
@@ -1902,13 +1911,13 @@
     </row>
     <row r="24" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="B24" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="D24" s="2" t="s">
         <v>10</v>
@@ -1917,7 +1926,7 @@
         <v>11</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="G24" s="2" t="s">
         <v>13</v>
@@ -1925,13 +1934,13 @@
     </row>
     <row r="25" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="B25" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="D25" s="2" t="s">
         <v>10</v>
@@ -1940,7 +1949,7 @@
         <v>11</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>36</v>
+        <v>79</v>
       </c>
       <c r="G25" s="2" t="s">
         <v>13</v>
@@ -1948,13 +1957,13 @@
     </row>
     <row r="26" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="B26" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="D26" s="2" t="s">
         <v>10</v>
@@ -1963,7 +1972,7 @@
         <v>11</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>61</v>
+        <v>82</v>
       </c>
       <c r="G26" s="2" t="s">
         <v>13</v>
@@ -2014,22 +2023,22 @@
     </row>
     <row r="2" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="E2" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="G2" s="2" t="s">
         <v>13</v>
@@ -2037,22 +2046,22 @@
     </row>
     <row r="3" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="E3" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="G3" s="2" t="s">
         <v>13</v>
@@ -2060,22 +2069,22 @@
     </row>
     <row r="4" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="E4" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="G4" s="2" t="s">
         <v>13</v>
@@ -2083,22 +2092,22 @@
     </row>
     <row r="5" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="E5" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="G5" s="2" t="s">
         <v>13</v>
@@ -2106,22 +2115,22 @@
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="E6" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="G6" s="2" t="s">
         <v>13</v>
@@ -2129,22 +2138,22 @@
     </row>
     <row r="7" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="E7" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="G7" s="2" t="s">
         <v>13</v>
@@ -2152,22 +2161,22 @@
     </row>
     <row r="8" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="E8" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>52</v>
+        <v>104</v>
       </c>
       <c r="G8" s="2" t="s">
         <v>13</v>
@@ -2175,22 +2184,22 @@
     </row>
     <row r="9" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="E9" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>52</v>
+        <v>41</v>
       </c>
       <c r="G9" s="2" t="s">
         <v>13</v>
@@ -2198,22 +2207,22 @@
     </row>
     <row r="10" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="E10" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="G10" s="2" t="s">
         <v>13</v>
@@ -2221,22 +2230,22 @@
     </row>
     <row r="11" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="E11" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
       <c r="G11" s="2" t="s">
         <v>13</v>
@@ -2244,22 +2253,22 @@
     </row>
     <row r="12" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="E12" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="G12" s="2" t="s">
         <v>13</v>
@@ -2267,22 +2276,22 @@
     </row>
     <row r="13" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="E13" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>112</v>
+        <v>73</v>
       </c>
       <c r="G13" s="2" t="s">
         <v>13</v>
@@ -2290,22 +2299,22 @@
     </row>
     <row r="14" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="E14" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="G14" s="2" t="s">
         <v>13</v>
@@ -2313,22 +2322,22 @@
     </row>
     <row r="15" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="E15" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>24</v>
+        <v>123</v>
       </c>
       <c r="G15" s="2" t="s">
         <v>13</v>
@@ -2336,22 +2345,22 @@
     </row>
     <row r="16" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="E16" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>24</v>
+        <v>101</v>
       </c>
       <c r="G16" s="2" t="s">
         <v>13</v>
@@ -2359,22 +2368,22 @@
     </row>
     <row r="17" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="B17" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F17" s="2" t="s">
         <v>79</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>121</v>
-      </c>
-      <c r="D17" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="E17" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F17" s="2" t="s">
-        <v>122</v>
       </c>
       <c r="G17" s="2" t="s">
         <v>13</v>
@@ -2382,22 +2391,22 @@
     </row>
     <row r="18" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>124</v>
+        <v>129</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="E18" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="G18" s="2" t="s">
         <v>13</v>
@@ -2405,22 +2414,22 @@
     </row>
     <row r="19" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>126</v>
+        <v>131</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>127</v>
+        <v>132</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="E19" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="G19" s="2" t="s">
         <v>13</v>
@@ -2428,22 +2437,22 @@
     </row>
     <row r="20" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="E20" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="G20" s="2" t="s">
         <v>13</v>
@@ -2451,22 +2460,22 @@
     </row>
     <row r="21" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="E21" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>134</v>
+        <v>70</v>
       </c>
       <c r="G21" s="2" t="s">
         <v>13</v>
@@ -2474,22 +2483,22 @@
     </row>
     <row r="22" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="E22" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="G22" s="2" t="s">
         <v>13</v>
@@ -2497,22 +2506,22 @@
     </row>
     <row r="23" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="E23" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="G23" s="2" t="s">
         <v>13</v>
@@ -2520,22 +2529,22 @@
     </row>
     <row r="24" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="E24" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="G24" s="2" t="s">
         <v>13</v>
@@ -2543,22 +2552,22 @@
     </row>
     <row r="25" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="E25" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="G25" s="2" t="s">
         <v>13</v>
@@ -2566,22 +2575,22 @@
     </row>
     <row r="26" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="E26" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="G26" s="2" t="s">
         <v>13</v>
@@ -2589,22 +2598,22 @@
     </row>
     <row r="27" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="E27" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="G27" s="2" t="s">
         <v>13</v>
@@ -2612,22 +2621,22 @@
     </row>
     <row r="28" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="E28" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F28" s="2" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="G28" s="2" t="s">
         <v>13</v>
@@ -2635,22 +2644,22 @@
     </row>
     <row r="29" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="E29" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F29" s="2" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="G29" s="2" t="s">
         <v>13</v>
@@ -2658,22 +2667,22 @@
     </row>
     <row r="30" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="E30" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F30" s="2" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="G30" s="2" t="s">
         <v>13</v>
@@ -2681,22 +2690,22 @@
     </row>
     <row r="31" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="E31" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F31" s="2" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="G31" s="2" t="s">
         <v>13</v>
@@ -2704,22 +2713,22 @@
     </row>
     <row r="32" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="E32" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F32" s="2" t="s">
-        <v>165</v>
+        <v>55</v>
       </c>
       <c r="G32" s="2" t="s">
         <v>13</v>
@@ -2727,22 +2736,22 @@
     </row>
     <row r="33" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="E33" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F33" s="2" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="G33" s="2" t="s">
         <v>13</v>
@@ -2750,22 +2759,22 @@
     </row>
     <row r="34" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="E34" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F34" s="2" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="G34" s="2" t="s">
         <v>13</v>
@@ -2773,22 +2782,22 @@
     </row>
     <row r="35" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="E35" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F35" s="2" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="G35" s="2" t="s">
         <v>13</v>
@@ -2796,22 +2805,22 @@
     </row>
     <row r="36" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="E36" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F36" s="2" t="s">
-        <v>177</v>
+        <v>58</v>
       </c>
       <c r="G36" s="2" t="s">
         <v>13</v>
@@ -2819,22 +2828,22 @@
     </row>
     <row r="37" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="E37" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F37" s="2" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="G37" s="2" t="s">
         <v>13</v>
@@ -2842,22 +2851,22 @@
     </row>
     <row r="38" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="E38" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F38" s="2" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="G38" s="2" t="s">
         <v>13</v>
@@ -2865,22 +2874,22 @@
     </row>
     <row r="39" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="E39" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F39" s="2" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="G39" s="2" t="s">
         <v>13</v>
@@ -2888,22 +2897,22 @@
     </row>
     <row r="40" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="E40" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F40" s="2" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="G40" s="2" t="s">
         <v>13</v>
@@ -2911,22 +2920,22 @@
     </row>
     <row r="41" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="D41" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="E41" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F41" s="2" t="s">
         <v>190</v>
-      </c>
-      <c r="B41" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="C41" s="2" t="s">
-        <v>191</v>
-      </c>
-      <c r="D41" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="E41" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F41" s="2" t="s">
-        <v>192</v>
       </c>
       <c r="G41" s="2" t="s">
         <v>13</v>
@@ -2992,7 +3001,7 @@
         <v>11</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>52</v>
+        <v>196</v>
       </c>
       <c r="G2" s="2" t="s">
         <v>13</v>
@@ -3000,13 +3009,13 @@
     </row>
     <row r="3" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>194</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>194</v>
@@ -3015,7 +3024,7 @@
         <v>11</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="G3" s="2" t="s">
         <v>13</v>
@@ -3023,13 +3032,13 @@
     </row>
     <row r="4" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>194</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>194</v>
@@ -3038,7 +3047,7 @@
         <v>11</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
       <c r="G4" s="2" t="s">
         <v>13</v>
@@ -3046,13 +3055,13 @@
     </row>
     <row r="5" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>194</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>194</v>
@@ -3061,7 +3070,7 @@
         <v>11</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>198</v>
+        <v>205</v>
       </c>
       <c r="G5" s="2" t="s">
         <v>13</v>
@@ -3069,13 +3078,13 @@
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>194</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>194</v>
@@ -3084,7 +3093,7 @@
         <v>11</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="G6" s="2" t="s">
         <v>13</v>
@@ -3092,13 +3101,13 @@
     </row>
     <row r="7" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>194</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>194</v>
@@ -3107,7 +3116,7 @@
         <v>11</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>33</v>
+        <v>210</v>
       </c>
       <c r="G7" s="2" t="s">
         <v>13</v>
@@ -3115,13 +3124,13 @@
     </row>
     <row r="8" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>207</v>
+        <v>211</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>194</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>208</v>
+        <v>212</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>194</v>
@@ -3130,7 +3139,7 @@
         <v>11</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>198</v>
+        <v>205</v>
       </c>
       <c r="G8" s="2" t="s">
         <v>13</v>
@@ -3138,13 +3147,13 @@
     </row>
     <row r="9" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>194</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>210</v>
+        <v>214</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>194</v>
@@ -3153,7 +3162,7 @@
         <v>11</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>198</v>
+        <v>205</v>
       </c>
       <c r="G9" s="2" t="s">
         <v>13</v>
@@ -3161,13 +3170,13 @@
     </row>
     <row r="10" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>194</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>212</v>
+        <v>216</v>
       </c>
       <c r="D10" s="2" t="s">
         <v>194</v>
@@ -3176,7 +3185,7 @@
         <v>11</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>213</v>
+        <v>199</v>
       </c>
       <c r="G10" s="2" t="s">
         <v>13</v>
@@ -3184,13 +3193,13 @@
     </row>
     <row r="11" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="B11" s="2" t="s">
         <v>194</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="D11" s="2" t="s">
         <v>194</v>
@@ -3199,7 +3208,7 @@
         <v>11</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>198</v>
+        <v>205</v>
       </c>
       <c r="G11" s="2" t="s">
         <v>13</v>
@@ -3207,13 +3216,13 @@
     </row>
     <row r="12" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="B12" s="2" t="s">
         <v>194</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="D12" s="2" t="s">
         <v>194</v>
@@ -3222,7 +3231,7 @@
         <v>11</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>198</v>
+        <v>205</v>
       </c>
       <c r="G12" s="2" t="s">
         <v>13</v>
@@ -3230,13 +3239,13 @@
     </row>
     <row r="13" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
       <c r="B13" s="2" t="s">
         <v>194</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="D13" s="2" t="s">
         <v>194</v>
@@ -3245,7 +3254,7 @@
         <v>11</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="G13" s="2" t="s">
         <v>13</v>
@@ -3253,13 +3262,13 @@
     </row>
     <row r="14" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="B14" s="2" t="s">
         <v>194</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="D14" s="2" t="s">
         <v>194</v>
@@ -3268,7 +3277,7 @@
         <v>11</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="G14" s="2" t="s">
         <v>13</v>
@@ -3276,13 +3285,13 @@
     </row>
     <row r="15" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="B15" s="2" t="s">
         <v>194</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="D15" s="2" t="s">
         <v>194</v>
@@ -3291,7 +3300,7 @@
         <v>11</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="G15" s="2" t="s">
         <v>13</v>
@@ -3299,13 +3308,13 @@
     </row>
     <row r="16" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="B16" s="2" t="s">
         <v>194</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="D16" s="2" t="s">
         <v>194</v>
@@ -3314,7 +3323,7 @@
         <v>11</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>198</v>
+        <v>205</v>
       </c>
       <c r="G16" s="2" t="s">
         <v>13</v>
@@ -3322,13 +3331,13 @@
     </row>
     <row r="17" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="B17" s="2" t="s">
         <v>194</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="D17" s="2" t="s">
         <v>194</v>
@@ -3337,7 +3346,7 @@
         <v>11</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>198</v>
+        <v>205</v>
       </c>
       <c r="G17" s="2" t="s">
         <v>13</v>
@@ -3345,13 +3354,13 @@
     </row>
     <row r="18" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="B18" s="2" t="s">
         <v>194</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="D18" s="2" t="s">
         <v>194</v>
@@ -3360,7 +3369,7 @@
         <v>11</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>198</v>
+        <v>205</v>
       </c>
       <c r="G18" s="2" t="s">
         <v>13</v>
@@ -3368,13 +3377,13 @@
     </row>
     <row r="19" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
       <c r="B19" s="2" t="s">
         <v>194</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="D19" s="2" t="s">
         <v>194</v>
@@ -3383,7 +3392,7 @@
         <v>11</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>198</v>
+        <v>205</v>
       </c>
       <c r="G19" s="2" t="s">
         <v>13</v>
@@ -3391,13 +3400,13 @@
     </row>
     <row r="20" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="B20" s="2" t="s">
         <v>194</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="D20" s="2" t="s">
         <v>194</v>
@@ -3406,7 +3415,7 @@
         <v>11</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>198</v>
+        <v>205</v>
       </c>
       <c r="G20" s="2" t="s">
         <v>13</v>
@@ -3414,13 +3423,13 @@
     </row>
     <row r="21" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="B21" s="2" t="s">
         <v>194</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
       <c r="D21" s="2" t="s">
         <v>194</v>
@@ -3429,7 +3438,7 @@
         <v>11</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>198</v>
+        <v>205</v>
       </c>
       <c r="G21" s="2" t="s">
         <v>13</v>
@@ -3480,22 +3489,22 @@
     </row>
     <row r="2" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="E2" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
       <c r="G2" s="2" t="s">
         <v>13</v>
@@ -3503,22 +3512,22 @@
     </row>
     <row r="3" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="B3" s="2" t="s">
         <v>240</v>
       </c>
-      <c r="B3" s="2" t="s">
-        <v>237</v>
-      </c>
       <c r="C3" s="2" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="E3" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>55</v>
+        <v>82</v>
       </c>
       <c r="G3" s="2" t="s">
         <v>13</v>
@@ -3526,22 +3535,22 @@
     </row>
     <row r="4" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="E4" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
       <c r="G4" s="2" t="s">
         <v>13</v>
@@ -3549,22 +3558,22 @@
     </row>
     <row r="5" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="E5" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>198</v>
+        <v>205</v>
       </c>
       <c r="G5" s="2" t="s">
         <v>13</v>
@@ -3572,22 +3581,22 @@
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="E6" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="G6" s="2" t="s">
         <v>13</v>
@@ -3595,22 +3604,22 @@
     </row>
     <row r="7" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="E7" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>252</v>
+        <v>64</v>
       </c>
       <c r="G7" s="2" t="s">
         <v>13</v>
@@ -3618,22 +3627,22 @@
     </row>
     <row r="8" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="E8" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="G8" s="2" t="s">
         <v>13</v>
@@ -3641,22 +3650,22 @@
     </row>
     <row r="9" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="E9" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>33</v>
+        <v>260</v>
       </c>
       <c r="G9" s="2" t="s">
         <v>13</v>
@@ -3664,22 +3673,22 @@
     </row>
     <row r="10" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>260</v>
+        <v>263</v>
       </c>
       <c r="E10" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="G10" s="2" t="s">
         <v>13</v>
@@ -3687,22 +3696,22 @@
     </row>
     <row r="11" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>262</v>
+        <v>265</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="C11" s="2" t="s">
+        <v>266</v>
+      </c>
+      <c r="D11" s="2" t="s">
         <v>263</v>
       </c>
-      <c r="D11" s="2" t="s">
-        <v>260</v>
-      </c>
       <c r="E11" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>198</v>
+        <v>205</v>
       </c>
       <c r="G11" s="2" t="s">
         <v>13</v>
@@ -3710,22 +3719,22 @@
     </row>
     <row r="12" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>264</v>
+        <v>267</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>265</v>
+        <v>268</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="E12" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>266</v>
+        <v>269</v>
       </c>
       <c r="G12" s="2" t="s">
         <v>13</v>
@@ -3733,22 +3742,22 @@
     </row>
     <row r="13" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>268</v>
+        <v>271</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="E13" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>269</v>
+        <v>272</v>
       </c>
       <c r="G13" s="2" t="s">
         <v>13</v>
@@ -3756,22 +3765,22 @@
     </row>
     <row r="14" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>271</v>
+        <v>274</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="E14" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>198</v>
+        <v>205</v>
       </c>
       <c r="G14" s="2" t="s">
         <v>13</v>
@@ -3779,22 +3788,22 @@
     </row>
     <row r="15" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>272</v>
+        <v>275</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>273</v>
+        <v>276</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="E15" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
       <c r="G15" s="2" t="s">
         <v>13</v>
@@ -3802,22 +3811,22 @@
     </row>
     <row r="16" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>275</v>
+        <v>278</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>260</v>
+        <v>263</v>
       </c>
       <c r="E16" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>277</v>
+        <v>280</v>
       </c>
       <c r="G16" s="2" t="s">
         <v>13</v>
@@ -3868,22 +3877,22 @@
     </row>
     <row r="2" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>280</v>
+        <v>283</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>281</v>
+        <v>284</v>
       </c>
       <c r="E2" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
       <c r="G2" s="2" t="s">
         <v>13</v>
@@ -3891,22 +3900,22 @@
     </row>
     <row r="3" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>283</v>
+        <v>286</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
       <c r="C3" s="2" t="s">
+        <v>287</v>
+      </c>
+      <c r="D3" s="2" t="s">
         <v>284</v>
       </c>
-      <c r="D3" s="2" t="s">
-        <v>281</v>
-      </c>
       <c r="E3" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>285</v>
+        <v>288</v>
       </c>
       <c r="G3" s="2" t="s">
         <v>13</v>
@@ -3914,22 +3923,22 @@
     </row>
     <row r="4" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>286</v>
+        <v>289</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
       <c r="E4" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>198</v>
+        <v>205</v>
       </c>
       <c r="G4" s="2" t="s">
         <v>13</v>
@@ -3937,22 +3946,22 @@
     </row>
     <row r="5" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
       <c r="E5" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
       <c r="G5" s="2" t="s">
         <v>13</v>
@@ -3960,22 +3969,22 @@
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>291</v>
+        <v>294</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>292</v>
+        <v>295</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>260</v>
+        <v>263</v>
       </c>
       <c r="E6" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>198</v>
+        <v>205</v>
       </c>
       <c r="G6" s="2" t="s">
         <v>13</v>
@@ -3983,22 +3992,22 @@
     </row>
     <row r="7" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>293</v>
+        <v>296</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>294</v>
+        <v>297</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
       <c r="E7" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="G7" s="2" t="s">
         <v>13</v>
@@ -4006,22 +4015,22 @@
     </row>
     <row r="8" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>296</v>
+        <v>299</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>297</v>
+        <v>300</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>281</v>
+        <v>284</v>
       </c>
       <c r="E8" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
       <c r="G8" s="2" t="s">
         <v>13</v>
@@ -4029,22 +4038,22 @@
     </row>
     <row r="9" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>299</v>
+        <v>302</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>300</v>
+        <v>303</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>281</v>
+        <v>284</v>
       </c>
       <c r="E9" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>301</v>
+        <v>22</v>
       </c>
       <c r="G9" s="2" t="s">
         <v>13</v>
@@ -4052,22 +4061,22 @@
     </row>
     <row r="10" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>281</v>
+        <v>284</v>
       </c>
       <c r="E10" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>134</v>
+        <v>306</v>
       </c>
       <c r="G10" s="2" t="s">
         <v>13</v>
@@ -4075,22 +4084,22 @@
     </row>
     <row r="11" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>304</v>
+        <v>307</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>305</v>
+        <v>308</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
       <c r="E11" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>198</v>
+        <v>205</v>
       </c>
       <c r="G11" s="2" t="s">
         <v>13</v>

</xml_diff>

<commit_message>
Configure CI/CD pipeline to automatically deploy build to GitHub Pages
</commit_message>
<xml_diff>
--- a/tests/reports/Test_Analysis_Report.xlsx
+++ b/tests/reports/Test_Analysis_Report.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="805" uniqueCount="309">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="805" uniqueCount="314">
   <si>
     <t>Test ID</t>
   </si>
@@ -56,7 +56,7 @@
     <t>Passed</t>
   </si>
   <si>
-    <t>2239ms</t>
+    <t>1816ms</t>
   </si>
   <si>
     <t>Assertion passed successfully</t>
@@ -68,7 +68,7 @@
     <t>Verify brand name PayBuddy header exists</t>
   </si>
   <si>
-    <t>322ms</t>
+    <t>88ms</t>
   </si>
   <si>
     <t>TC-WEB-UI-003</t>
@@ -77,7 +77,7 @@
     <t>Verify form email input label</t>
   </si>
   <si>
-    <t>53ms</t>
+    <t>50ms</t>
   </si>
   <si>
     <t>TC-WEB-UI-004</t>
@@ -86,579 +86,588 @@
     <t>Verify form password input label</t>
   </si>
   <si>
+    <t>37ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-005</t>
+  </si>
+  <si>
+    <t>Verify Sign In button is present</t>
+  </si>
+  <si>
     <t>54ms</t>
   </si>
   <si>
-    <t>TC-WEB-UI-005</t>
-  </si>
-  <si>
-    <t>Verify Sign In button is present</t>
-  </si>
-  <si>
-    <t>44ms</t>
-  </si>
-  <si>
     <t>TC-WEB-UI-006</t>
   </si>
   <si>
     <t>Verify secure access footer notice is present</t>
   </si>
   <si>
+    <t>30ms</t>
+  </si>
+  <si>
     <t>TC-WEB-UI-007</t>
   </si>
   <si>
     <t>Verify branding subtitle text exists</t>
   </si>
   <si>
+    <t>49ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-008</t>
+  </si>
+  <si>
+    <t>Verify email input field placeholder</t>
+  </si>
+  <si>
+    <t>48ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-009</t>
+  </si>
+  <si>
+    <t>Verify password input field placeholder</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-010</t>
+  </si>
+  <si>
+    <t>Verify font family CSS on headers</t>
+  </si>
+  <si>
     <t>52ms</t>
   </si>
   <si>
-    <t>TC-WEB-UI-008</t>
-  </si>
-  <si>
-    <t>Verify email input field placeholder</t>
-  </si>
-  <si>
-    <t>49ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UI-009</t>
-  </si>
-  <si>
-    <t>Verify password input field placeholder</t>
+    <t>TC-WEB-UI-011</t>
+  </si>
+  <si>
+    <t>Verify primary brand color on buttons</t>
+  </si>
+  <si>
+    <t>46ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-012</t>
+  </si>
+  <si>
+    <t>Verify centered block layout</t>
+  </si>
+  <si>
+    <t>56ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-013</t>
+  </si>
+  <si>
+    <t>Verify responsive structure at mobile width 360px</t>
+  </si>
+  <si>
+    <t>935ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-014</t>
+  </si>
+  <si>
+    <t>Verify responsive structure at tablet width 768px</t>
+  </si>
+  <si>
+    <t>912ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-015</t>
+  </si>
+  <si>
+    <t>Restore browser window maximization state</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-016</t>
+  </si>
+  <si>
+    <t>Verify HTML tag specification for email input</t>
+  </si>
+  <si>
+    <t>68ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-017</t>
+  </si>
+  <si>
+    <t>Verify HTML tag specification for password input</t>
+  </si>
+  <si>
+    <t>62ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-018</t>
+  </si>
+  <si>
+    <t>Verify card wrapper styles (border-radius)</t>
+  </si>
+  <si>
+    <t>35ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-019</t>
+  </si>
+  <si>
+    <t>Verify background styling matches design spec</t>
+  </si>
+  <si>
+    <t>73ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-020</t>
+  </si>
+  <si>
+    <t>Verify focus state click handler does not crash</t>
+  </si>
+  <si>
+    <t>152ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-021</t>
+  </si>
+  <si>
+    <t>Verify top-level container viewport classes</t>
+  </si>
+  <si>
+    <t>45ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-022</t>
+  </si>
+  <si>
+    <t>Verify branding and form division layout margins</t>
+  </si>
+  <si>
+    <t>40ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-023</t>
+  </si>
+  <si>
+    <t>Verify clear textual contrast for reader accessibility</t>
+  </si>
+  <si>
+    <t>38ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-024</t>
+  </si>
+  <si>
+    <t>Verify page scales properly without layout clipping</t>
+  </si>
+  <si>
+    <t>42ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UI-025</t>
+  </si>
+  <si>
+    <t>Verify smooth interactive transitions on button inputs</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-001</t>
+  </si>
+  <si>
+    <t>Functional</t>
+  </si>
+  <si>
+    <t>Verify invalid login rejection message</t>
+  </si>
+  <si>
+    <t>2196ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-002</t>
+  </si>
+  <si>
+    <t>Verify rejection of nonexistent email</t>
+  </si>
+  <si>
+    <t>1319ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-003</t>
+  </si>
+  <si>
+    <t>Verify successful login with valid credentials redirects to Dashboard</t>
+  </si>
+  <si>
+    <t>2462ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-004</t>
+  </si>
+  <si>
+    <t>Verify dashboard displays Total Customers count</t>
+  </si>
+  <si>
+    <t>531ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-005</t>
+  </si>
+  <si>
+    <t>Verify dashboard displays Active Sales count</t>
+  </si>
+  <si>
+    <t>78ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-006</t>
+  </si>
+  <si>
+    <t>Verify dashboard displays Pending Installments count</t>
+  </si>
+  <si>
+    <t>5121ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-007</t>
+  </si>
+  <si>
+    <t>Verify dashboard displays Today's Due count</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-008</t>
+  </si>
+  <si>
+    <t>Verify dashboard displays Outstanding Balance amount</t>
+  </si>
+  <si>
+    <t>29ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-009</t>
+  </si>
+  <si>
+    <t>Navigate to customers page and verify header</t>
+  </si>
+  <si>
+    <t>254ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-010</t>
+  </si>
+  <si>
+    <t>Verify add new customer input inputs are present</t>
+  </si>
+  <si>
+    <t>69ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-011</t>
+  </si>
+  <si>
+    <t>Verify customer creation and entry addition to table</t>
+  </si>
+  <si>
+    <t>3065ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-012</t>
+  </si>
+  <si>
+    <t>Verify presence of seeded customer</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-013</t>
+  </si>
+  <si>
+    <t>Navigate to specific customer profile page</t>
+  </si>
+  <si>
+    <t>1957ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-014</t>
+  </si>
+  <si>
+    <t>Verify phone number exists on profile detail bar</t>
   </si>
   <si>
     <t>51ms</t>
   </si>
   <si>
-    <t>TC-WEB-UI-010</t>
-  </si>
-  <si>
-    <t>Verify font family CSS on headers</t>
-  </si>
-  <si>
-    <t>TC-WEB-UI-011</t>
-  </si>
-  <si>
-    <t>Verify primary brand color on buttons</t>
-  </si>
-  <si>
-    <t>47ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UI-012</t>
-  </si>
-  <si>
-    <t>Verify centered block layout</t>
-  </si>
-  <si>
-    <t>TC-WEB-UI-013</t>
-  </si>
-  <si>
-    <t>Verify responsive structure at mobile width 360px</t>
-  </si>
-  <si>
-    <t>945ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UI-014</t>
-  </si>
-  <si>
-    <t>Verify responsive structure at tablet width 768px</t>
-  </si>
-  <si>
-    <t>942ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UI-015</t>
-  </si>
-  <si>
-    <t>Restore browser window maximization state</t>
-  </si>
-  <si>
-    <t>59ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UI-016</t>
-  </si>
-  <si>
-    <t>Verify HTML tag specification for email input</t>
-  </si>
-  <si>
-    <t>67ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UI-017</t>
-  </si>
-  <si>
-    <t>Verify HTML tag specification for password input</t>
-  </si>
-  <si>
-    <t>50ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UI-018</t>
-  </si>
-  <si>
-    <t>Verify card wrapper styles (border-radius)</t>
-  </si>
-  <si>
-    <t>110ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UI-019</t>
-  </si>
-  <si>
-    <t>Verify background styling matches design spec</t>
-  </si>
-  <si>
-    <t>45ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UI-020</t>
-  </si>
-  <si>
-    <t>Verify focus state click handler does not crash</t>
-  </si>
-  <si>
-    <t>156ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UI-021</t>
-  </si>
-  <si>
-    <t>Verify top-level container viewport classes</t>
-  </si>
-  <si>
-    <t>64ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UI-022</t>
-  </si>
-  <si>
-    <t>Verify branding and form division layout margins</t>
-  </si>
-  <si>
-    <t>61ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UI-023</t>
-  </si>
-  <si>
-    <t>Verify clear textual contrast for reader accessibility</t>
-  </si>
-  <si>
-    <t>56ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UI-024</t>
-  </si>
-  <si>
-    <t>Verify page scales properly without layout clipping</t>
-  </si>
-  <si>
-    <t>38ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UI-025</t>
-  </si>
-  <si>
-    <t>Verify smooth interactive transitions on button inputs</t>
+    <t>TC-WEB-FUNC-015</t>
+  </si>
+  <si>
+    <t>Verify Total Amount financial card is 1000 INR</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-016</t>
+  </si>
+  <si>
+    <t>Verify Paid Amount financial card is 0 INR</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-017</t>
+  </si>
+  <si>
+    <t>Verify Outstanding Balance financial card is 1000 INR</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-018</t>
+  </si>
+  <si>
+    <t>Verify E2E Test Item pending sale is loaded in sales list</t>
+  </si>
+  <si>
+    <t>58ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-019</t>
+  </si>
+  <si>
+    <t>Verify redirect to record payment page</t>
+  </si>
+  <si>
+    <t>1139ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-020</t>
+  </si>
+  <si>
+    <t>Verify remaining balance display match before payment</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-021</t>
+  </si>
+  <si>
+    <t>Record payment E2E execution and redirection validation</t>
+  </si>
+  <si>
+    <t>3532ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-022</t>
+  </si>
+  <si>
+    <t>Verify Outstanding Balance updates to 800 INR in customer card</t>
+  </si>
+  <si>
+    <t>1170ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-023</t>
+  </si>
+  <si>
+    <t>Verify Paid Amount updates to 200 INR in customer card</t>
   </si>
   <si>
     <t>33ms</t>
   </si>
   <si>
-    <t>TC-WEB-FUNC-001</t>
-  </si>
-  <si>
-    <t>Functional</t>
-  </si>
-  <si>
-    <t>Verify invalid login rejection message</t>
-  </si>
-  <si>
-    <t>1912ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-002</t>
-  </si>
-  <si>
-    <t>Verify rejection of nonexistent email</t>
-  </si>
-  <si>
-    <t>1667ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-003</t>
-  </si>
-  <si>
-    <t>Verify successful login with valid credentials redirects to Dashboard</t>
-  </si>
-  <si>
-    <t>2080ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-004</t>
-  </si>
-  <si>
-    <t>Verify dashboard displays Total Customers count</t>
-  </si>
-  <si>
-    <t>281ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-005</t>
-  </si>
-  <si>
-    <t>Verify dashboard displays Active Sales count</t>
-  </si>
-  <si>
-    <t>60ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-006</t>
-  </si>
-  <si>
-    <t>Verify dashboard displays Pending Installments count</t>
-  </si>
-  <si>
-    <t>35ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-007</t>
-  </si>
-  <si>
-    <t>Verify dashboard displays Today's Due count</t>
-  </si>
-  <si>
-    <t>36ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-008</t>
-  </si>
-  <si>
-    <t>Verify dashboard displays Outstanding Balance amount</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-009</t>
-  </si>
-  <si>
-    <t>Navigate to customers page and verify header</t>
-  </si>
-  <si>
-    <t>393ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-010</t>
-  </si>
-  <si>
-    <t>Verify add new customer input inputs are present</t>
-  </si>
-  <si>
-    <t>57ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-011</t>
-  </si>
-  <si>
-    <t>Verify customer creation and entry addition to table</t>
-  </si>
-  <si>
-    <t>3044ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-012</t>
-  </si>
-  <si>
-    <t>Verify presence of seeded customer</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-013</t>
-  </si>
-  <si>
-    <t>Navigate to specific customer profile page</t>
-  </si>
-  <si>
-    <t>1425ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-014</t>
-  </si>
-  <si>
-    <t>Verify phone number exists on profile detail bar</t>
+    <t>TC-WEB-FUNC-024</t>
+  </si>
+  <si>
+    <t>Verify recorded payment entry list matches mode UPI</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-025</t>
+  </si>
+  <si>
+    <t>Verify sales management index loads properly</t>
+  </si>
+  <si>
+    <t>882ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-026</t>
+  </si>
+  <si>
+    <t>Verify sales search filter works properly</t>
+  </si>
+  <si>
+    <t>843ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-027</t>
+  </si>
+  <si>
+    <t>Navigate to Create New Sale form</t>
+  </si>
+  <si>
+    <t>927ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-028</t>
+  </si>
+  <si>
+    <t>Verify total amount computed automatically (2 x 500 = 1000)</t>
+  </si>
+  <si>
+    <t>673ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-029</t>
+  </si>
+  <si>
+    <t>Create sale and verify redirect back to sales table</t>
+  </si>
+  <si>
+    <t>497ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-030</t>
+  </si>
+  <si>
+    <t>Verify Payments page path and title</t>
+  </si>
+  <si>
+    <t>891ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-031</t>
+  </si>
+  <si>
+    <t>Verify E2E transaction exists in master list</t>
+  </si>
+  <si>
+    <t>66ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-032</t>
+  </si>
+  <si>
+    <t>Verify Ledger Book page loads</t>
+  </si>
+  <si>
+    <t>874ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-033</t>
+  </si>
+  <si>
+    <t>Verify ledger records contain client name</t>
+  </si>
+  <si>
+    <t>98ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-034</t>
+  </si>
+  <si>
+    <t>Verify Installments page title</t>
+  </si>
+  <si>
+    <t>855ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-035</t>
+  </si>
+  <si>
+    <t>Verify customer details exist on installment board</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-036</t>
+  </si>
+  <si>
+    <t>Verify direct Dashboard URL redirect</t>
+  </si>
+  <si>
+    <t>148ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-037</t>
+  </si>
+  <si>
+    <t>Verify customer data updates dynamically on UI edit</t>
+  </si>
+  <si>
+    <t>4889ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-038</t>
+  </si>
+  <si>
+    <t>Verify logout route terminates session and redirects to sign in</t>
+  </si>
+  <si>
+    <t>5357ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-039</t>
+  </si>
+  <si>
+    <t>Verify unauthorized dashboard access redirects to login</t>
+  </si>
+  <si>
+    <t>2201ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-FUNC-040</t>
+  </si>
+  <si>
+    <t>Verify unauthorized customer details access redirects to login</t>
+  </si>
+  <si>
+    <t>2166ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UNIT-001</t>
+  </si>
+  <si>
+    <t>Unit</t>
+  </si>
+  <si>
+    <t>Test formatCurrency formatting positive amount</t>
+  </si>
+  <si>
+    <t>76ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UNIT-002</t>
+  </si>
+  <si>
+    <t>Test formatCurrency formatting zero amount</t>
+  </si>
+  <si>
+    <t>2ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UNIT-003</t>
+  </si>
+  <si>
+    <t>Test formatCurrency formatting negative amount</t>
+  </si>
+  <si>
+    <t>1ms</t>
+  </si>
+  <si>
+    <t>TC-WEB-UNIT-004</t>
+  </si>
+  <si>
+    <t>Test formatCurrency formatting large millions scale amount</t>
+  </si>
+  <si>
+    <t>TC-WEB-UNIT-005</t>
+  </si>
+  <si>
+    <t>Test formatCurrency decimal rounding functionality</t>
+  </si>
+  <si>
+    <t>TC-WEB-UNIT-006</t>
+  </si>
+  <si>
+    <t>Test formatDate string matching date details</t>
   </si>
   <si>
     <t>39ms</t>
   </si>
   <si>
-    <t>TC-WEB-FUNC-015</t>
-  </si>
-  <si>
-    <t>Verify Total Amount financial card is 1000 INR</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-016</t>
-  </si>
-  <si>
-    <t>Verify Paid Amount financial card is 0 INR</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-017</t>
-  </si>
-  <si>
-    <t>Verify Outstanding Balance financial card is 1000 INR</t>
-  </si>
-  <si>
-    <t>41ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-018</t>
-  </si>
-  <si>
-    <t>Verify E2E Test Item pending sale is loaded in sales list</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-019</t>
-  </si>
-  <si>
-    <t>Verify redirect to record payment page</t>
-  </si>
-  <si>
-    <t>1096ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-020</t>
-  </si>
-  <si>
-    <t>Verify remaining balance display match before payment</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-021</t>
-  </si>
-  <si>
-    <t>Record payment E2E execution and redirection validation</t>
-  </si>
-  <si>
-    <t>3240ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-022</t>
-  </si>
-  <si>
-    <t>Verify Outstanding Balance updates to 800 INR in customer card</t>
-  </si>
-  <si>
-    <t>1228ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-023</t>
-  </si>
-  <si>
-    <t>Verify Paid Amount updates to 200 INR in customer card</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-024</t>
-  </si>
-  <si>
-    <t>Verify recorded payment entry list matches mode UPI</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-025</t>
-  </si>
-  <si>
-    <t>Verify sales management index loads properly</t>
-  </si>
-  <si>
-    <t>728ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-026</t>
-  </si>
-  <si>
-    <t>Verify sales search filter works properly</t>
-  </si>
-  <si>
-    <t>794ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-027</t>
-  </si>
-  <si>
-    <t>Navigate to Create New Sale form</t>
-  </si>
-  <si>
-    <t>666ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-028</t>
-  </si>
-  <si>
-    <t>Verify total amount computed automatically (2 x 500 = 1000)</t>
-  </si>
-  <si>
-    <t>655ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-029</t>
-  </si>
-  <si>
-    <t>Create sale and verify redirect back to sales table</t>
-  </si>
-  <si>
-    <t>500ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-030</t>
-  </si>
-  <si>
-    <t>Verify Payments page path and title</t>
-  </si>
-  <si>
-    <t>662ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-031</t>
-  </si>
-  <si>
-    <t>Verify E2E transaction exists in master list</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-032</t>
-  </si>
-  <si>
-    <t>Verify Ledger Book page loads</t>
-  </si>
-  <si>
-    <t>743ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-033</t>
-  </si>
-  <si>
-    <t>Verify ledger records contain client name</t>
-  </si>
-  <si>
-    <t>71ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-034</t>
-  </si>
-  <si>
-    <t>Verify Installments page title</t>
-  </si>
-  <si>
-    <t>648ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-035</t>
-  </si>
-  <si>
-    <t>Verify customer details exist on installment board</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-036</t>
-  </si>
-  <si>
-    <t>Verify direct Dashboard URL redirect</t>
-  </si>
-  <si>
-    <t>123ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-037</t>
-  </si>
-  <si>
-    <t>Verify customer data updates dynamically on UI edit</t>
-  </si>
-  <si>
-    <t>4674ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-038</t>
-  </si>
-  <si>
-    <t>Verify logout route terminates session and redirects to sign in</t>
-  </si>
-  <si>
-    <t>809ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-039</t>
-  </si>
-  <si>
-    <t>Verify unauthorized dashboard access redirects to login</t>
-  </si>
-  <si>
-    <t>2153ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-FUNC-040</t>
-  </si>
-  <si>
-    <t>Verify unauthorized customer details access redirects to login</t>
-  </si>
-  <si>
-    <t>TC-WEB-UNIT-001</t>
-  </si>
-  <si>
-    <t>Unit</t>
-  </si>
-  <si>
-    <t>Test formatCurrency formatting positive amount</t>
-  </si>
-  <si>
-    <t>79ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UNIT-002</t>
-  </si>
-  <si>
-    <t>Test formatCurrency formatting zero amount</t>
-  </si>
-  <si>
-    <t>1ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UNIT-003</t>
-  </si>
-  <si>
-    <t>Test formatCurrency formatting negative amount</t>
-  </si>
-  <si>
-    <t>2ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UNIT-004</t>
-  </si>
-  <si>
-    <t>Test formatCurrency formatting large millions scale amount</t>
+    <t>TC-WEB-UNIT-007</t>
+  </si>
+  <si>
+    <t>Test formatDate fallback for null values</t>
   </si>
   <si>
     <t>0ms</t>
   </si>
   <si>
-    <t>TC-WEB-UNIT-005</t>
-  </si>
-  <si>
-    <t>Test formatCurrency decimal rounding functionality</t>
-  </si>
-  <si>
-    <t>TC-WEB-UNIT-006</t>
-  </si>
-  <si>
-    <t>Test formatDate string matching date details</t>
-  </si>
-  <si>
-    <t>22ms</t>
-  </si>
-  <si>
-    <t>TC-WEB-UNIT-007</t>
-  </si>
-  <si>
-    <t>Test formatDate fallback for null values</t>
-  </si>
-  <si>
     <t>TC-WEB-UNIT-008</t>
   </si>
   <si>
@@ -746,7 +755,7 @@
     <t>Verify email required constraint is enabled on form</t>
   </si>
   <si>
-    <t>191ms</t>
+    <t>5249ms</t>
   </si>
   <si>
     <t>TC-WEB-VAL-002</t>
@@ -755,13 +764,16 @@
     <t>Verify password required constraint is enabled on form</t>
   </si>
   <si>
+    <t>5116ms</t>
+  </si>
+  <si>
     <t>TC-WEB-VAL-003</t>
   </si>
   <si>
     <t>Verify browser client blocks submissions for invalid email inputs</t>
   </si>
   <si>
-    <t>253ms</t>
+    <t>5132ms</t>
   </si>
   <si>
     <t>TC-WEB-VAL-004</t>
@@ -776,7 +788,7 @@
     <t>Verify customer creation form prevents empty submit</t>
   </si>
   <si>
-    <t>3184ms</t>
+    <t>10165ms</t>
   </si>
   <si>
     <t>TC-WEB-VAL-006</t>
@@ -785,13 +797,16 @@
     <t>Verify phone input uses tel semantic element type</t>
   </si>
   <si>
+    <t>5094ms</t>
+  </si>
+  <si>
     <t>TC-WEB-VAL-007</t>
   </si>
   <si>
     <t>Verify sale quantity requires positive minimum value (&gt; 0)</t>
   </si>
   <si>
-    <t>624ms</t>
+    <t>887ms</t>
   </si>
   <si>
     <t>TC-WEB-VAL-008</t>
@@ -800,9 +815,6 @@
     <t>Verify unit price input restricts negative numbers</t>
   </si>
   <si>
-    <t>37ms</t>
-  </si>
-  <si>
     <t>TC-WEB-VAL-009</t>
   </si>
   <si>
@@ -812,7 +824,7 @@
     <t>Security</t>
   </si>
   <si>
-    <t>2472ms</t>
+    <t>2578ms</t>
   </si>
   <si>
     <t>TC-WEB-VAL-010</t>
@@ -827,7 +839,7 @@
     <t>Verify error prevents overpayment collections</t>
   </si>
   <si>
-    <t>1936ms</t>
+    <t>2374ms</t>
   </si>
   <si>
     <t>TC-WEB-VAL-012</t>
@@ -836,7 +848,7 @@
     <t>Verify collection input restricts 0 value submissions</t>
   </si>
   <si>
-    <t>1437ms</t>
+    <t>1336ms</t>
   </si>
   <si>
     <t>TC-WEB-VAL-013</t>
@@ -851,7 +863,7 @@
     <t>Verify wildcard URLs redirect to main route base</t>
   </si>
   <si>
-    <t>2128ms</t>
+    <t>2146ms</t>
   </si>
   <si>
     <t>TC-WEB-VAL-015</t>
@@ -860,7 +872,7 @@
     <t>Verify HTML password hidden mask attribute config</t>
   </si>
   <si>
-    <t>844ms</t>
+    <t>5313ms</t>
   </si>
   <si>
     <t>TC-WEB-DEP-001</t>
@@ -875,7 +887,7 @@
     <t>Performance</t>
   </si>
   <si>
-    <t>152ms</t>
+    <t>158ms</t>
   </si>
   <si>
     <t>TC-WEB-DEP-002</t>
@@ -884,7 +896,7 @@
     <t>Verify full render transition load time under limit</t>
   </si>
   <si>
-    <t>1451ms</t>
+    <t>10151ms</t>
   </si>
   <si>
     <t>TC-WEB-DEP-003</t>
@@ -899,7 +911,7 @@
     <t>Verify favicon.ico endpoint yields clean HTTP status</t>
   </si>
   <si>
-    <t>127ms</t>
+    <t>120ms</t>
   </si>
   <si>
     <t>TC-WEB-DEP-005</t>
@@ -914,7 +926,7 @@
     <t>Verify head links contain manifest registration details</t>
   </si>
   <si>
-    <t>184ms</t>
+    <t>183ms</t>
   </si>
   <si>
     <t>TC-WEB-DEP-007</t>
@@ -923,13 +935,16 @@
     <t>Verify console logs have no severe exceptions during login page session</t>
   </si>
   <si>
-    <t>8ms</t>
+    <t>9ms</t>
   </si>
   <si>
     <t>TC-WEB-DEP-008</t>
   </si>
   <si>
     <t>Verify standard responsive layouts align horizontally</t>
+  </si>
+  <si>
+    <t>82ms</t>
   </si>
   <si>
     <t>TC-WEB-DEP-009</t>
@@ -1535,7 +1550,7 @@
         <v>11</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="G7" s="2" t="s">
         <v>13</v>
@@ -1543,13 +1558,13 @@
     </row>
     <row r="8" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>10</v>
@@ -1558,7 +1573,7 @@
         <v>11</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G8" s="2" t="s">
         <v>13</v>
@@ -1566,13 +1581,13 @@
     </row>
     <row r="9" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>10</v>
@@ -1581,7 +1596,7 @@
         <v>11</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="G9" s="2" t="s">
         <v>13</v>
@@ -1589,13 +1604,13 @@
     </row>
     <row r="10" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D10" s="2" t="s">
         <v>10</v>
@@ -1604,7 +1619,7 @@
         <v>11</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="G10" s="2" t="s">
         <v>13</v>
@@ -1627,7 +1642,7 @@
         <v>11</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>22</v>
+        <v>39</v>
       </c>
       <c r="G11" s="2" t="s">
         <v>13</v>
@@ -1635,13 +1650,13 @@
     </row>
     <row r="12" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B12" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D12" s="2" t="s">
         <v>10</v>
@@ -1650,7 +1665,7 @@
         <v>11</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G12" s="2" t="s">
         <v>13</v>
@@ -1658,13 +1673,13 @@
     </row>
     <row r="13" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B13" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D13" s="2" t="s">
         <v>10</v>
@@ -1673,7 +1688,7 @@
         <v>11</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>30</v>
+        <v>45</v>
       </c>
       <c r="G13" s="2" t="s">
         <v>13</v>
@@ -1681,13 +1696,13 @@
     </row>
     <row r="14" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B14" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="D14" s="2" t="s">
         <v>10</v>
@@ -1696,7 +1711,7 @@
         <v>11</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="G14" s="2" t="s">
         <v>13</v>
@@ -1704,13 +1719,13 @@
     </row>
     <row r="15" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B15" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="D15" s="2" t="s">
         <v>10</v>
@@ -1719,7 +1734,7 @@
         <v>11</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="G15" s="2" t="s">
         <v>13</v>
@@ -1727,13 +1742,13 @@
     </row>
     <row r="16" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B16" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="D16" s="2" t="s">
         <v>10</v>
@@ -1742,7 +1757,7 @@
         <v>11</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>52</v>
+        <v>42</v>
       </c>
       <c r="G16" s="2" t="s">
         <v>13</v>
@@ -1750,13 +1765,13 @@
     </row>
     <row r="17" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B17" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D17" s="2" t="s">
         <v>10</v>
@@ -1765,7 +1780,7 @@
         <v>11</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G17" s="2" t="s">
         <v>13</v>
@@ -1773,13 +1788,13 @@
     </row>
     <row r="18" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B18" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D18" s="2" t="s">
         <v>10</v>
@@ -1788,7 +1803,7 @@
         <v>11</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="G18" s="2" t="s">
         <v>13</v>
@@ -1796,13 +1811,13 @@
     </row>
     <row r="19" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B19" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D19" s="2" t="s">
         <v>10</v>
@@ -1811,7 +1826,7 @@
         <v>11</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="G19" s="2" t="s">
         <v>13</v>
@@ -1819,13 +1834,13 @@
     </row>
     <row r="20" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B20" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D20" s="2" t="s">
         <v>10</v>
@@ -1834,7 +1849,7 @@
         <v>11</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="G20" s="2" t="s">
         <v>13</v>
@@ -1842,13 +1857,13 @@
     </row>
     <row r="21" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B21" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D21" s="2" t="s">
         <v>10</v>
@@ -1857,7 +1872,7 @@
         <v>11</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="G21" s="2" t="s">
         <v>13</v>
@@ -1865,13 +1880,13 @@
     </row>
     <row r="22" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B22" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D22" s="2" t="s">
         <v>10</v>
@@ -1880,7 +1895,7 @@
         <v>11</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G22" s="2" t="s">
         <v>13</v>
@@ -1888,13 +1903,13 @@
     </row>
     <row r="23" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B23" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D23" s="2" t="s">
         <v>10</v>
@@ -1903,7 +1918,7 @@
         <v>11</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="G23" s="2" t="s">
         <v>13</v>
@@ -1911,13 +1926,13 @@
     </row>
     <row r="24" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B24" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D24" s="2" t="s">
         <v>10</v>
@@ -1926,7 +1941,7 @@
         <v>11</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="G24" s="2" t="s">
         <v>13</v>
@@ -1934,13 +1949,13 @@
     </row>
     <row r="25" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B25" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D25" s="2" t="s">
         <v>10</v>
@@ -1949,7 +1964,7 @@
         <v>11</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="G25" s="2" t="s">
         <v>13</v>
@@ -1957,13 +1972,13 @@
     </row>
     <row r="26" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B26" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D26" s="2" t="s">
         <v>10</v>
@@ -1972,7 +1987,7 @@
         <v>11</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>82</v>
+        <v>74</v>
       </c>
       <c r="G26" s="2" t="s">
         <v>13</v>
@@ -2176,7 +2191,7 @@
         <v>11</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>104</v>
+        <v>56</v>
       </c>
       <c r="G8" s="2" t="s">
         <v>13</v>
@@ -2184,22 +2199,22 @@
     </row>
     <row r="9" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="C9" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="B9" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="C9" s="2" t="s">
+      <c r="D9" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F9" s="2" t="s">
         <v>106</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="E9" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F9" s="2" t="s">
-        <v>41</v>
       </c>
       <c r="G9" s="2" t="s">
         <v>13</v>
@@ -2291,7 +2306,7 @@
         <v>11</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>73</v>
+        <v>31</v>
       </c>
       <c r="G13" s="2" t="s">
         <v>13</v>
@@ -2360,7 +2375,7 @@
         <v>11</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>101</v>
+        <v>39</v>
       </c>
       <c r="G16" s="2" t="s">
         <v>13</v>
@@ -2383,7 +2398,7 @@
         <v>11</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>79</v>
+        <v>98</v>
       </c>
       <c r="G17" s="2" t="s">
         <v>13</v>
@@ -2406,7 +2421,7 @@
         <v>11</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>130</v>
+        <v>39</v>
       </c>
       <c r="G18" s="2" t="s">
         <v>13</v>
@@ -2414,22 +2429,22 @@
     </row>
     <row r="19" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="C19" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="B19" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="C19" s="2" t="s">
+      <c r="D19" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="E19" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F19" s="2" t="s">
         <v>132</v>
-      </c>
-      <c r="D19" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="E19" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F19" s="2" t="s">
-        <v>123</v>
       </c>
       <c r="G19" s="2" t="s">
         <v>13</v>
@@ -2475,7 +2490,7 @@
         <v>11</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G21" s="2" t="s">
         <v>13</v>
@@ -2544,7 +2559,7 @@
         <v>11</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>52</v>
+        <v>146</v>
       </c>
       <c r="G24" s="2" t="s">
         <v>13</v>
@@ -2552,13 +2567,13 @@
     </row>
     <row r="25" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="B25" s="2" t="s">
         <v>84</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="D25" s="2" t="s">
         <v>84</v>
@@ -2567,7 +2582,7 @@
         <v>11</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>22</v>
+        <v>80</v>
       </c>
       <c r="G25" s="2" t="s">
         <v>13</v>
@@ -2575,13 +2590,13 @@
     </row>
     <row r="26" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="B26" s="2" t="s">
         <v>84</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="D26" s="2" t="s">
         <v>84</v>
@@ -2590,7 +2605,7 @@
         <v>11</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="G26" s="2" t="s">
         <v>13</v>
@@ -2598,13 +2613,13 @@
     </row>
     <row r="27" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="B27" s="2" t="s">
         <v>84</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D27" s="2" t="s">
         <v>84</v>
@@ -2613,7 +2628,7 @@
         <v>11</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="G27" s="2" t="s">
         <v>13</v>
@@ -2621,13 +2636,13 @@
     </row>
     <row r="28" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="B28" s="2" t="s">
         <v>84</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="D28" s="2" t="s">
         <v>84</v>
@@ -2636,7 +2651,7 @@
         <v>11</v>
       </c>
       <c r="F28" s="2" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="G28" s="2" t="s">
         <v>13</v>
@@ -2644,13 +2659,13 @@
     </row>
     <row r="29" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B29" s="2" t="s">
         <v>84</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="D29" s="2" t="s">
         <v>84</v>
@@ -2659,7 +2674,7 @@
         <v>11</v>
       </c>
       <c r="F29" s="2" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="G29" s="2" t="s">
         <v>13</v>
@@ -2667,13 +2682,13 @@
     </row>
     <row r="30" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B30" s="2" t="s">
         <v>84</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="D30" s="2" t="s">
         <v>84</v>
@@ -2682,7 +2697,7 @@
         <v>11</v>
       </c>
       <c r="F30" s="2" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="G30" s="2" t="s">
         <v>13</v>
@@ -2690,13 +2705,13 @@
     </row>
     <row r="31" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="B31" s="2" t="s">
         <v>84</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="D31" s="2" t="s">
         <v>84</v>
@@ -2705,7 +2720,7 @@
         <v>11</v>
       </c>
       <c r="F31" s="2" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="G31" s="2" t="s">
         <v>13</v>
@@ -2713,13 +2728,13 @@
     </row>
     <row r="32" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="B32" s="2" t="s">
         <v>84</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="D32" s="2" t="s">
         <v>84</v>
@@ -2728,7 +2743,7 @@
         <v>11</v>
       </c>
       <c r="F32" s="2" t="s">
-        <v>55</v>
+        <v>169</v>
       </c>
       <c r="G32" s="2" t="s">
         <v>13</v>
@@ -2736,13 +2751,13 @@
     </row>
     <row r="33" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="B33" s="2" t="s">
         <v>84</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="D33" s="2" t="s">
         <v>84</v>
@@ -2751,7 +2766,7 @@
         <v>11</v>
       </c>
       <c r="F33" s="2" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="G33" s="2" t="s">
         <v>13</v>
@@ -2759,13 +2774,13 @@
     </row>
     <row r="34" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="B34" s="2" t="s">
         <v>84</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="D34" s="2" t="s">
         <v>84</v>
@@ -2774,7 +2789,7 @@
         <v>11</v>
       </c>
       <c r="F34" s="2" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="G34" s="2" t="s">
         <v>13</v>
@@ -2782,13 +2797,13 @@
     </row>
     <row r="35" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="B35" s="2" t="s">
         <v>84</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="D35" s="2" t="s">
         <v>84</v>
@@ -2797,7 +2812,7 @@
         <v>11</v>
       </c>
       <c r="F35" s="2" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="G35" s="2" t="s">
         <v>13</v>
@@ -2805,13 +2820,13 @@
     </row>
     <row r="36" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="B36" s="2" t="s">
         <v>84</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="D36" s="2" t="s">
         <v>84</v>
@@ -2820,7 +2835,7 @@
         <v>11</v>
       </c>
       <c r="F36" s="2" t="s">
-        <v>58</v>
+        <v>123</v>
       </c>
       <c r="G36" s="2" t="s">
         <v>13</v>
@@ -2828,13 +2843,13 @@
     </row>
     <row r="37" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="B37" s="2" t="s">
         <v>84</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="D37" s="2" t="s">
         <v>84</v>
@@ -2843,7 +2858,7 @@
         <v>11</v>
       </c>
       <c r="F37" s="2" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="G37" s="2" t="s">
         <v>13</v>
@@ -2851,13 +2866,13 @@
     </row>
     <row r="38" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="B38" s="2" t="s">
         <v>84</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="D38" s="2" t="s">
         <v>84</v>
@@ -2866,7 +2881,7 @@
         <v>11</v>
       </c>
       <c r="F38" s="2" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="G38" s="2" t="s">
         <v>13</v>
@@ -2874,13 +2889,13 @@
     </row>
     <row r="39" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="B39" s="2" t="s">
         <v>84</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="D39" s="2" t="s">
         <v>84</v>
@@ -2889,7 +2904,7 @@
         <v>11</v>
       </c>
       <c r="F39" s="2" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="G39" s="2" t="s">
         <v>13</v>
@@ -2897,13 +2912,13 @@
     </row>
     <row r="40" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B40" s="2" t="s">
         <v>84</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="D40" s="2" t="s">
         <v>84</v>
@@ -2912,7 +2927,7 @@
         <v>11</v>
       </c>
       <c r="F40" s="2" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="G40" s="2" t="s">
         <v>13</v>
@@ -2920,13 +2935,13 @@
     </row>
     <row r="41" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="B41" s="2" t="s">
         <v>84</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="D41" s="2" t="s">
         <v>84</v>
@@ -2935,7 +2950,7 @@
         <v>11</v>
       </c>
       <c r="F41" s="2" t="s">
-        <v>190</v>
+        <v>195</v>
       </c>
       <c r="G41" s="2" t="s">
         <v>13</v>
@@ -2986,22 +3001,22 @@
     </row>
     <row r="2" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="E2" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="G2" s="2" t="s">
         <v>13</v>
@@ -3009,22 +3024,22 @@
     </row>
     <row r="3" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="B3" s="2" t="s">
         <v>197</v>
       </c>
-      <c r="B3" s="2" t="s">
-        <v>194</v>
-      </c>
       <c r="C3" s="2" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="E3" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="G3" s="2" t="s">
         <v>13</v>
@@ -3032,22 +3047,22 @@
     </row>
     <row r="4" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="E4" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="G4" s="2" t="s">
         <v>13</v>
@@ -3055,16 +3070,16 @@
     </row>
     <row r="5" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="E5" s="3" t="s">
         <v>11</v>
@@ -3078,22 +3093,22 @@
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="E6" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="G6" s="2" t="s">
         <v>13</v>
@@ -3101,22 +3116,22 @@
     </row>
     <row r="7" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="E7" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="G7" s="2" t="s">
         <v>13</v>
@@ -3124,22 +3139,22 @@
     </row>
     <row r="8" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="E8" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>205</v>
+        <v>215</v>
       </c>
       <c r="G8" s="2" t="s">
         <v>13</v>
@@ -3147,22 +3162,22 @@
     </row>
     <row r="9" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="E9" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>205</v>
+        <v>215</v>
       </c>
       <c r="G9" s="2" t="s">
         <v>13</v>
@@ -3170,22 +3185,22 @@
     </row>
     <row r="10" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="E10" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="G10" s="2" t="s">
         <v>13</v>
@@ -3193,16 +3208,16 @@
     </row>
     <row r="11" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="E11" s="3" t="s">
         <v>11</v>
@@ -3216,16 +3231,16 @@
     </row>
     <row r="12" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="E12" s="3" t="s">
         <v>11</v>
@@ -3239,22 +3254,22 @@
     </row>
     <row r="13" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="E13" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>199</v>
+        <v>205</v>
       </c>
       <c r="G13" s="2" t="s">
         <v>13</v>
@@ -3262,22 +3277,22 @@
     </row>
     <row r="14" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="E14" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>199</v>
+        <v>215</v>
       </c>
       <c r="G14" s="2" t="s">
         <v>13</v>
@@ -3285,22 +3300,22 @@
     </row>
     <row r="15" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="E15" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>199</v>
+        <v>215</v>
       </c>
       <c r="G15" s="2" t="s">
         <v>13</v>
@@ -3308,22 +3323,22 @@
     </row>
     <row r="16" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="E16" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>205</v>
+        <v>215</v>
       </c>
       <c r="G16" s="2" t="s">
         <v>13</v>
@@ -3331,16 +3346,16 @@
     </row>
     <row r="17" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="E17" s="3" t="s">
         <v>11</v>
@@ -3354,22 +3369,22 @@
     </row>
     <row r="18" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="E18" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>205</v>
+        <v>215</v>
       </c>
       <c r="G18" s="2" t="s">
         <v>13</v>
@@ -3377,22 +3392,22 @@
     </row>
     <row r="19" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="E19" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>205</v>
+        <v>215</v>
       </c>
       <c r="G19" s="2" t="s">
         <v>13</v>
@@ -3400,22 +3415,22 @@
     </row>
     <row r="20" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="E20" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>205</v>
+        <v>215</v>
       </c>
       <c r="G20" s="2" t="s">
         <v>13</v>
@@ -3423,22 +3438,22 @@
     </row>
     <row r="21" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="E21" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>205</v>
+        <v>215</v>
       </c>
       <c r="G21" s="2" t="s">
         <v>13</v>
@@ -3489,22 +3504,22 @@
     </row>
     <row r="2" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="E2" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="G2" s="2" t="s">
         <v>13</v>
@@ -3512,22 +3527,22 @@
     </row>
     <row r="3" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
+        <v>246</v>
+      </c>
+      <c r="B3" s="2" t="s">
         <v>243</v>
       </c>
-      <c r="B3" s="2" t="s">
-        <v>240</v>
-      </c>
       <c r="C3" s="2" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="E3" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>82</v>
+        <v>248</v>
       </c>
       <c r="G3" s="2" t="s">
         <v>13</v>
@@ -3535,22 +3550,22 @@
     </row>
     <row r="4" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="E4" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
       <c r="G4" s="2" t="s">
         <v>13</v>
@@ -3558,22 +3573,22 @@
     </row>
     <row r="5" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>248</v>
+        <v>252</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>249</v>
+        <v>253</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="E5" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>205</v>
+        <v>215</v>
       </c>
       <c r="G5" s="2" t="s">
         <v>13</v>
@@ -3581,22 +3596,22 @@
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>250</v>
+        <v>254</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>251</v>
+        <v>255</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="E6" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>252</v>
+        <v>256</v>
       </c>
       <c r="G6" s="2" t="s">
         <v>13</v>
@@ -3604,22 +3619,22 @@
     </row>
     <row r="7" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>253</v>
+        <v>257</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>254</v>
+        <v>258</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="E7" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>64</v>
+        <v>259</v>
       </c>
       <c r="G7" s="2" t="s">
         <v>13</v>
@@ -3627,22 +3642,22 @@
     </row>
     <row r="8" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>255</v>
+        <v>260</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>256</v>
+        <v>261</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="E8" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>257</v>
+        <v>262</v>
       </c>
       <c r="G8" s="2" t="s">
         <v>13</v>
@@ -3650,22 +3665,22 @@
     </row>
     <row r="9" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>258</v>
+        <v>263</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>259</v>
+        <v>264</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="E9" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>260</v>
+        <v>106</v>
       </c>
       <c r="G9" s="2" t="s">
         <v>13</v>
@@ -3673,22 +3688,22 @@
     </row>
     <row r="10" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>261</v>
+        <v>265</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>262</v>
+        <v>266</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="E10" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="G10" s="2" t="s">
         <v>13</v>
@@ -3696,22 +3711,22 @@
     </row>
     <row r="11" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="E11" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>205</v>
+        <v>215</v>
       </c>
       <c r="G11" s="2" t="s">
         <v>13</v>
@@ -3719,22 +3734,22 @@
     </row>
     <row r="12" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>268</v>
+        <v>272</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="E12" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>269</v>
+        <v>273</v>
       </c>
       <c r="G12" s="2" t="s">
         <v>13</v>
@@ -3742,22 +3757,22 @@
     </row>
     <row r="13" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>270</v>
+        <v>274</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>271</v>
+        <v>275</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="E13" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>272</v>
+        <v>276</v>
       </c>
       <c r="G13" s="2" t="s">
         <v>13</v>
@@ -3765,22 +3780,22 @@
     </row>
     <row r="14" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>273</v>
+        <v>277</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>274</v>
+        <v>278</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="E14" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>205</v>
+        <v>215</v>
       </c>
       <c r="G14" s="2" t="s">
         <v>13</v>
@@ -3788,22 +3803,22 @@
     </row>
     <row r="15" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>275</v>
+        <v>279</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>276</v>
+        <v>280</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="E15" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>277</v>
+        <v>281</v>
       </c>
       <c r="G15" s="2" t="s">
         <v>13</v>
@@ -3811,22 +3826,22 @@
     </row>
     <row r="16" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>278</v>
+        <v>282</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>279</v>
+        <v>283</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="E16" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>280</v>
+        <v>284</v>
       </c>
       <c r="G16" s="2" t="s">
         <v>13</v>
@@ -3877,22 +3892,22 @@
     </row>
     <row r="2" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>281</v>
+        <v>285</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>282</v>
+        <v>286</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>283</v>
+        <v>287</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>284</v>
+        <v>288</v>
       </c>
       <c r="E2" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>285</v>
+        <v>289</v>
       </c>
       <c r="G2" s="2" t="s">
         <v>13</v>
@@ -3900,22 +3915,22 @@
     </row>
     <row r="3" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
+        <v>290</v>
+      </c>
+      <c r="B3" s="2" t="s">
         <v>286</v>
       </c>
-      <c r="B3" s="2" t="s">
-        <v>282</v>
-      </c>
       <c r="C3" s="2" t="s">
-        <v>287</v>
+        <v>291</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>284</v>
+        <v>288</v>
       </c>
       <c r="E3" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>288</v>
+        <v>292</v>
       </c>
       <c r="G3" s="2" t="s">
         <v>13</v>
@@ -3923,16 +3938,16 @@
     </row>
     <row r="4" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>289</v>
+        <v>293</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>282</v>
+        <v>286</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>290</v>
+        <v>294</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>282</v>
+        <v>286</v>
       </c>
       <c r="E4" s="3" t="s">
         <v>11</v>
@@ -3946,22 +3961,22 @@
     </row>
     <row r="5" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>291</v>
+        <v>295</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>282</v>
+        <v>286</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>292</v>
+        <v>296</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>282</v>
+        <v>286</v>
       </c>
       <c r="E5" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>293</v>
+        <v>297</v>
       </c>
       <c r="G5" s="2" t="s">
         <v>13</v>
@@ -3969,22 +3984,22 @@
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>294</v>
+        <v>298</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>282</v>
+        <v>286</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>295</v>
+        <v>299</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="E6" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>205</v>
+        <v>215</v>
       </c>
       <c r="G6" s="2" t="s">
         <v>13</v>
@@ -3992,22 +4007,22 @@
     </row>
     <row r="7" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>296</v>
+        <v>300</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>282</v>
+        <v>286</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>297</v>
+        <v>301</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>282</v>
+        <v>286</v>
       </c>
       <c r="E7" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>298</v>
+        <v>302</v>
       </c>
       <c r="G7" s="2" t="s">
         <v>13</v>
@@ -4015,22 +4030,22 @@
     </row>
     <row r="8" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>299</v>
+        <v>303</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>282</v>
+        <v>286</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>300</v>
+        <v>304</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>284</v>
+        <v>288</v>
       </c>
       <c r="E8" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>301</v>
+        <v>305</v>
       </c>
       <c r="G8" s="2" t="s">
         <v>13</v>
@@ -4038,22 +4053,22 @@
     </row>
     <row r="9" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>302</v>
+        <v>306</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>282</v>
+        <v>286</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>303</v>
+        <v>307</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>284</v>
+        <v>288</v>
       </c>
       <c r="E9" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>22</v>
+        <v>308</v>
       </c>
       <c r="G9" s="2" t="s">
         <v>13</v>
@@ -4061,22 +4076,22 @@
     </row>
     <row r="10" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>304</v>
+        <v>309</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>282</v>
+        <v>286</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>305</v>
+        <v>310</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>284</v>
+        <v>288</v>
       </c>
       <c r="E10" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>306</v>
+        <v>311</v>
       </c>
       <c r="G10" s="2" t="s">
         <v>13</v>
@@ -4084,22 +4099,22 @@
     </row>
     <row r="11" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>307</v>
+        <v>312</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>282</v>
+        <v>286</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>308</v>
+        <v>313</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>282</v>
+        <v>286</v>
       </c>
       <c r="E11" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>205</v>
+        <v>215</v>
       </c>
       <c r="G11" s="2" t="s">
         <v>13</v>

</xml_diff>